<commit_message>
Sync agreements from Excel URL column
- Excel column D renamed to URL with raw absolute document URLs
- Add NAO 2024 PV de désaccord and NPS 2023 working-time agreements
- Update NPS 2026, NAO 2025/2023 and other document links
- Derive link category from URL; document the new workflow
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="966" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BD03F5D-C5EE-41B5-A2FA-37A92DF9513C}"/>
+  <xr:revisionPtr revIDLastSave="1325" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16DC3395-6BEF-4AC5-AD91-A6D69BBBEF6A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="accords" sheetId="1" r:id="rId1"/>
     <sheet name="rules" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">accords!$A$1:$O$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">accords!$A$1:$P$31</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,14 +40,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="188">
   <si>
     <t>Accord ou négociation</t>
   </si>
   <si>
-    <t>Lien</t>
-  </si>
-  <si>
     <t>CGT</t>
   </si>
   <si>
@@ -69,9 +66,6 @@
     <t>Don de jours</t>
   </si>
   <si>
-    <t>HRLibrary</t>
-  </si>
-  <si>
     <t>RCC 2024</t>
   </si>
   <si>
@@ -81,9 +75,6 @@
     <t>Déplacements du personnel itinérant</t>
   </si>
   <si>
-    <t>Lien à retrouver</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -213,9 +204,6 @@
     <t>NPS</t>
   </si>
   <si>
-    <t>BDESE</t>
-  </si>
-  <si>
     <t>Signataire (accord signé par toutes les OS représentatives).</t>
   </si>
   <si>
@@ -291,9 +279,6 @@
     <t>Exercices 2025, 2026 et 2027. Enveloppe maximale = 4 % de la masse salariale × [CA vs objectif plan France (50 %) + brevets et publications (25 %) + ratio mobilité durable (25 %)]. Répartition : 50 % selon la durée de présence, 50 % selon le salaire.</t>
   </si>
   <si>
-    <t>Accord NPS signé le 19/12/2025 (réunions des 28/11 et 17/12/2025) : 1 JRTT/JRS collectif fixé au vendredi 15/05/2026 (pont de l'Ascension). S'appuie sur l'accord ARTT Paris-Saclay du 09/01/2001 (3 JRTT/JRS collectifs maximum).</t>
-  </si>
-  <si>
     <t>Avenant n°1 à la RCC du 19/12/2025, suite aux observations de l'inspection du travail (réunion du 14/01/2026) : modifie uniquement l'article 2.5 « Réponse apportée au salarié » (partie VI – départs volontaires).</t>
   </si>
   <si>
@@ -474,9 +459,6 @@
     <t>Accord égalité professionnelle.pdf</t>
   </si>
   <si>
-    <t>cgt39</t>
-  </si>
-  <si>
     <t>NAO_2026_Procès_verbal_d_accord_24 janvier_2026.pdf</t>
   </si>
   <si>
@@ -490,6 +472,138 @@
   </si>
   <si>
     <t>preview pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/BDESENNF-Centrale/_layouts/15/DocIdRedir.aspx?ID=AAIQPNNI5BUR-1489538130-830</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?id=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026/Accord_RCC_2026.pdf&amp;parent=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/Avenant%20n%c2%ba%201%20%c3%a0%20l'Accord%20CSE%20du%2021%20septembre%202018.pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-247229</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/viewer.aspx?sourcedoc=%7b78e118ec-38ae-4539-8422-29417de73e69%7d</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Accord%20collectif%20portant%20sur%20une%20Rupture%20Conventionnelle%20Collective%20(RCC)%20au%20sein%20de%20Nokia%20Networks%20France%20(compress%c3%a9).pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Retraite%20d'Entreprise%20Collectif%20PERCOL%20(16%20d%c3%a9cembre%202025).pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Entreprise%20au%20sein%20de%20Nokia%20Networks%20France%20(16%20d%c3%a9cembre%202025).pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20CET%20(24%20juillet%202025).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/GEPP%20-%20PV%20de%20de%CC%81saccord%202025%20VF-REVUE%20SUITE%20REMARQUES.pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-245115</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/PV%20d%C3%A9saccord%20Partage%20de%20la%20valeur%20VS.pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20cadre%20NPS%20nouvelle%20convention%20collective-%202024%20sign%C3%A9.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d%27int%C3%A9ressement%202025-2028.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20am%C3%A9nagement%20temps%20travail%20NPS%202024.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-242162</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-242235</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20don%20de%20jours%2014%20novembre%202024.pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/Draft%20accord%20harmonisation%20TI%202023.pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-241444</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-240670</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/Accord%20%C3%A9galit%C3%A9%20professionnelle.pdf?web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-237880</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25515</t>
+  </si>
+  <si>
+    <t>NAO 2024 – PV de désaccord</t>
+  </si>
+  <si>
+    <t>NAO politique salariale - PV de désaccord 2024 (+ avenant)</t>
+  </si>
+  <si>
+    <t>Pas d'accord : PV de désaccord NAO 2024 (dernière réunion le 07-08/02/2024), puis avenant au PV négocié le 02/04/2024. Augmentation moyenne jugée « pitoyable » ; mobilisation intersyndicale CFDT / CFE-CGC / CGT en mars 2024.</t>
+  </si>
+  <si>
+    <t>À vérifier : mobilisation intersyndicale contre la faiblesse des augmentations.</t>
+  </si>
+  <si>
+    <t>NAO -&gt; RCC -&gt; REPEAT : l'urgence de la radicalité (15/03/2024)</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25535</t>
+  </si>
+  <si>
+    <t>Accord aménagement temps travail NPS 2023.pdf</t>
+  </si>
+  <si>
+    <t>Note de service Direction NPS du 21/02/2023 : « signature unanime d'un accord »</t>
+  </si>
+  <si>
+    <t>Accord NPS 2023 : 2 JRTT/JRS collectifs (vendredi 19/05/2023 – pont de l'Ascension, et lundi 17/07/2023) ; journée supplémentaire payée (CTG) grâce à la signature ; journée de solidarité le lundi 29/05/2023.</t>
+  </si>
+  <si>
+    <t>Signataire (signature unanime).</t>
+  </si>
+  <si>
+    <t>Courriel Direction (M. Cudot) du 09/02/2024 (réunions des 06/12/2023, 25/01 et 08/02/2024) ; Bilan social NNF 2024 (liste des accords conclus en 2024) : « NAO 2024 - Procès verbal de désaccord (15 février 2024) » ; signataires à vérifier</t>
+  </si>
+  <si>
+    <t>Accord Aménagement Temps Travail NPS 2026 (19 décembre 2025).pdf</t>
+  </si>
+  <si>
+    <t>PDF signé (scan, Massy, 19/12/2025), p. 3 : signatures CFDT, CFE-CGC, CGT et CFTC (+ Direction S. Bermond)</t>
+  </si>
+  <si>
+    <t>Accord d'établissement Nokia Paris-Saclay (Massy, Nozay) signé le 19/12/2025 (réunions des 28/11 et 17/12/2025) : 1 JRTT/JRS collectif fixé au vendredi 15/05/2026 (pont de l'Ascension) ; journée de solidarité le lundi de Pentecôte 25/05/2026. S'appuie sur l'accord ARTT Paris-Saclay du 09/01/2001 (3 JRTT/JRS collectifs maximum).</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Temps%20de%20travail/Accord%20Am%C3%A9nagement%20Temps%20Travail%20NPS%202026%20(19%20d%C3%A9cembre%202025).pdf?d=w3902a5b4f83342a2845c60b07a2afe12&amp;csf=1&amp;web=1&amp;e=RchhtR</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Proc%C3%A8s%20verbal%20NAO%20(d%C3%A9saccord)%202025%20(27%20mars%202025).pdf?d=w9d7b62b129014c718603e94d2d39d5a1&amp;csf=1&amp;web=1&amp;e=xeQooW</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/NAO%202023%20-%20PV%20d%C3%A9saccord.pdf?d=w8c431def6f054edda1304f1db0b90a4b&amp;csf=1&amp;web=1&amp;e=EJaEFz</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/PV%20D%C3%A9saccord%20NAO%202024%20(15%20f%C3%A9vrier%202024).pdf?d=waee681ffe1e04075ad0db67395d7487a&amp;csf=1&amp;web=1&amp;e=B4eck9, https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Avenant%20Proc%C3%A8s-verbal%20de%20d%C3%A9saccord%20NAO%202024%20(9%20avril%202024).pdf?d=w4846416ec812482ea8212ce083de99e2&amp;csf=1&amp;web=1&amp;e=I3LJyw</t>
   </si>
 </sst>
 </file>
@@ -536,18 +650,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -564,7 +676,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -639,25 +751,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -680,9 +779,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -692,7 +788,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -704,54 +800,69 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="8">
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFD8A8"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -774,78 +885,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1153,104 +1192,104 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr defaultColWidth="12.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" style="10" customWidth="1"/>
-    <col min="3" max="3" width="41.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" style="10" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" style="10" customWidth="1"/>
-    <col min="7" max="9" width="9.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="49.5703125" style="10" customWidth="1"/>
-    <col min="11" max="12" width="14.28515625" style="10" customWidth="1"/>
-    <col min="13" max="14" width="57.140625" style="10" customWidth="1"/>
-    <col min="15" max="16" width="41.85546875" style="10" customWidth="1"/>
-    <col min="17" max="16384" width="12.140625" style="10"/>
+    <col min="1" max="1" width="8.28515625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="55.85546875" style="23" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" style="9" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="9" customWidth="1"/>
+    <col min="7" max="9" width="9.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="49.5703125" style="9" customWidth="1"/>
+    <col min="11" max="12" width="14.28515625" style="9" customWidth="1"/>
+    <col min="13" max="14" width="57.140625" style="9" customWidth="1"/>
+    <col min="15" max="16" width="41.85546875" style="9" customWidth="1"/>
+    <col min="17" max="16384" width="12.140625" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="K1" s="9" t="s">
+      <c r="M1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="N1" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>149</v>
+      <c r="P1" s="8" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="11">
+      <c r="A2" s="10">
         <v>2026</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="12" t="b">
+      <c r="D2" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="11" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G2:I2,TRUE),_xlpm.av,COUNTIF(G2:I2,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G2" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="12" t="b">
+      <c r="G2" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="K2" s="1">
         <v>45813</v>
@@ -1259,96 +1298,96 @@
         <v>46181</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P2" s="5"/>
     </row>
-    <row r="3" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
+    <row r="3" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="10">
         <v>2026</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="F3" s="11" t="b">
+        <f t="shared" ref="F3:F31" si="0">_xlfn.LET(_xlpm.ok,COUNTIF(G3:I3,TRUE),_xlpm.av,COUNTIF(G3:I3,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
+      </c>
+      <c r="G3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="K3" s="1">
+        <v>45989</v>
+      </c>
+      <c r="L3" s="1">
+        <v>46010</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="12" t="str">
-        <f t="shared" ref="F3:F29" si="0">_xlfn.LET(_xlpm.ok,COUNTIF(G3:I3,TRUE),_xlpm.av,COUNTIF(G3:I3,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
-        <v>À vérifier</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>14</v>
       </c>
       <c r="P3" s="5"/>
     </row>
     <row r="4" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="11">
+      <c r="A4" s="10">
         <v>2026</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="F4" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G4" s="12" t="b">
+      <c r="G4" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H4" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="12" t="b">
+      <c r="H4" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="K4" s="1">
         <v>46197</v>
@@ -1357,47 +1396,47 @@
         <v>46219</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="P4" s="3"/>
     </row>
     <row r="5" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="11">
+      <c r="A5" s="10">
         <v>2026</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="F5" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="F5" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G5" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="12" t="b">
+      <c r="G5" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="K5" s="1">
         <v>46202</v>
@@ -1406,47 +1445,47 @@
         <v>46212</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P5" s="2"/>
     </row>
     <row r="6" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
+      <c r="A6" s="10">
         <v>2026</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="F6" s="12" t="str">
+        <v>52</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="F6" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G6" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>6</v>
+      <c r="G6" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K6" s="1">
         <v>46041</v>
@@ -1455,96 +1494,96 @@
         <v>46048</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P6" s="2"/>
     </row>
     <row r="7" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="11">
+      <c r="A7" s="10">
         <v>2026</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G7" s="12" t="b">
+      <c r="G7" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="12" t="b">
+      <c r="H7" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L7" s="1">
         <v>46037</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P7" s="2"/>
     </row>
     <row r="8" spans="1:16" ht="120" x14ac:dyDescent="0.25">
-      <c r="A8" s="11">
+      <c r="A8" s="10">
         <v>2026</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="F8" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="F8" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G8" s="12" t="b">
+      <c r="G8" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="12" t="b">
+      <c r="H8" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="K8" s="1">
         <v>45980</v>
@@ -1553,47 +1592,47 @@
         <v>46010</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="P8" s="3"/>
     </row>
     <row r="9" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A9" s="11">
+      <c r="A9" s="10">
         <v>2025</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="F9" s="12" t="str">
+        <v>52</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="F9" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G9" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I9" s="12" t="s">
-        <v>6</v>
+      <c r="G9" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="K9" s="1">
         <v>45947</v>
@@ -1602,96 +1641,96 @@
         <v>46007</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P9" s="2"/>
     </row>
     <row r="10" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
+      <c r="A10" s="10">
         <v>2025</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="E10" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="12" t="str">
+      <c r="F10" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>6</v>
+      <c r="G10" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4">
         <v>45673</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P10" s="5"/>
     </row>
     <row r="11" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A11" s="11">
+      <c r="A11" s="10">
         <v>2025</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="F11" s="12" t="str">
+        <v>52</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="F11" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G11" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>6</v>
+      <c r="G11" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="K11" s="1">
         <v>45947</v>
@@ -1700,47 +1739,47 @@
         <v>46007</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P11" s="2"/>
     </row>
     <row r="12" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A12" s="11">
+      <c r="A12" s="10">
         <v>2025</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="F12" s="12" t="str">
+        <v>52</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F12" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G12" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>6</v>
+      <c r="G12" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="K12" s="1">
         <v>45813</v>
@@ -1750,47 +1789,47 @@
         <v>45862</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P12" s="2"/>
     </row>
     <row r="13" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="11">
+      <c r="A13" s="10">
         <v>2025</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>64</v>
+        <v>52</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="F13" s="12" t="b">
+        <v>153</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="F13" s="11" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G13" s="12" t="b">
+      <c r="G13" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H13" s="12" t="b">
+      <c r="H13" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="I13" s="12" t="b">
+      <c r="I13" s="11" t="b">
         <v>0</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="K13" s="1">
         <v>45708</v>
@@ -1799,47 +1838,47 @@
         <v>45930</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="P13" s="3"/>
     </row>
     <row r="14" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="11">
+      <c r="A14" s="10">
         <v>2025</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>74</v>
+        <v>52</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>70</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="F14" s="12" t="b">
+        <v>185</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" s="11" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G14" s="12" t="b">
+      <c r="G14" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="12" t="b">
+      <c r="H14" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="11" t="b">
         <v>0</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="K14" s="1">
         <v>45684</v>
@@ -1848,47 +1887,47 @@
         <v>45743</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="P14" s="3"/>
     </row>
     <row r="15" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A15" s="11">
+      <c r="A15" s="10">
         <v>2025</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G15" s="12" t="b">
+      <c r="G15" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H15" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I15" s="12" t="b">
+      <c r="H15" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="K15" s="1">
         <v>45680</v>
@@ -1897,145 +1936,145 @@
         <v>45712</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="P15" s="3"/>
     </row>
     <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="11">
+      <c r="A16" s="10">
         <v>2024</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>66</v>
+        <v>52</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>62</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="F16" s="12" t="str">
+        <v>155</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="F16" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G16" s="12" t="b">
+      <c r="G16" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I16" s="12" t="s">
-        <v>6</v>
+      <c r="H16" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="L16" s="1">
+        <v>45538</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P16" s="2"/>
     </row>
     <row r="17" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="11">
+      <c r="A17" s="10">
         <v>2024</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="F17" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="F17" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G17" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I17" s="12" t="b">
+      <c r="G17" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J17" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L17" s="1">
+        <v>45337</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O17" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="P17" s="3"/>
     </row>
     <row r="18" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="11">
+      <c r="A18" s="10">
         <v>2024</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="F18" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G18" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I18" s="12" t="b">
+      <c r="G18" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="K18" s="1">
         <v>45702</v>
@@ -2044,145 +2083,145 @@
         <v>45744</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P18" s="2"/>
     </row>
     <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="11">
+      <c r="A19" s="10">
         <v>2024</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F19" s="12" t="str">
+        <v>52</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G19" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I19" s="12" t="s">
-        <v>6</v>
+      <c r="G19" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P19" s="2"/>
     </row>
     <row r="20" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="11">
+      <c r="A20" s="10">
         <v>2024</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="F20" s="11" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="G20" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O20" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="F20" s="12" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G20" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I20" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="P20" s="2"/>
     </row>
     <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="11">
+      <c r="A21" s="10">
         <v>2024</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="F21" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="F21" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G21" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" s="12" t="b">
+      <c r="G21" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="K21" s="1">
         <v>45356</v>
@@ -2191,96 +2230,96 @@
         <v>45401</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="P21" s="3"/>
     </row>
     <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="11">
+      <c r="A22" s="10">
         <v>2024</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F22" s="12" t="str">
+        <v>52</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G22" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I22" s="12" t="s">
-        <v>6</v>
+      <c r="G22" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P22" s="2"/>
     </row>
     <row r="23" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A23" s="11">
+      <c r="A23" s="10">
         <v>2024</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="F23" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="F23" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G23" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" s="12" t="b">
+      <c r="G23" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="11" t="b">
         <v>1</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="K23" s="1">
         <v>45569</v>
@@ -2289,400 +2328,462 @@
         <v>45610</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P23" s="2"/>
     </row>
-    <row r="24" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="11">
+    <row r="24" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A24" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="F24" s="11" t="str">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G24:I24,TRUE),_xlpm.av,COUNTIF(G24:I24,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>À vérifier</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="K24" s="1">
+        <v>45266</v>
+      </c>
+      <c r="L24" s="1">
+        <v>45337</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="O24" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="P24" s="2"/>
+    </row>
+    <row r="25" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="10">
         <v>2023</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="F24" s="12" t="str">
+      <c r="B25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="F25" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G24" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I24" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="O24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="P24" s="2"/>
-    </row>
-    <row r="25" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A25" s="11">
-        <v>2023</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="F25" s="12" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G25" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H25" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" s="12" t="b">
-        <v>1</v>
+      <c r="G25" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L25" s="1">
-        <v>45259</v>
+        <v>5</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P25" s="2"/>
     </row>
-    <row r="26" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A26" s="11">
+    <row r="26" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="10">
         <v>2023</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F26" s="12" t="b">
+        <v>52</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="F26" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G26" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H26" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I26" s="12" t="b">
+      <c r="G26" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L26" s="1">
+        <v>45259</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="P26" s="2"/>
+    </row>
+    <row r="27" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A27" s="10">
+        <v>2023</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="11" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="G27" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L26" s="1">
+      <c r="J27" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L27" s="1">
         <v>45111</v>
       </c>
-      <c r="M26" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O26" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="P26" s="3"/>
+      <c r="M27" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O27" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="P27" s="3"/>
     </row>
-    <row r="27" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="11">
+    <row r="28" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" s="10">
         <v>2023</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="F27" s="12" t="str">
+      <c r="B28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" s="11" t="str">
         <f t="shared" si="0"/>
         <v>À vérifier</v>
       </c>
-      <c r="G27" s="12" t="b">
+      <c r="G28" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H27" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I27" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="O27" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="P27" s="3"/>
-    </row>
-    <row r="28" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28" s="11">
-        <v>2023</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="F28" s="12" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G28" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H28" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I28" s="12" t="b">
-        <v>1</v>
+      <c r="H28" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="K28" s="1">
-        <v>44845</v>
-      </c>
-      <c r="L28" s="1">
-        <v>45028</v>
+        <v>105</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>94</v>
+        <v>20</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="P28" s="3"/>
     </row>
     <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11">
+      <c r="A29" s="10">
         <v>2023</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="D29" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E29" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F29" s="12" t="b">
+      <c r="D29" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="F29" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G29:I29,TRUE),_xlpm.av,COUNTIF(G29:I29,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
+      </c>
+      <c r="G29" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="O29" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="P29" s="3"/>
+    </row>
+    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="10">
+        <v>2023</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="F30" s="11" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G29" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H29" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L29" s="1">
+      <c r="G30" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H30" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K30" s="1">
+        <v>44845</v>
+      </c>
+      <c r="L30" s="1">
+        <v>45028</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="O30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P30" s="3"/>
+    </row>
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10">
+        <v>2023</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="11" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="G31" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L31" s="1">
         <f>DATE(2022,11,17)</f>
         <v>44882</v>
       </c>
-      <c r="M29" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="O29" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="P29" s="2"/>
+      <c r="M31" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="O31" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="P31" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O29" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A2:O29">
-    <cfRule type="containsText" dxfId="16" priority="13" operator="containsText" text="vérifier">
+  <autoFilter ref="A1:P31" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A2:P31">
+    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="14" operator="containsText" text="retrouver">
+    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="15" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:F29">
-    <cfRule type="containsText" dxfId="10" priority="7" operator="containsText" text="vérifier">
-      <formula>NOT(ISERROR(SEARCH("vérifier",E2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="8" operator="containsText" text="retrouver">
-      <formula>NOT(ISERROR(SEARCH("retrouver",E2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="préciser">
-      <formula>NOT(ISERROR(SEARCH("préciser",E2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F29">
-    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="vérifier">
-      <formula>NOT(ISERROR(SEARCH("vérifier",F2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="retrouver">
-      <formula>NOT(ISERROR(SEARCH("retrouver",F2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="préciser">
-      <formula>NOT(ISERROR(SEARCH("préciser",F2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:I29">
-    <cfRule type="expression" dxfId="4" priority="16">
+  <conditionalFormatting sqref="F2:I31">
+    <cfRule type="expression" dxfId="4" priority="19">
       <formula>F2=TRUE</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:I29">
-    <cfRule type="expression" dxfId="3" priority="17">
+    <cfRule type="expression" dxfId="3" priority="20">
       <formula>F2=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P29">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="vérifier">
-      <formula>NOT(ISERROR(SEARCH("vérifier",P2)))</formula>
+  <conditionalFormatting sqref="D2:D31">
+    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
+      <formula>OR(ISNUMBER(SEARCH("HRLibrary",$D2)),ISNUMBER(SEARCH("BDESE",$D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="retrouver">
-      <formula>NOT(ISERROR(SEARCH("retrouver",P2)))</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D31">
+    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
+      <formula>ISNUMBER(SEARCH("CGT39",$D2))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="préciser">
-      <formula>NOT(ISERROR(SEARCH("préciser",P2)))</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D31">
+    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
+      <formula>LEN(TRIM($D2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="D26" r:id="rId1" display="CGT39" xr:uid="{B652B381-BF1A-487C-AC64-0676C07A41E5}"/>
-    <hyperlink ref="D25" r:id="rId2" display="CGT39" xr:uid="{E09AFAE3-55E4-48CF-9CC2-C94F4CFE3964}"/>
-    <hyperlink ref="D23" r:id="rId3" display="../../../HRLibrary/Controlled Documents/HR Regions/Europe South/France/HR SOPs-Guidelines-Policy/Harmonized/Accords conventions 2024/Accord don de jours 14 novembre 2024.pdf?web=1" xr:uid="{C0F3AF27-9BBF-41DE-87E5-6C57562A3040}"/>
-    <hyperlink ref="D22" r:id="rId4" display="../../../HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-242235" xr:uid="{97ED7A41-5492-4B4E-B9B1-FD66AA38F5ED}"/>
-    <hyperlink ref="D21" r:id="rId5" display="../../../HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-242162" xr:uid="{B481510D-8BA3-473E-8F71-AA111D58111B}"/>
-    <hyperlink ref="D20" r:id="rId6" display="CGT39" xr:uid="{E1B57F18-24A4-447A-B247-AFB7D41174D1}"/>
-    <hyperlink ref="D17" r:id="rId7" display="CGT39" xr:uid="{AD36386D-F9A0-4B76-91EF-7EE0E3767AC8}"/>
-    <hyperlink ref="D12" r:id="rId8" display="CGT39" xr:uid="{C393D335-5FCB-4556-AD47-7898F9F2E919}"/>
-    <hyperlink ref="D11" r:id="rId9" display="../../../HRLibrary/Controlled Documents/HR Regions/Europe South/France/HR SOPs-Guidelines-Policy/Harmonized/Accords conventions 2025/Accord d'entreprise relatif au Plan d'Epargne Entreprise au sein de Nokia Networks France (16 d%c3%a9cembre 2025).pdf?web=1" xr:uid="{30E86710-B52D-4ECD-B40D-3B6B0BB50BB9}"/>
-    <hyperlink ref="D9" r:id="rId10" display="../../../HRLibrary/Controlled Documents/HR Regions/Europe South/France/HR SOPs-Guidelines-Policy/Harmonized/Accords conventions 2025/Accord d'entreprise relatif au Plan d'Epargne Retraite d'Entreprise Collectif PERCOL (16 d%c3%a9cembre 2025).pdf?web=1" xr:uid="{0AB087BA-41E9-4E66-91C5-A041426D7484}"/>
-    <hyperlink ref="D8" r:id="rId11" display="../../../HRLibrary/Controlled Documents/HR Regions/Europe South/France/Plan-de-transformation/RCC 2025/Accord collectif portant sur une Rupture Conventionnelle Collective (RCC) au sein de Nokia Networks France (compress%c3%a9).pdf?web=1" xr:uid="{1BD937E8-DE87-4153-A504-4D327A7B8634}"/>
-    <hyperlink ref="D7" r:id="rId12" display="../../../HRLibrary/_layouts/15/viewer.aspx?sourcedoc=%7b78e118ec-38ae-4539-8422-29417de73e69%7d" xr:uid="{4599B013-D148-4BBA-9419-0C0B6B45A3E0}"/>
-    <hyperlink ref="D6" r:id="rId13" display="../../../HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-247229" xr:uid="{E7B78842-1717-4059-BE2E-776C7090974C}"/>
-    <hyperlink ref="D5" r:id="rId14" display="../../../HRLibrary/Controlled Documents/HR Regions/Europe South/France/HR SOPs-Guidelines-Policy/Harmonized/Accords conventions 2026/Avenant n%c2%ba 1 %c3%a0 l'Accord CSE du 21 septembre 2018.pdf?web=1" xr:uid="{74C437F8-3478-486C-BC3C-0105299AE4C3}"/>
-    <hyperlink ref="D4" r:id="rId15" display="CGT39" xr:uid="{7CCCDB63-5C71-49B7-AAC7-102208F2A556}"/>
-    <hyperlink ref="D2" r:id="rId16" display="CGT39" xr:uid="{2334AD23-DAF8-4F25-9AD4-3238A1FF52C8}"/>
-    <hyperlink ref="D15" r:id="rId17" display="https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-245115" xr:uid="{D2342114-7FD0-46C6-BA8A-FE5A719E5D12}"/>
-    <hyperlink ref="D18" r:id="rId18" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d%27int%C3%A9ressement%202025-2028.pdf" xr:uid="{658BDE47-7E8C-4FDD-AC90-F4BE0A4F5590}"/>
-    <hyperlink ref="D29" r:id="rId19" display="https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-237880" xr:uid="{F3CA397A-3C4F-4EB2-9E78-5E3F6CF5AD0A}"/>
-    <hyperlink ref="O4" r:id="rId20" display="Votre ressenti pour la RCC 2026-2 (26/06/2026)" xr:uid="{59D95BD5-7957-4DC2-9292-2CBBBB953C0D}"/>
-    <hyperlink ref="O8" r:id="rId21" xr:uid="{B5450024-F62E-4456-B70D-13EE54625FA9}"/>
-    <hyperlink ref="O13" r:id="rId22" display="Rappel dans le tract RCC de novembre 2025" xr:uid="{8A361D52-2C0D-4A5E-B963-5A59F5A00104}"/>
-    <hyperlink ref="O14" r:id="rId23" display="Salaires : les négos ça ne marche pas (26/03/2025)" xr:uid="{5D4473E7-1C88-48FE-A14D-A15093F3B79B}"/>
-    <hyperlink ref="O15" r:id="rId24" display="Avenant Télétravail : signer pour 40 centimes ? (19/02/2025)" xr:uid="{558A19AF-8D80-4D08-ABC2-4A3E7D1CD93A}"/>
-    <hyperlink ref="O17" r:id="rId25" display="Et toi alors, t'es coté combien ? (13/11/2023)" xr:uid="{01E3DB2C-8C96-4A47-9002-9C3BFBFA84FF}"/>
-    <hyperlink ref="O21" r:id="rId26" display="Bilan de la RCC 2024 (06/11/2024) ; " xr:uid="{22B006CE-6E87-4246-B4EA-8BA01364E20A}"/>
-    <hyperlink ref="O26" r:id="rId27" display="RCC : des motifs de vigilance (09/2023) ; " xr:uid="{065592F7-3619-4EE0-A07C-438E248C4E8F}"/>
-    <hyperlink ref="O27" r:id="rId28" xr:uid="{FF1EF8E1-6A04-432C-8713-D23076AA8098}"/>
-    <hyperlink ref="O28" r:id="rId29" xr:uid="{1699107D-21CE-4FF6-AE63-2552D0557C45}"/>
+    <hyperlink ref="O4" r:id="rId1" display="Votre ressenti pour la RCC 2026-2 (26/06/2026)" xr:uid="{59D95BD5-7957-4DC2-9292-2CBBBB953C0D}"/>
+    <hyperlink ref="O8" r:id="rId2" xr:uid="{B5450024-F62E-4456-B70D-13EE54625FA9}"/>
+    <hyperlink ref="O13" r:id="rId3" display="Rappel dans le tract RCC de novembre 2025" xr:uid="{8A361D52-2C0D-4A5E-B963-5A59F5A00104}"/>
+    <hyperlink ref="O14" r:id="rId4" display="Salaires : les négos ça ne marche pas (26/03/2025)" xr:uid="{5D4473E7-1C88-48FE-A14D-A15093F3B79B}"/>
+    <hyperlink ref="O15" r:id="rId5" display="Avenant Télétravail : signer pour 40 centimes ? (19/02/2025)" xr:uid="{558A19AF-8D80-4D08-ABC2-4A3E7D1CD93A}"/>
+    <hyperlink ref="O17" r:id="rId6" display="Et toi alors, t'es coté combien ? (13/11/2023)" xr:uid="{01E3DB2C-8C96-4A47-9002-9C3BFBFA84FF}"/>
+    <hyperlink ref="O21" r:id="rId7" display="Bilan de la RCC 2024 (06/11/2024) ; " xr:uid="{22B006CE-6E87-4246-B4EA-8BA01364E20A}"/>
+    <hyperlink ref="O27" r:id="rId8" display="RCC : des motifs de vigilance (09/2023) ; " xr:uid="{065592F7-3619-4EE0-A07C-438E248C4E8F}"/>
+    <hyperlink ref="O28" r:id="rId9" xr:uid="{FF1EF8E1-6A04-432C-8713-D23076AA8098}"/>
+    <hyperlink ref="O30" r:id="rId10" xr:uid="{1699107D-21CE-4FF6-AE63-2552D0557C45}"/>
+    <hyperlink ref="D4" r:id="rId11" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?id=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026/Accord_RCC_2026.pdf&amp;parent=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026" xr:uid="{2EC36556-9A1E-448F-990C-1BFE28A28515}"/>
+    <hyperlink ref="D20" r:id="rId12" xr:uid="{A9AF55B6-9AF4-441B-BF54-A1A9640D2C9D}"/>
+    <hyperlink ref="D24" r:id="rId13" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/PV%20D%C3%A9saccord%20NAO%202024%20(15%20f%C3%A9vrier%202024).pdf?d=waee681ffe1e04075ad0db67395d7487a&amp;csf=1&amp;web=1&amp;e=B4eck9," xr:uid="{F6B82D88-92B4-4369-B825-E6CFE444F804}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId30"/>
+  <pageSetup orientation="portrait" r:id="rId14"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
   </headerFooter>
@@ -2702,11 +2803,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -2756,7 +2852,7 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2765,7 +2861,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
@@ -2782,7 +2878,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -3053,15 +3149,12 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
@@ -3069,7 +3162,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -3077,7 +3170,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3088,8 +3181,32 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
+    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
+    <ds:schemaRef ds:uri="98344022-9d6c-42ca-8763-b68a110aeabc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5384275B-3603-46F1-AC57-45AFF030DC9D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Ignore local copies PDFs
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1325" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16DC3395-6BEF-4AC5-AD91-A6D69BBBEF6A}"/>
+  <xr:revisionPtr revIDLastSave="1331" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2DD2DDF-6932-45B9-BAEB-B7620373C3B9}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="accords" sheetId="1" r:id="rId1"/>
@@ -756,7 +756,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -821,10 +821,7 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -833,39 +830,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFD8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FFFFFFFF"/>
@@ -885,6 +849,39 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFD8A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -923,10 +920,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1198,7 +1191,7 @@
     <col min="1" max="1" width="8.28515625" style="9" customWidth="1"/>
     <col min="2" max="2" width="7.5703125" style="9" customWidth="1"/>
     <col min="3" max="3" width="41.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="55.85546875" style="23" customWidth="1"/>
+    <col min="4" max="4" width="46" style="22" customWidth="1"/>
     <col min="5" max="5" width="21.7109375" style="9" customWidth="1"/>
     <col min="6" max="6" width="15.28515625" style="9" customWidth="1"/>
     <col min="7" max="9" width="9.28515625" style="9" bestFit="1" customWidth="1"/>
@@ -1661,7 +1654,7 @@
       <c r="C10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="20" t="s">
         <v>169</v>
       </c>
       <c r="E10" s="13" t="s">
@@ -2593,7 +2586,7 @@
       <c r="C29" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="20" t="s">
         <v>175</v>
       </c>
       <c r="E29" s="14" t="s">
@@ -2744,27 +2737,23 @@
       <formula>NOT(ISERROR(SEARCH("préciser",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:I31">
-    <cfRule type="expression" dxfId="4" priority="19">
-      <formula>F2=TRUE</formula>
+  <conditionalFormatting sqref="D2:D31">
+    <cfRule type="expression" dxfId="4" priority="1" stopIfTrue="1">
+      <formula>LEN(TRIM($D2))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="20">
-      <formula>F2=FALSE</formula>
+    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
+      <formula>ISNUMBER(SEARCH("CGT39",$D2))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D31">
     <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
       <formula>OR(ISNUMBER(SEARCH("HRLibrary",$D2)),ISNUMBER(SEARCH("BDESE",$D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D31">
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("CGT39",$D2))</formula>
+  <conditionalFormatting sqref="F2:I31">
+    <cfRule type="expression" dxfId="1" priority="19">
+      <formula>F2=TRUE</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D31">
-    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>LEN(TRIM($D2))=0</formula>
+    <cfRule type="expression" dxfId="0" priority="20">
+      <formula>F2=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -2781,9 +2770,11 @@
     <hyperlink ref="D4" r:id="rId11" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?id=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026/Accord_RCC_2026.pdf&amp;parent=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026" xr:uid="{2EC36556-9A1E-448F-990C-1BFE28A28515}"/>
     <hyperlink ref="D20" r:id="rId12" xr:uid="{A9AF55B6-9AF4-441B-BF54-A1A9640D2C9D}"/>
     <hyperlink ref="D24" r:id="rId13" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/PV%20D%C3%A9saccord%20NAO%202024%20(15%20f%C3%A9vrier%202024).pdf?d=waee681ffe1e04075ad0db67395d7487a&amp;csf=1&amp;web=1&amp;e=B4eck9," xr:uid="{F6B82D88-92B4-4369-B825-E6CFE444F804}"/>
+    <hyperlink ref="D29" r:id="rId14" xr:uid="{C043EA89-0A53-4B71-AC0C-5C4306E62617}"/>
+    <hyperlink ref="D10" r:id="rId15" xr:uid="{5C4C6E25-614E-4F25-8AA8-26F96EA1D6FC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId14"/>
+  <pageSetup orientation="portrait" r:id="rId16"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
   </headerFooter>
@@ -2804,56 +2795,6 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
@@ -2861,7 +2802,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
@@ -2878,7 +2819,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -3149,20 +3090,62 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -3170,7 +3153,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3181,7 +3164,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3201,10 +3184,18 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Sync agreement links and local PDFs
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1331" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2DD2DDF-6932-45B9-BAEB-B7620373C3B9}"/>
+  <xr:revisionPtr revIDLastSave="1436" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52B98D3D-5680-4D95-9DF0-AE8DAACC3B7D}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="195">
   <si>
     <t>Accord ou négociation</t>
   </si>
@@ -99,9 +99,6 @@
     <t>Non signataire (détail du vote interne non retrouvé).</t>
   </si>
   <si>
-    <t>Brèves de printemps (21/04/2023)</t>
-  </si>
-  <si>
     <t>Pas d'accord signé. Enveloppe appliquée unilatéralement : 3,21 % cadres, 5 % non-cadres. Contestation des nombreux 0 % d'augmentation.</t>
   </si>
   <si>
@@ -240,9 +237,6 @@
     <t>Comité Groupe France (CGF)</t>
   </si>
   <si>
-    <t>Harmonisation des bonus TI (projet)</t>
-  </si>
-  <si>
     <t>Substitution non-cadres</t>
   </si>
   <si>
@@ -360,21 +354,6 @@
     <t>À vérifier (aucune source trouvée)</t>
   </si>
   <si>
-    <t>Pour ceux qui restent (19/12/2025)</t>
-  </si>
-  <si>
-    <t>N-ième RCC, 2ème de 2026 : retour sondage salariés (26/06/2026)</t>
-  </si>
-  <si>
-    <t>Happy Thanksgiving chez Nokia : l'industrie française dindon de la farce (28/11/2025)</t>
-  </si>
-  <si>
-    <t>Salaires +0,68 % : les négos ça ne marche pas, il faut se mobiliser (26/03/2025)</t>
-  </si>
-  <si>
-    <t>Avenant Télétravail : signer pour 40 centimes ? Chronique d'une occasion manquée (19/02/2025)</t>
-  </si>
-  <si>
     <t>PDF signé « Accord_RCC_2026 » (Adobe Sign, 16/07/2026), p. 54 : signatures CFDT (S. Regnouard, R. Tutrel) et CFE-CGC (V. Gervais-Bazin) ; bloc CGT vide</t>
   </si>
   <si>
@@ -399,15 +378,6 @@
     <t>À vérifier : seule la version « mise à la signature » (non signée, 20/01/2025) a été trouvée</t>
   </si>
   <si>
-    <t>Et toi alors, t'es coté combien ? (31/10/2023)</t>
-  </si>
-  <si>
-    <t>Bilan de la RCC 2024 : Nokia a (encore) montré son vrai visage (05/11/2024)</t>
-  </si>
-  <si>
-    <t>Rentrée 2023 – Volontariat RCC : des motifs de vigilance (18/09/2023)</t>
-  </si>
-  <si>
     <t>file name</t>
   </si>
   <si>
@@ -429,9 +399,6 @@
     <t>Accord CET (24 juillet 2025).pdf</t>
   </si>
   <si>
-    <t>GEPP - PV de désaccord 2025 VF-REVUE SUITE REMARQUES.pdf</t>
-  </si>
-  <si>
     <t>Procès verbal NAO (désaccord) 2025 (27 mars 2025).pdf</t>
   </si>
   <si>
@@ -450,9 +417,6 @@
     <t>Accord don de jours 14 novembre 2024.pdf</t>
   </si>
   <si>
-    <t>Draft accord harmonisation TI 2023.pdf</t>
-  </si>
-  <si>
     <t>NAO 2023 - PV désaccord.pdf</t>
   </si>
   <si>
@@ -474,42 +438,9 @@
     <t>preview pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/BDESENNF-Centrale/_layouts/15/DocIdRedir.aspx?ID=AAIQPNNI5BUR-1489538130-830</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?id=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026/Accord_RCC_2026.pdf&amp;parent=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/Avenant%20n%c2%ba%201%20%c3%a0%20l'Accord%20CSE%20du%2021%20septembre%202018.pdf?web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-247229</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/viewer.aspx?sourcedoc=%7b78e118ec-38ae-4539-8422-29417de73e69%7d</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Accord%20collectif%20portant%20sur%20une%20Rupture%20Conventionnelle%20Collective%20(RCC)%20au%20sein%20de%20Nokia%20Networks%20France%20(compress%c3%a9).pdf?web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Retraite%20d'Entreprise%20Collectif%20PERCOL%20(16%20d%c3%a9cembre%202025).pdf?web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Entreprise%20au%20sein%20de%20Nokia%20Networks%20France%20(16%20d%c3%a9cembre%202025).pdf?web=1</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20CET%20(24%20juillet%202025).pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/GEPP%20-%20PV%20de%20de%CC%81saccord%202025%20VF-REVUE%20SUITE%20REMARQUES.pdf?web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-245115</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/PV%20d%C3%A9saccord%20Partage%20de%20la%20valeur%20VS.pdf?web=1</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20cadre%20NPS%20nouvelle%20convention%20collective-%202024%20sign%C3%A9.pdf</t>
   </si>
   <si>
@@ -519,60 +450,21 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20am%C3%A9nagement%20temps%20travail%20NPS%202024.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-242162</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-242235</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20don%20de%20jours%2014%20novembre%202024.pdf?web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/Draft%20accord%20harmonisation%20TI%202023.pdf?web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-241444</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-240670</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/wall-of-negos/Accord%20%C3%A9galit%C3%A9%20professionnelle.pdf?web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/_layouts/15/DocIdRedir.aspx?ID=BTI3POTITA3Q-1865654459-237880</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
     <t>URL</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25515</t>
-  </si>
-  <si>
     <t>NAO 2024 – PV de désaccord</t>
   </si>
   <si>
-    <t>NAO politique salariale - PV de désaccord 2024 (+ avenant)</t>
-  </si>
-  <si>
     <t>Pas d'accord : PV de désaccord NAO 2024 (dernière réunion le 07-08/02/2024), puis avenant au PV négocié le 02/04/2024. Augmentation moyenne jugée « pitoyable » ; mobilisation intersyndicale CFDT / CFE-CGC / CGT en mars 2024.</t>
   </si>
   <si>
     <t>À vérifier : mobilisation intersyndicale contre la faiblesse des augmentations.</t>
   </si>
   <si>
-    <t>NAO -&gt; RCC -&gt; REPEAT : l'urgence de la radicalité (15/03/2024)</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25535</t>
-  </si>
-  <si>
-    <t>Accord aménagement temps travail NPS 2023.pdf</t>
-  </si>
-  <si>
     <t>Note de service Direction NPS du 21/02/2023 : « signature unanime d'un accord »</t>
   </si>
   <si>
@@ -594,16 +486,145 @@
     <t>Accord d'établissement Nokia Paris-Saclay (Massy, Nozay) signé le 19/12/2025 (réunions des 28/11 et 17/12/2025) : 1 JRTT/JRS collectif fixé au vendredi 15/05/2026 (pont de l'Ascension) ; journée de solidarité le lundi de Pentecôte 25/05/2026. S'appuie sur l'accord ARTT Paris-Saclay du 09/01/2001 (3 JRTT/JRS collectifs maximum).</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Temps%20de%20travail/Accord%20Am%C3%A9nagement%20Temps%20Travail%20NPS%202026%20(19%20d%C3%A9cembre%202025).pdf?d=w3902a5b4f83342a2845c60b07a2afe12&amp;csf=1&amp;web=1&amp;e=RchhtR</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Proc%C3%A8s%20verbal%20NAO%20(d%C3%A9saccord)%202025%20(27%20mars%202025).pdf?d=w9d7b62b129014c718603e94d2d39d5a1&amp;csf=1&amp;web=1&amp;e=xeQooW</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/NAO%202023%20-%20PV%20d%C3%A9saccord.pdf?d=w8c431def6f054edda1304f1db0b90a4b&amp;csf=1&amp;web=1&amp;e=EJaEFz</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/PV%20D%C3%A9saccord%20NAO%202024%20(15%20f%C3%A9vrier%202024).pdf?d=waee681ffe1e04075ad0db67395d7487a&amp;csf=1&amp;web=1&amp;e=B4eck9, https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Avenant%20Proc%C3%A8s-verbal%20de%20d%C3%A9saccord%20NAO%202024%20(9%20avril%202024).pdf?d=w4846416ec812482ea8212ce083de99e2&amp;csf=1&amp;web=1&amp;e=I3LJyw</t>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/NAO_2026_Proc%c3%a8s_verbal_d_accord_24%20janvier_2026.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/BDESENNF-Centrale/Shared%20Documents/01.%20BDESE%20Centrale/02%20-%20Investissements/01%20-%20Investissement%20social/Handicap/Accord%20handicap%202026.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/GEPP%20PV%20de%20d%C3%A9saccord%20mis%20%C3%A0%20signature.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202022/Accord%20%C3%A9tablissement%20am%C3%A9nagement%20temps%20de%20travail%202022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20%C3%A9galit%C3%A9%20professionnelle.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20remboursement%20sant%C3%A9%20-%202023.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Avenant%20accord%20t%c3%a9l%c3%a9travail%20avril%202022.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202023/Accord%20RCC%202023.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20de%20substitution%20non%20cadres%20-%2030%20novembre%202023.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202024/Accord%20RCC%202024%20(19%20avril%202024).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accord%20CGF.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026/Accord_RCC_2026.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/PV%20d%C3%A9saccord%20Partage%20de%20la%20valeur%20VS.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/NAO%202023%20-%20PV%20d%C3%A9saccord.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20don%20de%20jours%2014%20novembre%202024.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Avenant%20Proc%C3%A8s-verbal%20de%20d%C3%A9saccord%20NAO%202024%20(9%20avril%202024).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Entreprise%20au%20sein%20de%20Nokia%20Networks%20France%20(16%20d%c3%a9cembre%202025).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Retraite%20d'Entreprise%20Collectif%20PERCOL%20(16%20d%c3%a9cembre%202025).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Proc%C3%A8s%20verbal%20NAO%20(d%C3%A9saccord)%202025%20(27%20mars%202025).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/Avenant%20n%c2%ba%201%20%c3%a0%20l'Accord%20CSE%20du%2021%20septembre%202018.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Temps%20de%20travail/Accord%20Am%C3%A9nagement%20Temps%20Travail%20NPS%202026%20(19%20d%C3%A9cembre%202025).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Accord%20collectif%20portant%20sur%20une%20Rupture%20Conventionnelle%20Collective%20(RCC)%20au%20sein%20de%20Nokia%20Networks%20France%20(compress%c3%a9).pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Avenant%20RCC%202025.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salariés/tracts%20diffusés/2023/Tract%20brèves%20de%20printemps.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2026/2026_06_TRACT-RetourSondageRCC2026-2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract_pour_ceux_qui_restent.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract_rcc_2026.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract-salaires-2025.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract-avenant-TL-v2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2024/tract_bilan_rcc24_v4.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2023/ncc%20cotation%203.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2023/Tract%20Volontariat%20RCC.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2023/Tract%20br%C3%A8ves%20de%20printemps.pdf</t>
+  </si>
+  <si>
+    <t>Accord CGF.pdf</t>
+  </si>
+  <si>
+    <t>Accord établissement aménagement temps de travail 2022.pdf</t>
+  </si>
+  <si>
+    <t>Avenant RCC 2025.pdf</t>
+  </si>
+  <si>
+    <t>GEPP PV de désaccord mis à signature.pdf</t>
+  </si>
+  <si>
+    <t>Avenant accord télétravail avril 2022.pdf</t>
+  </si>
+  <si>
+    <t>2025 Accord etablissement NAO Mis à la signature.pdf</t>
+  </si>
+  <si>
+    <t>Avenant Procès-verbal de désaccord NAO 2024 (9 avril 2024).pdf</t>
+  </si>
+  <si>
+    <t>Accord RCC 2023.pdf</t>
+  </si>
+  <si>
+    <t>Accord remboursement santé - 2023.pdf</t>
+  </si>
+  <si>
+    <t>Accord harmonisation taux variable cible.pdf</t>
+  </si>
+  <si>
+    <t>Accord collectif portant sur l’harmonisation des taux de variable cible des salariés « non sales » au regard de leur job grade</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/Accord%20harmonisation%20taux%20variable%20cible.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/2025%20Accord%20etablissement%20NAO%20Mis%20%C3%A0%20la%20signature.pdf</t>
+  </si>
+  <si>
+    <t>ACCORD HANDICAP VERSION REVUE LE 8 juin 2026.pdf</t>
   </si>
 </sst>
 </file>
@@ -818,10 +839,10 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1191,14 +1212,15 @@
     <col min="1" max="1" width="8.28515625" style="9" customWidth="1"/>
     <col min="2" max="2" width="7.5703125" style="9" customWidth="1"/>
     <col min="3" max="3" width="41.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46" style="22" customWidth="1"/>
+    <col min="4" max="4" width="114.28515625" style="21" customWidth="1"/>
     <col min="5" max="5" width="21.7109375" style="9" customWidth="1"/>
     <col min="6" max="6" width="15.28515625" style="9" customWidth="1"/>
     <col min="7" max="9" width="9.28515625" style="9" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="49.5703125" style="9" customWidth="1"/>
     <col min="11" max="12" width="14.28515625" style="9" customWidth="1"/>
     <col min="13" max="14" width="57.140625" style="9" customWidth="1"/>
-    <col min="15" max="16" width="41.85546875" style="9" customWidth="1"/>
+    <col min="15" max="15" width="82.140625" style="9" customWidth="1"/>
+    <col min="16" max="16" width="41.85546875" style="9" customWidth="1"/>
     <col min="17" max="16384" width="12.140625" style="9"/>
   </cols>
   <sheetData>
@@ -1207,19 +1229,19 @@
         <v>12</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>168</v>
+        <v>137</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>1</v>
@@ -1231,7 +1253,7 @@
         <v>3</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>14</v>
@@ -1249,174 +1271,174 @@
         <v>17</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="10">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="E2" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="11" t="b">
+      <c r="F2" s="11" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G2:I2,TRUE),_xlpm.av,COUNTIF(G2:I2,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
-        <v>1</v>
+        <v>À vérifier</v>
       </c>
       <c r="G2" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="11" t="b">
-        <v>1</v>
+      <c r="H2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="K2" s="1">
-        <v>45813</v>
-      </c>
-      <c r="L2" s="1">
-        <v>46181</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="O2" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="5"/>
+      <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="10">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>184</v>
-      </c>
-      <c r="E3" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="F3" s="11" t="str">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G3:I3,TRUE),_xlpm.av,COUNTIF(G3:I3,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>À vérifier</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="P3" s="2"/>
+    </row>
+    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="F3" s="11" t="b">
-        <f t="shared" ref="F3:F31" si="0">_xlfn.LET(_xlpm.ok,COUNTIF(G3:I3,TRUE),_xlpm.av,COUNTIF(G3:I3,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
-        <v>1</v>
-      </c>
-      <c r="G3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="K3" s="1">
-        <v>45989</v>
-      </c>
-      <c r="L3" s="1">
-        <v>46010</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="O3" s="5" t="s">
+      <c r="F4" s="11" t="str">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G4:I4,TRUE),_xlpm.av,COUNTIF(G4:I4,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>À vérifier</v>
+      </c>
+      <c r="G4" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="P3" s="5"/>
+      <c r="P4" s="2"/>
     </row>
-    <row r="4" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="10">
-        <v>2026</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>145</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="F4" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G4" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="H4" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46197</v>
-      </c>
-      <c r="L4" s="1">
-        <v>46219</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="P4" s="3"/>
-    </row>
-    <row r="5" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="10">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>146</v>
+        <v>9</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>151</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>124</v>
+        <v>182</v>
       </c>
       <c r="F5" s="11" t="b">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G5:I5,TRUE),_xlpm.av,COUNTIF(G5:I5,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
       <c r="G5" s="11" t="b">
@@ -1429,47 +1451,47 @@
         <v>1</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46202</v>
-      </c>
-      <c r="L5" s="1">
-        <v>46212</v>
+        <v>141</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>48</v>
+        <v>142</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O5" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="O5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="P5" s="2"/>
+      <c r="P5" s="3"/>
     </row>
-    <row r="6" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="10">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="18" t="s">
-        <v>147</v>
+      <c r="D6" s="20" t="s">
+        <v>161</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="F6" s="11" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G6:I6,TRUE),_xlpm.av,COUNTIF(G6:I6,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
       <c r="G6" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>5</v>
@@ -1478,47 +1500,47 @@
         <v>5</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46041</v>
-      </c>
-      <c r="L6" s="1">
-        <v>46048</v>
+        <v>103</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>76</v>
+        <v>19</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P6" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="P6" s="3"/>
     </row>
-    <row r="7" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="10">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>148</v>
+        <v>9</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>135</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>11</v>
+        <v>123</v>
       </c>
       <c r="F7" s="11" t="b">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G7:I7,TRUE),_xlpm.av,COUNTIF(G7:I7,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
       <c r="G7" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" s="11" t="b">
         <v>1</v>
@@ -1527,43 +1549,43 @@
         <v>1</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L7" s="1">
-        <v>46037</v>
+      <c r="L7" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>79</v>
+        <v>27</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="O7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="P7" s="2"/>
     </row>
-    <row r="8" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="10">
         <v>2026</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>149</v>
+        <v>71</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>159</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="F8" s="11" t="b">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G8:I8,TRUE),_xlpm.av,COUNTIF(G8:I8,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
       <c r="G8" s="11" t="b">
@@ -1576,117 +1598,117 @@
         <v>1</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="K8" s="1">
-        <v>45980</v>
+        <v>46197</v>
       </c>
       <c r="L8" s="1">
-        <v>46010</v>
+        <v>46219</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>106</v>
+        <v>172</v>
       </c>
       <c r="P8" s="3"/>
     </row>
-    <row r="9" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="10">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>150</v>
+        <v>55</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>167</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="F9" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>À vérifier</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>5</v>
+        <v>114</v>
+      </c>
+      <c r="F9" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G9:I9,TRUE),_xlpm.av,COUNTIF(G9:I9,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
+      </c>
+      <c r="G9" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" s="11" t="b">
+        <v>1</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="K9" s="1">
-        <v>45947</v>
+        <v>46202</v>
       </c>
       <c r="L9" s="1">
-        <v>46007</v>
+        <v>46212</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>81</v>
+        <v>47</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="O9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="10">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>À vérifier</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="L10" s="4">
-        <v>45673</v>
+        <v>194</v>
+      </c>
+      <c r="F10" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G10:I10,TRUE),_xlpm.av,COUNTIF(G10:I10,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
+      </c>
+      <c r="G10" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K10" s="1">
+        <v>45813</v>
+      </c>
+      <c r="L10" s="1">
+        <v>46181</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="O10" s="5" t="s">
         <v>11</v>
@@ -1695,26 +1717,26 @@
     </row>
     <row r="11" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="10">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>151</v>
+        <v>67</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>148</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>127</v>
       </c>
       <c r="F11" s="11" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G11:I11,TRUE),_xlpm.av,COUNTIF(G11:I11,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G11" s="11" t="s">
-        <v>5</v>
+      <c r="G11" s="11" t="b">
+        <v>1</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>5</v>
@@ -1723,143 +1745,142 @@
         <v>5</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="K11" s="1">
-        <v>45947</v>
+        <v>46041</v>
       </c>
       <c r="L11" s="1">
-        <v>46007</v>
+        <v>46048</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="P11" s="2"/>
     </row>
-    <row r="12" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="10">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>152</v>
+        <v>72</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>170</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="F12" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>À vérifier</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I12" s="11" t="s">
-        <v>5</v>
+        <v>183</v>
+      </c>
+      <c r="F12" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G12:I12,TRUE),_xlpm.av,COUNTIF(G12:I12,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11" t="b">
+        <v>1</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="K12" s="1">
-        <v>45813</v>
+        <v>94</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="L12" s="1">
-        <f>DATE(2025,7,24)</f>
-        <v>45862</v>
+        <v>46037</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>77</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="O12" s="2" t="s">
         <v>11</v>
       </c>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="10">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>129</v>
+        <v>9</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>145</v>
       </c>
       <c r="F13" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G13:I13,TRUE),_xlpm.av,COUNTIF(G13:I13,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
       </c>
       <c r="G13" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>97</v>
+        <v>146</v>
       </c>
       <c r="K13" s="1">
-        <v>45708</v>
+        <v>45989</v>
       </c>
       <c r="L13" s="1">
-        <v>45930</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="P13" s="3"/>
+        <v>46010</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="O13" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="P13" s="5"/>
     </row>
-    <row r="14" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="21" t="s">
-        <v>185</v>
+      <c r="D14" s="20" t="s">
+        <v>169</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="F14" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G14:I14,TRUE),_xlpm.av,COUNTIF(G14:I14,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
       </c>
       <c r="G14" s="11" t="b">
         <v>0</v>
@@ -1868,99 +1889,99 @@
         <v>1</v>
       </c>
       <c r="I14" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="K14" s="1">
-        <v>45684</v>
+        <v>45980</v>
       </c>
       <c r="L14" s="1">
-        <v>45743</v>
+        <v>46010</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>109</v>
+        <v>173</v>
       </c>
       <c r="P14" s="3"/>
     </row>
-    <row r="15" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="10">
         <v>2025</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>154</v>
+        <v>57</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>164</v>
       </c>
       <c r="E15" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" s="11" t="str">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G15:I15,TRUE),_xlpm.av,COUNTIF(G15:I15,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>À vérifier</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K15" s="1">
+        <v>45947</v>
+      </c>
+      <c r="L15" s="1">
+        <v>46007</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F15" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G15" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="H15" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I15" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="K15" s="1">
-        <v>45680</v>
-      </c>
-      <c r="L15" s="1">
-        <v>45712</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="P15" s="3"/>
+      <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="10">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>155</v>
+        <v>56</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>165</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="F16" s="11" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G16:I16,TRUE),_xlpm.av,COUNTIF(G16:I16,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G16" s="11" t="b">
-        <v>0</v>
+      <c r="G16" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="H16" s="11" t="s">
         <v>5</v>
@@ -1969,166 +1990,167 @@
         <v>5</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>5</v>
+        <v>103</v>
+      </c>
+      <c r="K16" s="1">
+        <v>45947</v>
       </c>
       <c r="L16" s="1">
-        <v>45538</v>
+        <v>46007</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="O16" s="2" t="s">
         <v>11</v>
       </c>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="10">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>156</v>
+        <v>59</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>150</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>132</v>
+        <v>184</v>
       </c>
       <c r="F17" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G17:I17,TRUE),_xlpm.av,COUNTIF(G17:I17,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>0</v>
       </c>
       <c r="G17" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>5</v>
+        <v>95</v>
+      </c>
+      <c r="K17" s="1">
+        <v>45708</v>
       </c>
       <c r="L17" s="1">
-        <v>45337</v>
+        <v>45930</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>119</v>
+        <v>174</v>
       </c>
       <c r="P17" s="3"/>
     </row>
     <row r="18" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="10">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="F18" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G18" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I18" s="11" t="b">
-        <v>1</v>
+        <v>118</v>
+      </c>
+      <c r="F18" s="11" t="str">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G18:I18,TRUE),_xlpm.av,COUNTIF(G18:I18,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>À vérifier</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K18" s="1">
-        <v>45702</v>
+        <v>45813</v>
       </c>
       <c r="L18" s="1">
-        <v>45744</v>
+        <f>DATE(2025,7,24)</f>
+        <v>45862</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="O18" s="2" t="s">
         <v>11</v>
       </c>
       <c r="P18" s="2"/>
     </row>
-    <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="10">
         <v>2024</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>167</v>
+        <v>63</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>134</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>À vérifier</v>
+        <v>122</v>
+      </c>
+      <c r="F19" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G19:I19,TRUE),_xlpm.av,COUNTIF(G19:I19,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
       </c>
       <c r="G19" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="H19" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>5</v>
+      <c r="H19" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" s="11" t="b">
+        <v>1</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>5</v>
+        <v>97</v>
+      </c>
+      <c r="K19" s="1">
+        <v>45702</v>
+      </c>
+      <c r="L19" s="1">
+        <v>45744</v>
       </c>
       <c r="M19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="O19" s="2" t="s">
         <v>11</v>
@@ -2137,75 +2159,75 @@
     </row>
     <row r="20" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="10">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="F20" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G20:I20,TRUE),_xlpm.av,COUNTIF(G20:I20,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>0</v>
       </c>
       <c r="G20" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="11" t="b">
         <v>1</v>
       </c>
       <c r="I20" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>5</v>
+        <v>96</v>
+      </c>
+      <c r="K20" s="1">
+        <v>45684</v>
+      </c>
+      <c r="L20" s="1">
+        <v>45743</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P20" s="2"/>
+        <v>35</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="P20" s="3"/>
     </row>
-    <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" s="10">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>159</v>
+        <v>60</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>154</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>140</v>
+        <v>185</v>
       </c>
       <c r="F21" s="11" t="b">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G21:I21,TRUE),_xlpm.av,COUNTIF(G21:I21,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
       <c r="G21" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" s="11" t="b">
         <v>1</v>
@@ -2214,92 +2236,92 @@
         <v>1</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K21" s="1">
-        <v>45356</v>
+        <v>45680</v>
       </c>
       <c r="L21" s="1">
-        <v>45401</v>
+        <v>45712</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>120</v>
+        <v>176</v>
       </c>
       <c r="P21" s="3"/>
     </row>
-    <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="E22" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="F22" s="11" t="str">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G22:I22,TRUE),_xlpm.av,COUNTIF(G22:I22,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>À vérifier</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L22" s="4">
+        <v>45673</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="N22" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="O22" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F22" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>À vérifier</v>
-      </c>
-      <c r="G22" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I22" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P22" s="2"/>
+      <c r="P22" s="5"/>
     </row>
     <row r="23" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="10">
         <v>2024</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="18" t="s">
-        <v>161</v>
+      <c r="D23" s="20" t="s">
+        <v>162</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="F23" s="11" t="b">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G23:I23,TRUE),_xlpm.av,COUNTIF(G23:I23,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
       <c r="G23" s="11" t="b">
@@ -2312,7 +2334,7 @@
         <v>1</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="K23" s="1">
         <v>45569</v>
@@ -2321,38 +2343,38 @@
         <v>45610</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>11</v>
       </c>
       <c r="P23" s="2"/>
     </row>
-    <row r="24" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="10">
         <v>2024</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>170</v>
+        <v>61</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>171</v>
+        <v>120</v>
       </c>
       <c r="F24" s="11" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G24:I24,TRUE),_xlpm.av,COUNTIF(G24:I24,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G24" s="11" t="s">
-        <v>5</v>
+      <c r="G24" s="11" t="b">
+        <v>0</v>
       </c>
       <c r="H24" s="11" t="s">
         <v>5</v>
@@ -2361,236 +2383,236 @@
         <v>5</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="K24" s="1">
-        <v>45266</v>
+        <v>103</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="L24" s="1">
-        <v>45337</v>
+        <v>45538</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>172</v>
+        <v>32</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>173</v>
+        <v>33</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>174</v>
+        <v>11</v>
       </c>
       <c r="P24" s="2"/>
     </row>
-    <row r="25" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="10">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>162</v>
+        <v>8</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>157</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="F25" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>À vérifier</v>
-      </c>
-      <c r="G25" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I25" s="11" t="s">
-        <v>5</v>
+        <v>128</v>
+      </c>
+      <c r="F25" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G25:I25,TRUE),_xlpm.av,COUNTIF(G25:I25,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
+      </c>
+      <c r="G25" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" s="11" t="b">
+        <v>1</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>5</v>
+        <v>99</v>
+      </c>
+      <c r="K25" s="1">
+        <v>45356</v>
+      </c>
+      <c r="L25" s="1">
+        <v>45401</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="O25" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P25" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="O25" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="P25" s="3"/>
     </row>
     <row r="26" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="10">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D26" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="F26" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G26:I26,TRUE),_xlpm.av,COUNTIF(G26:I26,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
+      </c>
+      <c r="G26" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L26" s="1">
+        <v>45337</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O26" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="P26" s="3"/>
+    </row>
+    <row r="27" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="E26" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="F26" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G26" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H26" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I26" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L26" s="1">
-        <v>45259</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P26" s="2"/>
+      <c r="E27" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="F27" s="11" t="str">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G27:I27,TRUE),_xlpm.av,COUNTIF(G27:I27,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>À vérifier</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K27" s="1">
+        <v>45266</v>
+      </c>
+      <c r="L27" s="1">
+        <v>45337</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="O27" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="P27" s="2"/>
     </row>
-    <row r="27" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A27" s="10">
-        <v>2023</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" s="11" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G27" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H27" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I27" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L27" s="1">
-        <v>45111</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="O27" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="P27" s="3"/>
-    </row>
-    <row r="28" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="10">
         <v>2023</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>186</v>
+        <v>65</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>156</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="F28" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>À vérifier</v>
+        <v>129</v>
+      </c>
+      <c r="F28" s="11" t="b">
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G28:I28,TRUE),_xlpm.av,COUNTIF(G28:I28,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
+        <v>1</v>
       </c>
       <c r="G28" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I28" s="11" t="s">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="H28" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" s="11" t="b">
+        <v>1</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L28" s="1" t="s">
-        <v>5</v>
+      <c r="L28" s="1">
+        <v>45259</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="N28" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="O28" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P28" s="3"/>
+      <c r="O28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="P28" s="2"/>
     </row>
     <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10">
         <v>2023</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="F29" s="11" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G29:I29,TRUE),_xlpm.av,COUNTIF(G29:I29,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
@@ -2603,25 +2625,25 @@
         <v>1</v>
       </c>
       <c r="I29" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>177</v>
+        <v>101</v>
       </c>
       <c r="K29" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L29" s="1" t="s">
-        <v>5</v>
+      <c r="L29" s="1">
+        <v>45111</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>178</v>
+        <v>86</v>
       </c>
       <c r="N29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O29" s="3" t="s">
         <v>179</v>
-      </c>
-      <c r="O29" s="3" t="s">
-        <v>11</v>
       </c>
       <c r="P29" s="3"/>
     </row>
@@ -2630,19 +2652,19 @@
         <v>2023</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="21" t="s">
-        <v>165</v>
+      <c r="D30" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="F30" s="11" t="b">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G30:I30,TRUE),_xlpm.av,COUNTIF(G30:I30,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
       <c r="G30" s="11" t="b">
@@ -2655,7 +2677,7 @@
         <v>1</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="K30" s="1">
         <v>44845</v>
@@ -2664,13 +2686,13 @@
         <v>45028</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N30" s="2" t="s">
         <v>18</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>19</v>
+        <v>180</v>
       </c>
       <c r="P30" s="3"/>
     </row>
@@ -2679,19 +2701,19 @@
         <v>2023</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>166</v>
+        <v>66</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>153</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="F31" s="11" t="b">
-        <f t="shared" si="0"/>
+        <f>_xlfn.LET(_xlpm.ok,COUNTIF(G31:I31,TRUE),_xlpm.av,COUNTIF(G31:I31,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
       <c r="G31" s="11" t="b">
@@ -2704,7 +2726,7 @@
         <v>1</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>5</v>
@@ -2714,10 +2736,10 @@
         <v>44882</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O31" s="2" t="s">
         <v>11</v>
@@ -2725,7 +2747,14 @@
       <c r="P31" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P31" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P31" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P31">
+      <sortCondition descending="1" ref="L2:L31"/>
+    </sortState>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P31">
+    <sortCondition descending="1" ref="L2:L31"/>
+  </sortState>
   <conditionalFormatting sqref="A2:P31">
     <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",A2)))</formula>
@@ -2757,24 +2786,36 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="O4" r:id="rId1" display="Votre ressenti pour la RCC 2026-2 (26/06/2026)" xr:uid="{59D95BD5-7957-4DC2-9292-2CBBBB953C0D}"/>
-    <hyperlink ref="O8" r:id="rId2" xr:uid="{B5450024-F62E-4456-B70D-13EE54625FA9}"/>
-    <hyperlink ref="O13" r:id="rId3" display="Rappel dans le tract RCC de novembre 2025" xr:uid="{8A361D52-2C0D-4A5E-B963-5A59F5A00104}"/>
-    <hyperlink ref="O14" r:id="rId4" display="Salaires : les négos ça ne marche pas (26/03/2025)" xr:uid="{5D4473E7-1C88-48FE-A14D-A15093F3B79B}"/>
-    <hyperlink ref="O15" r:id="rId5" display="Avenant Télétravail : signer pour 40 centimes ? (19/02/2025)" xr:uid="{558A19AF-8D80-4D08-ABC2-4A3E7D1CD93A}"/>
-    <hyperlink ref="O17" r:id="rId6" display="Et toi alors, t'es coté combien ? (13/11/2023)" xr:uid="{01E3DB2C-8C96-4A47-9002-9C3BFBFA84FF}"/>
-    <hyperlink ref="O21" r:id="rId7" display="Bilan de la RCC 2024 (06/11/2024) ; " xr:uid="{22B006CE-6E87-4246-B4EA-8BA01364E20A}"/>
-    <hyperlink ref="O27" r:id="rId8" display="RCC : des motifs de vigilance (09/2023) ; " xr:uid="{065592F7-3619-4EE0-A07C-438E248C4E8F}"/>
-    <hyperlink ref="O28" r:id="rId9" xr:uid="{FF1EF8E1-6A04-432C-8713-D23076AA8098}"/>
-    <hyperlink ref="O30" r:id="rId10" xr:uid="{1699107D-21CE-4FF6-AE63-2552D0557C45}"/>
-    <hyperlink ref="D4" r:id="rId11" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?id=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026/Accord_RCC_2026.pdf&amp;parent=/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026" xr:uid="{2EC36556-9A1E-448F-990C-1BFE28A28515}"/>
-    <hyperlink ref="D20" r:id="rId12" xr:uid="{A9AF55B6-9AF4-441B-BF54-A1A9640D2C9D}"/>
-    <hyperlink ref="D24" r:id="rId13" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/PV%20D%C3%A9saccord%20NAO%202024%20(15%20f%C3%A9vrier%202024).pdf?d=waee681ffe1e04075ad0db67395d7487a&amp;csf=1&amp;web=1&amp;e=B4eck9," xr:uid="{F6B82D88-92B4-4369-B825-E6CFE444F804}"/>
-    <hyperlink ref="D29" r:id="rId14" xr:uid="{C043EA89-0A53-4B71-AC0C-5C4306E62617}"/>
-    <hyperlink ref="D10" r:id="rId15" xr:uid="{5C4C6E25-614E-4F25-8AA8-26F96EA1D6FC}"/>
+    <hyperlink ref="D8" r:id="rId1" xr:uid="{2EC36556-9A1E-448F-990C-1BFE28A28515}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{A9AF55B6-9AF4-441B-BF54-A1A9640D2C9D}"/>
+    <hyperlink ref="D27" r:id="rId3" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Avenant%20Proc%C3%A8s-verbal%20de%20d%C3%A9saccord%20NAO%202024%20(9%20avril%202024).pdf" xr:uid="{F6B82D88-92B4-4369-B825-E6CFE444F804}"/>
+    <hyperlink ref="D17" r:id="rId4" xr:uid="{6A46598A-BCC9-4794-AE14-7CBA11E19EBB}"/>
+    <hyperlink ref="D22" r:id="rId5" xr:uid="{5C4C6E25-614E-4F25-8AA8-26F96EA1D6FC}"/>
+    <hyperlink ref="D30" r:id="rId6" xr:uid="{B32EB3EF-DF8F-4ACB-9052-ED0420F2EB20}"/>
+    <hyperlink ref="D3" r:id="rId7" xr:uid="{38397C78-3308-4427-88D7-4FD669271978}"/>
+    <hyperlink ref="D24" r:id="rId8" xr:uid="{C9C0BF18-CF80-4BAF-B84A-71DFE1F4CEF1}"/>
+    <hyperlink ref="D5" r:id="rId9" xr:uid="{C043EA89-0A53-4B71-AC0C-5C4306E62617}"/>
+    <hyperlink ref="D31" r:id="rId10" xr:uid="{9603D9FE-6A53-4857-AF9A-7B4CEFEEA9BC}"/>
+    <hyperlink ref="D9" r:id="rId11" xr:uid="{82282E9B-CCA9-434A-AE8B-F46BDD379264}"/>
+    <hyperlink ref="D11" r:id="rId12" xr:uid="{9C779CF0-9D36-4133-B425-014C0E592614}"/>
+    <hyperlink ref="D12" r:id="rId13" xr:uid="{1CAF7A33-3FE3-42CD-B630-103D55FCDBB0}"/>
+    <hyperlink ref="D10" r:id="rId14" xr:uid="{85C39618-C574-4EEC-8C06-0BC340D4273B}"/>
+    <hyperlink ref="D13" r:id="rId15" xr:uid="{E88B21CF-4C2B-47AB-B153-EB4D68F183C9}"/>
+    <hyperlink ref="D15" r:id="rId16" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Entreprise%20au%20sein%20de%20Nokia%20Networks%20France%20(16%20d%c3%a9cembre%202025).pdf" xr:uid="{BF514F36-2459-4883-A6C8-AB19CDC9D51E}"/>
+    <hyperlink ref="D6" r:id="rId17" xr:uid="{4293582A-4729-404B-A1F9-27BD5C6AE9EF}"/>
+    <hyperlink ref="D20" r:id="rId18" xr:uid="{66CCDBE2-5BD8-413A-AB11-C366112FA221}"/>
+    <hyperlink ref="D21" r:id="rId19" xr:uid="{7BD096EF-D447-4D18-8E0D-8B7CA7667DD0}"/>
+    <hyperlink ref="D29" r:id="rId20" xr:uid="{1DF5F389-89B7-4CD3-9441-863D74582C91}"/>
+    <hyperlink ref="D28" r:id="rId21" xr:uid="{4269F357-C8F2-420C-B59A-A22ABA10DA95}"/>
+    <hyperlink ref="D25" r:id="rId22" xr:uid="{E700AC18-B723-46FB-8F25-E39C3349C173}"/>
+    <hyperlink ref="D4" r:id="rId23" xr:uid="{AC32DDA2-E891-4AAF-A605-5D7F14DCCD21}"/>
+    <hyperlink ref="D23" r:id="rId24" xr:uid="{29A2B983-F112-4EE6-9B44-0F1CB988C6C1}"/>
+    <hyperlink ref="D16" r:id="rId25" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Retraite%20d'Entreprise%20Collectif%20PERCOL%20(16%20d%c3%a9cembre%202025).pdf" xr:uid="{ADB6C391-B664-442C-84BE-32EB612092D0}"/>
+    <hyperlink ref="D14" r:id="rId26" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Accord%20collectif%20portant%20sur%20une%20Rupture%20Conventionnelle%20Collective%20(RCC)%20au%20sein%20de%20Nokia%20Networks%20France%20(compress%c3%a9).pdf" xr:uid="{CDF018D6-A914-4E6F-BC99-C9BC7058618D}"/>
+    <hyperlink ref="O27" r:id="rId27" xr:uid="{795404A2-F15F-4A6A-94CF-0EC12677A11E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId16"/>
+  <pageSetup orientation="portrait" r:id="rId28"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
   </headerFooter>
@@ -2795,31 +2836,10 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
-    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
-    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
-      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
-      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -3090,9 +3110,30 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
+    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
+    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
+      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
+      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3146,25 +3187,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
-    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3184,10 +3214,21 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
+    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add signature capture links and simplify titles
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1436" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52B98D3D-5680-4D95-9DF0-AE8DAACC3B7D}"/>
+  <xr:revisionPtr revIDLastSave="1582" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB48B3DE-F597-4F07-BACB-FF00FFB411E5}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="227">
   <si>
     <t>Accord ou négociation</t>
   </si>
@@ -69,9 +69,6 @@
     <t>RCC 2024</t>
   </si>
   <si>
-    <t>Aménagement du temps de travail</t>
-  </si>
-  <si>
     <t>Déplacements du personnel itinérant</t>
   </si>
   <si>
@@ -207,9 +204,6 @@
     <t>Handicap</t>
   </si>
   <si>
-    <t>Avenant nº 1 – CSE (21 septembre 2018)</t>
-  </si>
-  <si>
     <t>Plan d'Epargne Retraite d'Entreprise Collectif (PERCOL)</t>
   </si>
   <si>
@@ -222,15 +216,9 @@
     <t>GEPP – PV de désaccord</t>
   </si>
   <si>
-    <t>Avenant télétravail (avril 2022)</t>
-  </si>
-  <si>
     <t>Partage de la valeur – PV de désaccord</t>
   </si>
   <si>
-    <t>Nouvelle convention collective (accord-cadre)</t>
-  </si>
-  <si>
     <t>Intéressement 2025-2028</t>
   </si>
   <si>
@@ -243,24 +231,9 @@
     <t>Remboursement santé</t>
   </si>
   <si>
-    <t>NAO 2026 – Procès-verbal d'accord</t>
-  </si>
-  <si>
-    <t>NAO 2025 – PV de désaccord</t>
-  </si>
-  <si>
-    <t>NAO 2023 – PV de désaccord</t>
-  </si>
-  <si>
-    <t>RCC 2026 n°1 (signée en décembre 2025)</t>
-  </si>
-  <si>
     <t>RCC 2026 n°2</t>
   </si>
   <si>
-    <t>Avenant à la RCC 2026 n°1</t>
-  </si>
-  <si>
     <t>Renouvellement de la politique handicap NNF (1er accord agréé en 2006 ; taux d'emploi &gt; 6 % depuis 2020). Rôles des acteurs : salariés, people managers, santé au travail, service social, Mission handicap. Négocié du 5 juin 2025 au 16 février 2026. Avancée principale : cotisations retraite prises en charge à 100 % en temps partiel choisi (TPC).</t>
   </si>
   <si>
@@ -435,9 +408,6 @@
     <t>Validité</t>
   </si>
   <si>
-    <t>preview pdf</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20CET%20(24%20juillet%202025).pdf</t>
   </si>
   <si>
@@ -456,9 +426,6 @@
     <t>URL</t>
   </si>
   <si>
-    <t>NAO 2024 – PV de désaccord</t>
-  </si>
-  <si>
     <t>Pas d'accord : PV de désaccord NAO 2024 (dernière réunion le 07-08/02/2024), puis avenant au PV négocié le 02/04/2024. Augmentation moyenne jugée « pitoyable » ; mobilisation intersyndicale CFDT / CFE-CGC / CGT en mars 2024.</t>
   </si>
   <si>
@@ -552,9 +519,6 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Accord%20collectif%20portant%20sur%20une%20Rupture%20Conventionnelle%20Collective%20(RCC)%20au%20sein%20de%20Nokia%20Networks%20France%20(compress%c3%a9).pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Avenant%20RCC%202025.pdf</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salariés/tracts%20diffusés/2023/Tract%20brèves%20de%20printemps.pdf</t>
   </si>
   <si>
@@ -591,6 +555,9 @@
     <t>Accord établissement aménagement temps de travail 2022.pdf</t>
   </si>
   <si>
+    <t>Accord handicap 2026.pdf</t>
+  </si>
+  <si>
     <t>Avenant RCC 2025.pdf</t>
   </si>
   <si>
@@ -615,16 +582,145 @@
     <t>Accord harmonisation taux variable cible.pdf</t>
   </si>
   <si>
-    <t>Accord collectif portant sur l’harmonisation des taux de variable cible des salariés « non sales » au regard de leur job grade</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/Accord%20harmonisation%20taux%20variable%20cible.pdf</t>
   </si>
   <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/2025%20Accord%20etablissement%20NAO%20Mis%20%C3%A0%20la%20signature.pdf</t>
   </si>
   <si>
-    <t>ACCORD HANDICAP VERSION REVUE LE 8 juin 2026.pdf</t>
+    <t>page signature</t>
+  </si>
+  <si>
+    <t>RCC 2026 n°1</t>
+  </si>
+  <si>
+    <t>Aménagement du temps de travail 2026</t>
+  </si>
+  <si>
+    <t>Avenant RCC 2026 n°1</t>
+  </si>
+  <si>
+    <t>NAO 2026</t>
+  </si>
+  <si>
+    <t>NAO 2024</t>
+  </si>
+  <si>
+    <t>NAO 2025</t>
+  </si>
+  <si>
+    <t>Aménagement du temps de travail 2024</t>
+  </si>
+  <si>
+    <t>NAO 2023</t>
+  </si>
+  <si>
+    <t>Aménagement du temps de travail 2023</t>
+  </si>
+  <si>
+    <t>Avenant télétravail</t>
+  </si>
+  <si>
+    <t>Aménagement du temps de travail 2025</t>
+  </si>
+  <si>
+    <t>Nouvelle convention collective</t>
+  </si>
+  <si>
+    <t>Harmonisation du taux de bonus</t>
+  </si>
+  <si>
+    <t>Avenant CSE</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Avenant%20RCC%202025.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_Harmonisation_TI_final_p10.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CGF_p10_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_etablissement_amenagement_temps_de_travail_2022_p04_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_NAO_2023_PV_desaccord_p10.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2024_p04_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2026_p54_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_no_1_a_l_Accord_CSE_du_21_septembre_2018_p10_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_handicap_2026_p15-16_signatures.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2026_Proces_verbal_d_accord_24_janvier_2026_p07_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_RCC_2025_p07_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Amenagement_Temps_Travail_NPS_2026_19_decembre_2025_p03_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_collectif_portant_sur_une_Rupture_Conventionnelle_Collective_RCC__p52_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Entreprise_au_sein_de_Noki_p17-18_signatures.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Retraite_d_Entreprise_Coll_p20-21_signatures.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_GEPP_PV_de_desaccord_mis_a_signature_p12_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CET_24_juillet_2025_p13-14_signatures.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_interessement_2025_2028_p16_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_Proces_verbal_NAO_desaccord_2025_27_mars_2025_p11_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_accord_teletravail_avril_2022_p07_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_NPS_2025_accord_mis_a_signature_p4.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_don_de_jours_14_novembre_2024_p11_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_Partage_valeur_PV_p6.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2024_19_avril_2024_p47_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_cadre_NPS_nouvelle_convention_collective_2024_signe_p06_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Proces_verbal_de_desaccord_NAO_2024_9_avril_2024_p05_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_de_substitution_non_cadres_30_novembre_2023_p09_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2023_p49_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_Accord_egalite_professionnelle_p20_signature.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_remboursement_sante_2023_p11_signature.jpg</t>
   </si>
 </sst>
 </file>
@@ -777,15 +873,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -845,6 +938,22 @@
     <xf numFmtId="49" fontId="2" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1206,1554 +1315,1612 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultColWidth="12.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="41.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="114.28515625" style="21" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" style="9" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" style="9" customWidth="1"/>
-    <col min="7" max="9" width="9.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="49.5703125" style="9" customWidth="1"/>
-    <col min="11" max="12" width="14.28515625" style="9" customWidth="1"/>
-    <col min="13" max="14" width="57.140625" style="9" customWidth="1"/>
-    <col min="15" max="15" width="82.140625" style="9" customWidth="1"/>
-    <col min="16" max="16" width="41.85546875" style="9" customWidth="1"/>
-    <col min="17" max="16384" width="12.140625" style="9"/>
+    <col min="1" max="1" width="8.28515625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27" style="20" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" style="8" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="8" customWidth="1"/>
+    <col min="7" max="9" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="41.85546875" style="8" customWidth="1"/>
+    <col min="11" max="11" width="49.5703125" style="8" customWidth="1"/>
+    <col min="12" max="13" width="14.28515625" style="8" customWidth="1"/>
+    <col min="14" max="15" width="57.140625" style="8" customWidth="1"/>
+    <col min="16" max="16" width="55.85546875" style="26" customWidth="1"/>
+    <col min="18" max="16384" width="12.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="L1" s="8" t="s">
+      <c r="O1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="N1" s="8" t="s">
+      <c r="P1" s="22" t="s">
         <v>16</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="10">
+      <c r="A2" s="9">
         <v>2024</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="12" t="s">
+      <c r="B2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="11" t="str">
+      <c r="F2" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G2:I2,TRUE),_xlpm.av,COUNTIF(G2:I2,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G2" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>98</v>
-      </c>
+      <c r="G2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="2"/>
       <c r="K2" s="1" t="s">
-        <v>5</v>
+        <v>89</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>29</v>
+      <c r="M2" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P2" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="P2" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="3" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="10">
+    <row r="3" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
         <v>2023</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>191</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>192</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="F3" s="11" t="str">
+      <c r="B3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="F3" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G3:I3,TRUE),_xlpm.av,COUNTIF(G3:I3,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>103</v>
+      <c r="G3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" s="27" t="s">
+        <v>198</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>5</v>
+        <v>94</v>
       </c>
       <c r="L3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>21</v>
+      <c r="M3" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P3" s="2"/>
+        <v>5</v>
+      </c>
+      <c r="P3" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="10">
+      <c r="A4" s="9">
         <v>2024</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>158</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="F4" s="11" t="str">
+      <c r="B4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="F4" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G4:I4,TRUE),_xlpm.av,COUNTIF(G4:I4,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G4" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>98</v>
+      <c r="G4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="27" t="s">
+        <v>199</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>5</v>
+        <v>89</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="N4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P4" s="2"/>
+      <c r="P4" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="5" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="10">
+      <c r="A5" s="9">
         <v>2023</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="F5" s="11" t="b">
+      <c r="B5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G5:I5,TRUE),_xlpm.av,COUNTIF(G5:I5,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G5" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>141</v>
+      <c r="G5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="27" t="s">
+        <v>200</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>5</v>
+        <v>130</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M5" s="2" t="s">
-        <v>142</v>
+      <c r="M5" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="P5" s="3"/>
+        <v>131</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="P5" s="24" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="6" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="10">
+      <c r="A6" s="9">
         <v>2023</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="F6" s="11" t="str">
+      <c r="B6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F6" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G6:I6,TRUE),_xlpm.av,COUNTIF(G6:I6,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G6" s="11" t="b">
+      <c r="G6" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I6" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>103</v>
+      <c r="H6" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J6" s="27" t="s">
+        <v>201</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>5</v>
+        <v>94</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M6" s="2" t="s">
-        <v>19</v>
+      <c r="M6" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="P6" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" s="24" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="7" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="10">
+      <c r="A7" s="9">
         <v>2024</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="11" t="b">
+      <c r="B7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="F7" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G7:I7,TRUE),_xlpm.av,COUNTIF(G7:I7,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G7" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>108</v>
+      <c r="G7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" s="27" t="s">
+        <v>202</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="O7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P7" s="2"/>
+      <c r="P7" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="8" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="10">
+      <c r="A8" s="9">
         <v>2026</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="F8" s="11" t="b">
+      <c r="B8" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G8:I8,TRUE),_xlpm.av,COUNTIF(G8:I8,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G8" s="11" t="b">
+      <c r="G8" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="K8" s="1">
+      <c r="H8" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L8" s="1">
         <v>46197</v>
       </c>
-      <c r="L8" s="1">
+      <c r="M8" s="1">
         <v>46219</v>
       </c>
-      <c r="M8" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="N8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="P8" s="3"/>
+        <v>47</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P8" s="24" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="9" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="10">
+      <c r="A9" s="9">
         <v>2026</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>167</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="F9" s="11" t="b">
+      <c r="B9" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G9:I9,TRUE),_xlpm.av,COUNTIF(G9:I9,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G9" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="K9" s="1">
+      <c r="G9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" s="27" t="s">
+        <v>204</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L9" s="1">
         <v>46202</v>
       </c>
-      <c r="L9" s="1">
+      <c r="M9" s="1">
         <v>46212</v>
       </c>
-      <c r="M9" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="N9" s="2" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P9" s="2"/>
+        <v>29</v>
+      </c>
+      <c r="P9" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="10" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
+      <c r="A10" s="9">
         <v>2026</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="F10" s="11" t="b">
+      <c r="B10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="F10" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G10:I10,TRUE),_xlpm.av,COUNTIF(G10:I10,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G10" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="K10" s="1">
+      <c r="G10" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="27" t="s">
+        <v>205</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L10" s="1">
         <v>45813</v>
       </c>
-      <c r="L10" s="1">
+      <c r="M10" s="1">
         <v>46181</v>
       </c>
-      <c r="M10" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="N10" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="O10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="P10" s="5"/>
+      <c r="N10" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P10" s="25" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A11" s="10">
+      <c r="A11" s="9">
         <v>2026</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>148</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="F11" s="11" t="str">
+      <c r="B11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G11:I11,TRUE),_xlpm.av,COUNTIF(G11:I11,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="K11" s="1">
+      <c r="G11" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J11" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L11" s="1">
         <v>46041</v>
       </c>
-      <c r="L11" s="1">
+      <c r="M11" s="1">
         <v>46048</v>
       </c>
-      <c r="M11" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="N11" s="2" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P11" s="2"/>
+        <v>45</v>
+      </c>
+      <c r="P11" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="12" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" s="10">
+      <c r="A12" s="9">
         <v>2026</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>170</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="F12" s="11" t="b">
+      <c r="B12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="F12" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G12:I12,TRUE),_xlpm.av,COUNTIF(G12:I12,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G12" s="11" t="b">
+      <c r="G12" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>94</v>
+      <c r="H12" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" s="27" t="s">
+        <v>207</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L12" s="1">
+        <v>85</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M12" s="1">
         <v>46037</v>
       </c>
-      <c r="M12" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="N12" s="2" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P12" s="2"/>
+        <v>39</v>
+      </c>
+      <c r="P12" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="13" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A13" s="10">
+      <c r="A13" s="9">
         <v>2026</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="F13" s="11" t="b">
+      <c r="B13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="F13" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G13:I13,TRUE),_xlpm.av,COUNTIF(G13:I13,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G13" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="K13" s="1">
+      <c r="G13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" s="27" t="s">
+        <v>208</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="L13" s="1">
         <v>45989</v>
       </c>
-      <c r="L13" s="1">
+      <c r="M13" s="1">
         <v>46010</v>
       </c>
-      <c r="M13" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="N13" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="O13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="P13" s="5"/>
+      <c r="N13" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P13" s="25" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="14" spans="1:16" ht="120" x14ac:dyDescent="0.25">
-      <c r="A14" s="10">
+      <c r="A14" s="9">
         <v>2026</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>169</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="F14" s="11" t="b">
+      <c r="B14" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F14" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G14:I14,TRUE),_xlpm.av,COUNTIF(G14:I14,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G14" s="11" t="b">
+      <c r="G14" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="K14" s="1">
+      <c r="H14" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="L14" s="1">
         <v>45980</v>
       </c>
-      <c r="L14" s="1">
+      <c r="M14" s="1">
         <v>46010</v>
       </c>
-      <c r="M14" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="N14" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="P14" s="3"/>
+        <v>69</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P14" s="24" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="15" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A15" s="10">
+      <c r="A15" s="9">
         <v>2025</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>164</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="F15" s="11" t="str">
+      <c r="B15" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="F15" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G15:I15,TRUE),_xlpm.av,COUNTIF(G15:I15,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G15" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H15" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K15" s="1">
+      <c r="G15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J15" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L15" s="1">
         <v>45947</v>
       </c>
-      <c r="L15" s="1">
+      <c r="M15" s="1">
         <v>46007</v>
       </c>
-      <c r="M15" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="N15" s="2" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P15" s="2"/>
+        <v>36</v>
+      </c>
+      <c r="P15" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="16" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A16" s="10">
+      <c r="A16" s="9">
         <v>2025</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>165</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="F16" s="11" t="str">
+      <c r="B16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="F16" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G16:I16,TRUE),_xlpm.av,COUNTIF(G16:I16,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G16" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K16" s="1">
+      <c r="G16" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J16" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L16" s="1">
         <v>45947</v>
       </c>
-      <c r="L16" s="1">
+      <c r="M16" s="1">
         <v>46007</v>
       </c>
-      <c r="M16" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="N16" s="2" t="s">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P16" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="P16" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="17" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="10">
+      <c r="A17" s="9">
         <v>2025</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="F17" s="11" t="b">
+      <c r="B17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="F17" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G17:I17,TRUE),_xlpm.av,COUNTIF(G17:I17,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>0</v>
       </c>
-      <c r="G17" s="11" t="b">
+      <c r="G17" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H17" s="11" t="b">
+      <c r="H17" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I17" s="11" t="b">
+      <c r="I17" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="K17" s="1">
+      <c r="J17" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L17" s="1">
         <v>45708</v>
       </c>
-      <c r="L17" s="1">
+      <c r="M17" s="1">
         <v>45930</v>
       </c>
-      <c r="M17" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="N17" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="P17" s="3"/>
+        <v>72</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="P17" s="24" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="18" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="10">
+      <c r="A18" s="9">
         <v>2025</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="F18" s="11" t="str">
+      <c r="B18" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="F18" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G18:I18,TRUE),_xlpm.av,COUNTIF(G18:I18,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G18" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K18" s="1">
+      <c r="G18" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J18" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L18" s="1">
         <v>45813</v>
       </c>
-      <c r="L18" s="1">
+      <c r="M18" s="1">
         <f>DATE(2025,7,24)</f>
         <v>45862</v>
       </c>
-      <c r="M18" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="N18" s="2" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P18" s="2"/>
+        <v>44</v>
+      </c>
+      <c r="P18" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A19" s="10">
+      <c r="A19" s="9">
         <v>2024</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="F19" s="11" t="b">
+      <c r="B19" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G19:I19,TRUE),_xlpm.av,COUNTIF(G19:I19,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G19" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I19" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K19" s="1">
+      <c r="G19" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L19" s="1">
         <v>45702</v>
       </c>
-      <c r="L19" s="1">
+      <c r="M19" s="1">
         <v>45744</v>
       </c>
-      <c r="M19" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="N19" s="2" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P19" s="2"/>
+        <v>29</v>
+      </c>
+      <c r="P19" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="20" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="10">
+      <c r="A20" s="9">
         <v>2025</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>166</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="F20" s="11" t="b">
+      <c r="B20" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="F20" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G20:I20,TRUE),_xlpm.av,COUNTIF(G20:I20,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>0</v>
       </c>
-      <c r="G20" s="11" t="b">
+      <c r="G20" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H20" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I20" s="11" t="b">
+      <c r="H20" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K20" s="1">
+      <c r="J20" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="L20" s="1">
         <v>45684</v>
       </c>
-      <c r="L20" s="1">
+      <c r="M20" s="1">
         <v>45743</v>
       </c>
-      <c r="M20" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="N20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="P20" s="3"/>
+        <v>43</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P20" s="24" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="21" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A21" s="10">
+      <c r="A21" s="9">
         <v>2025</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="F21" s="11" t="b">
+      <c r="B21" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="F21" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G21:I21,TRUE),_xlpm.av,COUNTIF(G21:I21,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G21" s="11" t="b">
+      <c r="G21" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H21" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="K21" s="1">
+      <c r="H21" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J21" s="27" t="s">
+        <v>216</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="L21" s="1">
         <v>45680</v>
       </c>
-      <c r="L21" s="1">
+      <c r="M21" s="1">
         <v>45712</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="N21" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="O21" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="P21" s="3"/>
+        <v>73</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P21" s="24" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="22" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="10">
+      <c r="A22" s="9">
         <v>2025</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="20" t="s">
+      <c r="B22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="E22" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="F22" s="11" t="str">
+      <c r="D22" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F22" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G22:I22,TRUE),_xlpm.av,COUNTIF(G22:I22,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G22" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H22" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I22" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="L22" s="4">
+      <c r="G22" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I22" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J22" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="M22" s="3">
         <v>45673</v>
       </c>
-      <c r="M22" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="N22" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="O22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="P22" s="5"/>
+      <c r="N22" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="P22" s="25" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="23" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A23" s="10">
+      <c r="A23" s="9">
         <v>2024</v>
       </c>
-      <c r="B23" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="B23" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="F23" s="11" t="b">
+      <c r="D23" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="F23" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G23:I23,TRUE),_xlpm.av,COUNTIF(G23:I23,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G23" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="K23" s="1">
+      <c r="G23" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J23" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="L23" s="1">
         <v>45569</v>
       </c>
-      <c r="L23" s="1">
+      <c r="M23" s="1">
         <v>45610</v>
       </c>
-      <c r="M23" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="N23" s="2" t="s">
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P23" s="2"/>
+        <v>21</v>
+      </c>
+      <c r="P23" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="24" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="10">
+      <c r="A24" s="9">
         <v>2024</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="F24" s="11" t="str">
+      <c r="B24" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F24" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G24:I24,TRUE),_xlpm.av,COUNTIF(G24:I24,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G24" s="11" t="b">
+      <c r="G24" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H24" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I24" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>103</v>
+      <c r="H24" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J24" s="27" t="s">
+        <v>219</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L24" s="1">
+        <v>94</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M24" s="1">
         <v>45538</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="N24" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N24" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="O24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P24" s="2"/>
+      <c r="P24" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="10">
+      <c r="A25" s="9">
         <v>2024</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C25" s="12" t="s">
+      <c r="B25" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="F25" s="11" t="b">
+      <c r="D25" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="F25" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G25:I25,TRUE),_xlpm.av,COUNTIF(G25:I25,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G25" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H25" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="K25" s="1">
+      <c r="G25" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J25" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="L25" s="1">
         <v>45356</v>
       </c>
-      <c r="L25" s="1">
+      <c r="M25" s="1">
         <v>45401</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="N25" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="N25" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O25" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="P25" s="3"/>
+      <c r="P25" s="24" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="26" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A26" s="10">
+      <c r="A26" s="9">
         <v>2024</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="F26" s="11" t="b">
+      <c r="B26" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="F26" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G26:I26,TRUE),_xlpm.av,COUNTIF(G26:I26,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G26" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H26" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I26" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>107</v>
+      <c r="G26" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" s="27" t="s">
+        <v>221</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L26" s="1">
+        <v>98</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M26" s="1">
         <v>45337</v>
       </c>
-      <c r="M26" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="N26" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O26" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="P26" s="3"/>
+        <v>74</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="P26" s="24" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="27" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A27" s="10">
+      <c r="A27" s="9">
         <v>2024</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>163</v>
-      </c>
-      <c r="E27" s="14" t="s">
+      <c r="B27" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="F27" s="11" t="str">
+      <c r="D27" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="F27" s="10" t="str">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G27:I27,TRUE),_xlpm.av,COUNTIF(G27:I27,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>À vérifier</v>
       </c>
-      <c r="G27" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H27" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="I27" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="K27" s="1">
+      <c r="G27" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="J27" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="L27" s="1">
         <v>45266</v>
       </c>
-      <c r="L27" s="1">
+      <c r="M27" s="1">
         <v>45337</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>139</v>
-      </c>
       <c r="N27" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="O27" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="P27" s="2"/>
+        <v>128</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="P27" s="24" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="28" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28" s="10">
+      <c r="A28" s="9">
         <v>2023</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="E28" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="F28" s="11" t="b">
+      <c r="B28" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="F28" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G28:I28,TRUE),_xlpm.av,COUNTIF(G28:I28,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G28" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H28" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I28" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>100</v>
+      <c r="G28" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J28" s="27" t="s">
+        <v>223</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L28" s="1">
+        <v>91</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M28" s="1">
         <v>45259</v>
       </c>
-      <c r="M28" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="N28" s="2" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P28" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="P28" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10">
+      <c r="A29" s="9">
         <v>2023</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C29" s="12" t="s">
+      <c r="B29" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="F29" s="11" t="b">
+      <c r="D29" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="F29" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G29:I29,TRUE),_xlpm.av,COUNTIF(G29:I29,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G29" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H29" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="11" t="b">
+      <c r="G29" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="J29" s="1" t="s">
-        <v>101</v>
+      <c r="J29" s="27" t="s">
+        <v>224</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L29" s="1">
+        <v>92</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M29" s="1">
         <v>45111</v>
       </c>
-      <c r="M29" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="N29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="O29" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="P29" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="O29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="P29" s="24" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10">
+      <c r="A30" s="9">
         <v>2023</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C30" s="12" t="s">
+      <c r="B30" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="F30" s="11" t="b">
+      <c r="D30" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G30:I30,TRUE),_xlpm.av,COUNTIF(G30:I30,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G30" s="11" t="b">
+      <c r="G30" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H30" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I30" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="K30" s="1">
+      <c r="H30" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="L30" s="1">
         <v>44845</v>
       </c>
-      <c r="L30" s="1">
+      <c r="M30" s="1">
         <v>45028</v>
       </c>
-      <c r="M30" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="N30" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="O30" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="P30" s="3"/>
+        <v>78</v>
+      </c>
+      <c r="O30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P30" s="24" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="10">
+      <c r="A31" s="9">
         <v>2023</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="F31" s="11" t="b">
+      <c r="B31" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="F31" s="10" t="b">
         <f>_xlfn.LET(_xlpm.ok,COUNTIF(G31:I31,TRUE),_xlpm.av,COUNTIF(G31:I31,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE)))</f>
         <v>1</v>
       </c>
-      <c r="G31" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H31" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I31" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>102</v>
+      <c r="G31" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J31" s="27" t="s">
+        <v>226</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L31" s="1">
+        <v>93</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M31" s="1">
         <f>DATE(2022,11,17)</f>
         <v>44882</v>
       </c>
-      <c r="M31" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="N31" s="2" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P31" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="P31" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P31" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P31">
-      <sortCondition descending="1" ref="L2:L31"/>
+  <autoFilter ref="A1:Q31" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q31">
+      <sortCondition descending="1" ref="M2:M31"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P31">
-    <sortCondition descending="1" ref="L2:L31"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q31">
+    <sortCondition descending="1" ref="M2:M31"/>
   </sortState>
   <conditionalFormatting sqref="A2:P31">
     <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="vérifier">
@@ -2777,7 +2944,7 @@
       <formula>OR(ISNUMBER(SEARCH("HRLibrary",$D2)),ISNUMBER(SEARCH("BDESE",$D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:I31">
+  <conditionalFormatting sqref="F2:J31">
     <cfRule type="expression" dxfId="1" priority="19">
       <formula>F2=TRUE</formula>
     </cfRule>
@@ -2812,7 +2979,7 @@
     <hyperlink ref="D23" r:id="rId24" xr:uid="{29A2B983-F112-4EE6-9B44-0F1CB988C6C1}"/>
     <hyperlink ref="D16" r:id="rId25" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Retraite%20d'Entreprise%20Collectif%20PERCOL%20(16%20d%c3%a9cembre%202025).pdf" xr:uid="{ADB6C391-B664-442C-84BE-32EB612092D0}"/>
     <hyperlink ref="D14" r:id="rId26" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Accord%20collectif%20portant%20sur%20une%20Rupture%20Conventionnelle%20Collective%20(RCC)%20au%20sein%20de%20Nokia%20Networks%20France%20(compress%c3%a9).pdf" xr:uid="{CDF018D6-A914-4E6F-BC99-C9BC7058618D}"/>
-    <hyperlink ref="O27" r:id="rId27" xr:uid="{795404A2-F15F-4A6A-94CF-0EC12677A11E}"/>
+    <hyperlink ref="P27" r:id="rId27" xr:uid="{795404A2-F15F-4A6A-94CF-0EC12677A11E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId28"/>

</xml_diff>

<commit_message>
Sync agreements from Excel: Lannion and new agreements, signature captures
- 42 agreements regenerated from Excel (columns matched by header)
- 13 new agreements (LAN, NPS, NNF) with signatures, captures and sources
- Site filter (default NNF); tract titles from Excel
- Signature captures regenerated/renamed from local PDFs; obsolete ones removed
- MISE_A_JOUR_EXCEL.md: column mapping by header name
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1790" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4017F709-2427-4F0C-8126-F957E53A2314}"/>
+  <xr:revisionPtr revIDLastSave="1859" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73BCEF42-075F-4444-8AB9-6F669D0531C1}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="accords" sheetId="1" r:id="rId1"/>
     <sheet name="rules" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">accords!$A$1:$P$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">accords!$A$1:$Q$30</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="215">
   <si>
     <t>Accord ou négociation</t>
   </si>
@@ -96,9 +96,6 @@
     <t>Signataire (logique pragmatique), avec alertes : pressions au volontariat, décimation des équipes, absence de garanties sur les activités en France, lien RCC / absence d'augmentation.</t>
   </si>
   <si>
-    <t>Projet d'accord d'harmonisation des bonus (TI) — document de travail retrouvé.</t>
-  </si>
-  <si>
     <t>Signataire : soutien à l'élargissement, demande d'un seuil préservant les congés des aidants.</t>
   </si>
   <si>
@@ -114,9 +111,6 @@
     <t>Signataire, puis bilan critique : délocalisations, perte de savoir-faire, charge de travail, RPS, externalisations.</t>
   </si>
   <si>
-    <t>Contenu, dates et versions à retrouver.</t>
-  </si>
-  <si>
     <t>Signataire (confirmé par le bilan annuel).</t>
   </si>
   <si>
@@ -126,9 +120,6 @@
     <t>Non signataire : désaccords sur la classification et la cotation.</t>
   </si>
   <si>
-    <t>Calendrier, contenu final et signataires à retrouver.</t>
-  </si>
-  <si>
     <t>Non signataire.</t>
   </si>
   <si>
@@ -294,15 +285,9 @@
     <t>PDF signé (scan, 08/12/2023), p. 4 : signatures CFDT, CFE-CGC, CGT et CFTC</t>
   </si>
   <si>
-    <t>PDF « Accord don de jours 14 novembre 2024 signé » (scan), p. 11 : signatures CFDT, CFE-CGC et CGT</t>
-  </si>
-  <si>
     <t>PDF signé (scan, 13/04/2023), p. 20 : signatures CFDT (R. Tutrel) et CFE-CGC ; bloc CGT vide</t>
   </si>
   <si>
-    <t>À vérifier : seule la version « mise à la signature » (non signée, 20/01/2025) a été trouvée</t>
-  </si>
-  <si>
     <t>file name</t>
   </si>
   <si>
@@ -402,15 +387,9 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/NAO_2026_Proc%c3%a8s_verbal_d_accord_24%20janvier_2026.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/BDESENNF-Centrale/Shared%20Documents/01.%20BDESE%20Centrale/02%20-%20Investissements/01%20-%20Investissement%20social/Handicap/Accord%20handicap%202026.pdf</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/GEPP%20PV%20de%20d%C3%A9saccord%20mis%20%C3%A0%20signature.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202022/Accord%20%C3%A9tablissement%20am%C3%A9nagement%20temps%20de%20travail%202022.pdf</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20%C3%A9galit%C3%A9%20professionnelle.pdf</t>
   </si>
   <si>
@@ -435,9 +414,6 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202026/Accord_RCC_2026.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/PV%20d%C3%A9saccord%20Partage%20de%20la%20valeur%20VS.pdf</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/NAO%202023%20-%20PV%20d%C3%A9saccord.pdf</t>
   </si>
   <si>
@@ -513,9 +489,6 @@
     <t>Avenant accord télétravail avril 2022.pdf</t>
   </si>
   <si>
-    <t>2025 Accord etablissement NAO Mis à la signature.pdf</t>
-  </si>
-  <si>
     <t>Avenant Procès-verbal de désaccord NAO 2024 (9 avril 2024).pdf</t>
   </si>
   <si>
@@ -525,9 +498,6 @@
     <t>Accord remboursement santé - 2023.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/2025%20Accord%20etablissement%20NAO%20Mis%20%C3%A0%20la%20signature.pdf</t>
-  </si>
-  <si>
     <t>page signature</t>
   </si>
   <si>
@@ -567,9 +537,6 @@
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CGF_p10_signature.jpg</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_etablissement_amenagement_temps_de_travail_2022_p04_signature.jpg</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2024_p04_signature.jpg</t>
   </si>
   <si>
@@ -579,9 +546,6 @@
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_no_1_a_l_Accord_CSE_du_21_septembre_2018_p10_signature.jpg</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_handicap_2026_p15-16_signatures.jpg</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2026_Proces_verbal_d_accord_24_janvier_2026_p07_signature.jpg</t>
   </si>
   <si>
@@ -609,9 +573,6 @@
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_accord_teletravail_avril_2022_p07_signature.jpg</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_NPS_2025_accord_mis_a_signature_p4.jpg</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_don_de_jours_14_novembre_2024_p11_signature.jpg</t>
   </si>
   <si>
@@ -666,9 +627,6 @@
     <t>p.9 : signatures de la Direction, de la CFDT, de la CFE-CGC et de la CGT.</t>
   </si>
   <si>
-    <t>p.4 : signatures de la Direction, de la CFDT, de la CFE-CGC, de la CGT et de la CFTC (accord portant sur 2022).</t>
-  </si>
-  <si>
     <t>p.16 : signatures de la Direction, de la CFDT, de la CFE-CGC et de la CGT.</t>
   </si>
   <si>
@@ -678,12 +636,6 @@
     <t>p.52 : signatures de la CFDT et de la CFE-CGC ; aucune signature de la CGT visible. Confirmé par l’avenant et la décision DREETS (76,51 %).</t>
   </si>
   <si>
-    <t>p.15–16 : date et signatures absentes de cet exemplaire ; signatures confirmées par l’annonce officielle Viva Engage et le vote AG CGT du 21/05/2026.</t>
-  </si>
-  <si>
-    <t>Aménagement du temps de travail 2022</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_egalite_professionnelle_p20_signature.jpg</t>
   </si>
   <si>
@@ -694,6 +646,45 @@
   </si>
   <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Harmonisation_TI_final_p10.jpg</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FHRLibrary%2FControlled%20Documents%2FHR%20Regions%2FEurope%20South%2FFrance%2FArchive%2FSOP%20%2D%20Guidelines%20%2D%20HARMONIZED%2FAccord%202025%20NPS%20%2D%20am%C3%A9nagement%20temps%20de%20travail%20%2820%20janvier%202025%29%2Epdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/NokiaNetworksFrance%2Fnps%2FDocuments%20partages%2FNotes%20de%20service%20NPS%2F2023%20Accord%20Amenagement%20temps%20travail%20sign%C3%A9%2Epdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?viewid=98338bf1-f1d6-4255-96fd-c8be2f7ddc8a&amp;FolderCTID=0x0120008156B534D558334ABAC4AD879F1E6E6B&amp;id=%2Fsites%2FHRLibrary%2FControlled+Documents%2FHR+Regions%2FEurope+South%2FFrance%2FHR+SOPs-Guidelines-Policy%2FHarmonized%2FAccords+conventions+2026%2FAccord+d%27entreprise+relatif+%C3%A0+la+situation+de+handicap+NNF.pdf</t>
+  </si>
+  <si>
+    <t>Aménagement du temps de travail 2023</t>
+  </si>
+  <si>
+    <t>p.15–16 : signatures de la Direction (p.15, A. Vavon, M. Cudot ; Massy, 19/06/2026), de la CFDT, de la CFE-CGC et de la CGT (p.16).</t>
+  </si>
+  <si>
+    <t>Accord 2025 NPS - aménagement temps de travail (20 janvier 2025).pdf</t>
+  </si>
+  <si>
+    <t>p.4 : signatures de la Direction (S. Bermond), de la CFDT, de la CFE-CGC, de la CGT et de la CFTC.</t>
+  </si>
+  <si>
+    <t>p. 11 : signatures CFDT, CFE-CGC et CGT</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions%2FEurope%20South%2FFrance%2FHR%20SOPs%2DGuidelines%2DPolicy%2FHarmonized%2FAccords%20conventions%202024%2FPV%20d%C3%A9saccord%20Partage%20de%20la%20valeur%20VS%2Epdf</t>
+  </si>
+  <si>
+    <t>Négociation imposée par la loi n° 2023-1107 du 29/11/2023 (augmentation exceptionnelle du bénéfice net fiscal). Pas d'accord à l'issue de la réunion du 31/05/2024. Revendications : une hausse du CA doit déclencher une prime. Décision unilatérale de la Direction : « bénéfice exceptionnel » = bénéfice net fiscal &gt; 15 % du CA France ; négociation sur le montant de la prime seulement au-delà de ce seuil.</t>
+  </si>
+  <si>
+    <t>Dernière phase d'harmonisation des taux de variable cible (TI) des salariés « non sales » de NNF sur le taux Nokia de leur Job Grade (historique : grille ALU 2015, classification Nokia 2017, accord NAO du 19/04/2022, courrier intersyndical du 04/05/2023). Réunion du 18/12/2023. À compter du 01/01/2024, tout salarié sous le taux Nokia passe au taux de son Job Grade : JG5-6 5 %, JG7 7,5 %, JG8 10 %, JG9 12,5 %, JG10 15 %, JG11 20 %, JG12 25 %, JG13 30 %. Au-dessus du taux Nokia : les augmentations restent affectées au fixe. Durée déterminée.</t>
+  </si>
+  <si>
+    <t>Accord d'établissement Nokia Paris-Saclay (Massy, Nozay) pour 2024 (réunions des 24/11 et 08/12/2023) : 1 JRTT/JRS collectif fixé au vendredi 10/05/2024 (pont de l'Ascension, établissement fermé) ; les 2 autres JRTT/JRS sont posés librement. S'appuie sur l'accord ARTT du 19/10/2000 repris par l'accord d'établissement du 09/01/2001 (3 JRTT/JRS collectifs maximum).</t>
+  </si>
+  <si>
+    <t>remarque</t>
   </si>
 </sst>
 </file>
@@ -1025,6 +1016,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1288,7 +1283,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr defaultColWidth="12.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="8" customWidth="1"/>
@@ -1296,133 +1291,137 @@
     <col min="3" max="3" width="41.28515625" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27" style="19" customWidth="1"/>
     <col min="5" max="5" width="21.7109375" style="8" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" style="8" customWidth="1"/>
-    <col min="7" max="9" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.42578125" style="25" customWidth="1"/>
-    <col min="11" max="11" width="49.5703125" style="8" customWidth="1"/>
-    <col min="12" max="12" width="14.28515625" style="8" customWidth="1"/>
-    <col min="13" max="14" width="57.140625" style="8" customWidth="1"/>
-    <col min="15" max="15" width="55.85546875" style="25" customWidth="1"/>
-    <col min="16" max="16" width="12.140625" style="27"/>
-    <col min="17" max="16384" width="12.140625" style="8"/>
+    <col min="6" max="6" width="14.28515625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="8" customWidth="1"/>
+    <col min="8" max="10" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.42578125" style="25" customWidth="1"/>
+    <col min="12" max="12" width="49.5703125" style="8" customWidth="1"/>
+    <col min="13" max="15" width="57.140625" style="8" customWidth="1"/>
+    <col min="16" max="16" width="55.85546875" style="25" customWidth="1"/>
+    <col min="17" max="17" width="12.140625" style="27"/>
+    <col min="18" max="16384" width="12.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>100</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>80</v>
+      <c r="K1" s="21" t="s">
+        <v>152</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>11</v>
       </c>
       <c r="N1" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="O1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="21" t="s">
+      <c r="P1" s="21" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>2026</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C2)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G2:I2,TRUE),_xlpm.av,COUNTIF(G2:I2,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>83</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46219</v>
       </c>
       <c r="G2" s="10" t="b">
+        <f t="shared" ref="G2:G30" si="0">IF(ISNUMBER(SEARCH("PV de désaccord",C2)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H2:J2,TRUE),_xlpm.av,COUNTIF(H2:J2,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
+        <v>1</v>
+      </c>
+      <c r="H2" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H2" s="10" t="b">
-        <v>1</v>
-      </c>
       <c r="I2" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J2" s="26" t="s">
-        <v>177</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="L2" s="1">
-        <v>46219</v>
+      <c r="J2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="O2" s="23" t="s">
-        <v>142</v>
+        <v>41</v>
+      </c>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P2" s="23" t="s">
+        <v>134</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>2026</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C3)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G3:I3,TRUE),_xlpm.av,COUNTIF(G3:I3,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>84</v>
+      </c>
+      <c r="F3" s="1">
+        <v>46212</v>
       </c>
       <c r="G3" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H3" s="10" t="b">
@@ -1431,46 +1430,47 @@
       <c r="I3" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J3" s="26" t="s">
-        <v>178</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="L3" s="1">
-        <v>46212</v>
+      <c r="J3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O3" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P3" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>2026</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>50</v>
-      </c>
       <c r="D4" s="18" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="F4" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C4)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G4:I4,TRUE),_xlpm.av,COUNTIF(G4:I4,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>145</v>
+      </c>
+      <c r="F4" s="1">
+        <v>46192</v>
       </c>
       <c r="G4" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H4" s="10" t="b">
@@ -1479,46 +1479,45 @@
       <c r="I4" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J4" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="L4" s="1">
-        <v>46181</v>
+      <c r="J4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" s="26"/>
+      <c r="L4" s="1" t="s">
+        <v>206</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="O4" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P4" s="24" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2026</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C5)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G5:I5,TRUE),_xlpm.av,COUNTIF(G5:I5,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>97</v>
+      </c>
+      <c r="F5" s="1">
+        <v>46048</v>
       </c>
       <c r="G5" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H5" s="10" t="b">
@@ -1527,94 +1526,96 @@
       <c r="I5" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J5" s="26" t="s">
-        <v>180</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="L5" s="1">
-        <v>46048</v>
+      <c r="J5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O5" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P5" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>2026</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="F6" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C6)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G6:I6,TRUE),_xlpm.av,COUNTIF(G6:I6,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>146</v>
+      </c>
+      <c r="F6" s="1">
+        <v>46037</v>
       </c>
       <c r="G6" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H6" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="10" t="b">
-        <v>1</v>
-      </c>
       <c r="I6" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J6" s="26" t="s">
-        <v>181</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="L6" s="1">
-        <v>46037</v>
+      <c r="J6" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="O6" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P6" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>2026</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="F7" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C7)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G7:I7,TRUE),_xlpm.av,COUNTIF(G7:I7,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>111</v>
+      </c>
+      <c r="F7" s="1">
+        <v>46010</v>
       </c>
       <c r="G7" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H7" s="10" t="b">
@@ -1623,191 +1624,195 @@
       <c r="I7" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J7" s="26" t="s">
-        <v>182</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="L7" s="1">
-        <v>46010</v>
+      <c r="J7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="O7" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P7" s="24" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>2026</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="F8" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C8)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G8:I8,TRUE),_xlpm.av,COUNTIF(G8:I8,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>85</v>
+      </c>
+      <c r="F8" s="1">
+        <v>46010</v>
       </c>
       <c r="G8" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H8" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="10" t="b">
-        <v>1</v>
-      </c>
       <c r="I8" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J8" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="L8" s="1">
-        <v>46010</v>
+      <c r="J8" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>197</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O8" s="23" t="s">
-        <v>143</v>
+        <v>65</v>
+      </c>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="P8" s="23" t="s">
+        <v>135</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>2025</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="F9" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C9)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G9:I9,TRUE),_xlpm.av,COUNTIF(G9:I9,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>87</v>
+      </c>
+      <c r="F9" s="1">
+        <v>46007</v>
       </c>
       <c r="G9" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H9" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="10" t="b">
-        <v>1</v>
-      </c>
       <c r="I9" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J9" s="26" t="s">
-        <v>184</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="L9" s="1">
-        <v>46007</v>
+      <c r="J9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>183</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="O9" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="P9" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>2025</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="F10" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C10)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G10:I10,TRUE),_xlpm.av,COUNTIF(G10:I10,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>86</v>
+      </c>
+      <c r="F10" s="1">
+        <v>46007</v>
       </c>
       <c r="G10" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H10" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="10" t="b">
-        <v>1</v>
-      </c>
       <c r="I10" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J10" s="26" t="s">
+      <c r="J10" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="L10" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="L10" s="1">
-        <v>46007</v>
-      </c>
       <c r="M10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="O10" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>2025</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="F11" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C11)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G11:I11,TRUE),_xlpm.av,COUNTIF(G11:I11,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>9</v>
+        <v>147</v>
+      </c>
+      <c r="F11" s="1">
+        <v>45930</v>
+      </c>
+      <c r="G11" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>9</v>
@@ -1815,95 +1820,97 @@
       <c r="I11" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J11" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L11" s="1">
-        <v>45930</v>
+      <c r="J11" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O11" s="23" t="s">
-        <v>144</v>
+        <v>68</v>
+      </c>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P11" s="23" t="s">
+        <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
         <v>2025</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F12" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C12)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G12:I12,TRUE),_xlpm.av,COUNTIF(G12:I12,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
-      </c>
-      <c r="G12" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="J12" s="26" t="s">
-        <v>186</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="L12" s="1">
+        <v>88</v>
+      </c>
+      <c r="F12" s="1">
         <f>DATE(2025,7,24)</f>
         <v>45862</v>
       </c>
+      <c r="G12" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H12" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>184</v>
+      </c>
       <c r="M12" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="O12" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P12" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
         <v>2024</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="F13" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C13)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G13:I13,TRUE),_xlpm.av,COUNTIF(G13:I13,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>92</v>
+      </c>
+      <c r="F13" s="1">
+        <v>45744</v>
       </c>
       <c r="G13" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H13" s="10" t="b">
@@ -1912,190 +1919,192 @@
       <c r="I13" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J13" t="s">
-        <v>187</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="L13" s="1">
-        <v>45744</v>
+      <c r="J13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="s">
+        <v>175</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>195</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O13" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P13" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
         <v>2025</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D14" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F14" s="1">
+        <v>45743</v>
+      </c>
+      <c r="G14" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K14" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P14" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="E14" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="F14" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C14)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G14:I14,TRUE),_xlpm.av,COUNTIF(G14:I14,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="J14" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L14" s="1">
-        <v>45743</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O14" s="23" t="s">
-        <v>145</v>
-      </c>
     </row>
-    <row r="15" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>2025</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="F15" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C15)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G15:I15,TRUE),_xlpm.av,COUNTIF(G15:I15,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>148</v>
+      </c>
+      <c r="F15" s="1">
+        <v>45712</v>
       </c>
       <c r="G15" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H15" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H15" s="10" t="b">
-        <v>1</v>
-      </c>
       <c r="I15" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J15" s="26" t="s">
-        <v>188</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L15" s="1">
-        <v>45712</v>
+      <c r="J15" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>78</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O15" s="23" t="s">
-        <v>146</v>
+        <v>69</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P15" s="23" t="s">
+        <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>2025</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>161</v>
+        <v>202</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="F16" s="10" t="str">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C16)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G16:I16,TRUE),_xlpm.av,COUNTIF(G16:I16,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>À vérifier</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="J16" s="26" t="s">
-        <v>189</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="L16" s="3">
-        <v>45673</v>
+        <v>207</v>
+      </c>
+      <c r="F16" s="3">
+        <v>45677</v>
+      </c>
+      <c r="G16" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H16" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" s="26"/>
+      <c r="L16" s="3" t="s">
+        <v>208</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="N16" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="O16" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P16" s="24" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>2024</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="F17" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C17)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G17:I17,TRUE),_xlpm.av,COUNTIF(G17:I17,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>94</v>
+      </c>
+      <c r="F17" s="1">
+        <v>45610</v>
       </c>
       <c r="G17" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H17" s="10" t="b">
@@ -2104,47 +2113,48 @@
       <c r="I17" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J17" s="26" t="s">
-        <v>190</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L17" s="1">
-        <v>45610</v>
+      <c r="J17" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>209</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="O17" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="P17" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="105" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>2024</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>131</v>
+        <v>210</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="F18" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C18)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G18:I18,TRUE),_xlpm.av,COUNTIF(G18:I18,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>9</v>
+        <v>90</v>
+      </c>
+      <c r="F18" s="1">
+        <v>45538</v>
+      </c>
+      <c r="G18" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>9</v>
@@ -2152,46 +2162,47 @@
       <c r="I18" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J18" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L18" s="1">
-        <v>45538</v>
+      <c r="J18" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K18" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O18" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P18" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>2024</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="F19" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C19)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G19:I19,TRUE),_xlpm.av,COUNTIF(G19:I19,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>98</v>
+      </c>
+      <c r="F19" s="1">
+        <v>45401</v>
       </c>
       <c r="G19" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H19" s="10" t="b">
@@ -2200,46 +2211,47 @@
       <c r="I19" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J19" s="26" t="s">
-        <v>191</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="L19" s="1">
-        <v>45401</v>
+      <c r="J19" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="M19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="N19" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O19" s="23" t="s">
-        <v>147</v>
+      <c r="P19" s="23" t="s">
+        <v>139</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
         <v>2024</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="F20" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C20)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G20:I20,TRUE),_xlpm.av,COUNTIF(G20:I20,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>143</v>
+      </c>
+      <c r="F20" s="1">
+        <v>45366</v>
       </c>
       <c r="G20" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H20" s="10" t="b">
@@ -2248,46 +2260,47 @@
       <c r="I20" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J20" s="26" t="s">
-        <v>174</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="L20" s="1">
-        <v>45366</v>
+      <c r="J20" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="M20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="N20" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="O20" s="22" t="s">
+      <c r="P20" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>2024</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="D21" s="17" t="s">
-        <v>107</v>
+        <v>160</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>102</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="F21" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C21)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G21:I21,TRUE),_xlpm.av,COUNTIF(G21:I21,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>91</v>
+      </c>
+      <c r="F21" s="1">
+        <v>45337</v>
       </c>
       <c r="G21" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H21" s="10" t="b">
@@ -2296,47 +2309,48 @@
       <c r="I21" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J21" s="26" t="s">
-        <v>192</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="L21" s="1">
-        <v>45337</v>
+      <c r="J21" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" s="26" t="s">
+        <v>179</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>79</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O21" s="23" t="s">
-        <v>148</v>
+        <v>70</v>
+      </c>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P21" s="23" t="s">
+        <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>2024</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="F22" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C22)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G22:I22,TRUE),_xlpm.av,COUNTIF(G22:I22,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>9</v>
+        <v>149</v>
+      </c>
+      <c r="F22" s="1">
+        <v>45337</v>
+      </c>
+      <c r="G22" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>9</v>
@@ -2344,46 +2358,47 @@
       <c r="I22" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J22" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L22" s="1">
-        <v>45337</v>
+      <c r="J22" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K22" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="O22" s="23" t="s">
-        <v>147</v>
+        <v>107</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="P22" s="23" t="s">
+        <v>139</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="150" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>2023</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="F23" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C23)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G23:I23,TRUE),_xlpm.av,COUNTIF(G23:I23,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>199</v>
+      </c>
+      <c r="F23" s="1">
+        <v>45279</v>
       </c>
       <c r="G23" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H23" s="10" t="b">
@@ -2392,46 +2407,47 @@
       <c r="I23" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J23" s="26" t="s">
-        <v>217</v>
-      </c>
-      <c r="K23" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="L23" s="1">
-        <v>45279</v>
+      <c r="J23" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K23" s="26" t="s">
+        <v>201</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="N23" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="O23" s="22" t="s">
+      <c r="P23" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="105" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>2024</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="F24" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C24)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G24:I24,TRUE),_xlpm.av,COUNTIF(G24:I24,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>93</v>
+      </c>
+      <c r="F24" s="1">
+        <v>45268</v>
       </c>
       <c r="G24" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H24" s="10" t="b">
@@ -2440,46 +2456,47 @@
       <c r="I24" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J24" t="s">
-        <v>176</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L24" s="1">
-        <v>45268</v>
+      <c r="J24" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" t="s">
+        <v>165</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O24" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P24" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>2023</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="F25" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C25)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G25:I25,TRUE),_xlpm.av,COUNTIF(G25:I25,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>99</v>
+      </c>
+      <c r="F25" s="1">
+        <v>45259</v>
       </c>
       <c r="G25" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H25" s="10" t="b">
@@ -2488,95 +2505,97 @@
       <c r="I25" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J25" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="L25" s="1">
-        <v>45259</v>
+      <c r="J25" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25" s="26" t="s">
+        <v>180</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>194</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="O25" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="N25" s="2"/>
+      <c r="O25" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P25" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>2023</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>6</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="F26" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C26)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G26:I26,TRUE),_xlpm.av,COUNTIF(G26:I26,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>150</v>
+      </c>
+      <c r="F26" s="1">
+        <v>45111</v>
       </c>
       <c r="G26" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H26" s="10" t="b">
         <v>1</v>
       </c>
       <c r="I26" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="J26" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="L26" s="1">
-        <v>45111</v>
+      <c r="K26" s="26" t="s">
+        <v>181</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="N26" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="N26" s="2"/>
+      <c r="O26" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O26" s="23" t="s">
-        <v>149</v>
+      <c r="P26" s="23" t="s">
+        <v>141</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>2023</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="F27" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C27)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G27:I27,TRUE),_xlpm.av,COUNTIF(G27:I27,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
-      </c>
-      <c r="G27" s="10" t="s">
-        <v>9</v>
+        <v>95</v>
+      </c>
+      <c r="F27" s="1">
+        <v>45028</v>
+      </c>
+      <c r="G27" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="H27" s="10" t="s">
         <v>9</v>
@@ -2584,143 +2603,146 @@
       <c r="I27" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J27" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L27" s="1">
-        <v>45028</v>
+      <c r="J27" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K27" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="M27" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N27" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="O27" s="23" t="s">
-        <v>141</v>
+      <c r="N27" s="2"/>
+      <c r="O27" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="P27" s="23" t="s">
+        <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>2023</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>4</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="F28" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C28)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G28:I28,TRUE),_xlpm.av,COUNTIF(G28:I28,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>96</v>
+      </c>
+      <c r="F28" s="1">
+        <v>45028</v>
       </c>
       <c r="G28" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H28" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="H28" s="10" t="b">
-        <v>1</v>
-      </c>
       <c r="I28" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J28" s="26" t="s">
-        <v>214</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="L28" s="1">
-        <v>45028</v>
+      <c r="J28" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K28" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="N28" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="O28" s="23" t="s">
-        <v>150</v>
+      <c r="P28" s="23" t="s">
+        <v>142</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>2023</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="F29" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C29)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G29:I29,TRUE),_xlpm.av,COUNTIF(G29:I29,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
-      </c>
-      <c r="G29" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H29" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="J29" s="26" t="s">
-        <v>195</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="L29" s="1">
+        <v>151</v>
+      </c>
+      <c r="F29" s="1">
         <f>DATE(2022,11,17)</f>
         <v>44882</v>
       </c>
+      <c r="G29" s="10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H29" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J29" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K29" s="26" t="s">
+        <v>182</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>189</v>
+      </c>
       <c r="M29" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="O29" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="N29" s="2"/>
+      <c r="O29" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="P29" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>122</v>
+        <v>203</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="F30" s="10" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C30)),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(G30:I30,TRUE),_xlpm.av,COUNTIF(G30:I30,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))</f>
-        <v>1</v>
+        <v>144</v>
+      </c>
+      <c r="F30" s="1">
+        <v>44967</v>
       </c>
       <c r="G30" s="10" t="b">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H30" s="10" t="b">
@@ -2729,31 +2751,27 @@
       <c r="I30" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J30" s="26" t="s">
-        <v>175</v>
-      </c>
-      <c r="K30" s="1" t="s">
+      <c r="J30" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K30" s="26"/>
+      <c r="L30" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="L30" s="1">
-        <v>44543</v>
-      </c>
       <c r="M30" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="O30" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="N30" s="2"/>
+      <c r="O30" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="P30" s="23" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P30" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P30">
-    <sortCondition descending="1" ref="L2:L30"/>
-  </sortState>
-  <conditionalFormatting sqref="A2:O30">
+  <autoFilter ref="A1:Q30" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A2:P30">
     <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",A2)))</formula>
     </cfRule>
@@ -2775,12 +2793,12 @@
       <formula>OR(ISNUMBER(SEARCH("HRLibrary",$D2)),ISNUMBER(SEARCH("BDESE",$D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:J30">
+  <conditionalFormatting sqref="G2:K30">
     <cfRule type="expression" dxfId="1" priority="19">
-      <formula>F2=TRUE</formula>
+      <formula>G2=TRUE</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="20">
-      <formula>F2=FALSE</formula>
+      <formula>G2=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -2788,7 +2806,7 @@
     <hyperlink ref="D24" r:id="rId2" xr:uid="{A9AF55B6-9AF4-441B-BF54-A1A9640D2C9D}"/>
     <hyperlink ref="D22" r:id="rId3" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Avenant%20Proc%C3%A8s-verbal%20de%20d%C3%A9saccord%20NAO%202024%20(9%20avril%202024).pdf" xr:uid="{F6B82D88-92B4-4369-B825-E6CFE444F804}"/>
     <hyperlink ref="D11" r:id="rId4" xr:uid="{6A46598A-BCC9-4794-AE14-7CBA11E19EBB}"/>
-    <hyperlink ref="D16" r:id="rId5" xr:uid="{5C4C6E25-614E-4F25-8AA8-26F96EA1D6FC}"/>
+    <hyperlink ref="D16" r:id="rId5" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FHRLibrary%2FControlled%20Documents%2FHR%20Regions%2FEurope%20South%2FFrance%2FArchive%2FSOP%20%2D%20Guidelines%20%2D%20HARMONIZED%2FAccord%202025%20NPS%20%2D%20am%C3%A9nagement%20temps%20de%20travail%20%2820%20janvier%202025%29%2Epdf" xr:uid="{5C4C6E25-614E-4F25-8AA8-26F96EA1D6FC}"/>
     <hyperlink ref="D28" r:id="rId6" xr:uid="{B32EB3EF-DF8F-4ACB-9052-ED0420F2EB20}"/>
     <hyperlink ref="D18" r:id="rId7" xr:uid="{C9C0BF18-CF80-4BAF-B84A-71DFE1F4CEF1}"/>
     <hyperlink ref="D30" r:id="rId8" xr:uid="{C043EA89-0A53-4B71-AC0C-5C4306E62617}"/>
@@ -2796,7 +2814,7 @@
     <hyperlink ref="D3" r:id="rId10" xr:uid="{82282E9B-CCA9-434A-AE8B-F46BDD379264}"/>
     <hyperlink ref="D5" r:id="rId11" xr:uid="{9C779CF0-9D36-4133-B425-014C0E592614}"/>
     <hyperlink ref="D6" r:id="rId12" xr:uid="{1CAF7A33-3FE3-42CD-B630-103D55FCDBB0}"/>
-    <hyperlink ref="D4" r:id="rId13" xr:uid="{85C39618-C574-4EEC-8C06-0BC340D4273B}"/>
+    <hyperlink ref="D4" r:id="rId13" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/Forms/AllItems.aspx?viewid=98338bf1-f1d6-4255-96fd-c8be2f7ddc8a&amp;FolderCTID=0x0120008156B534D558334ABAC4AD879F1E6E6B&amp;id=%2Fsites%2FHRLibrary%2FControlled+Documents%2FHR+Regions%2FEurope+South%2FFrance%2FHR+SOPs-Guidelines-Policy%2FHarmonized%2FAccords+conventions+2026%2FAccord+d%27entreprise+relatif+%C3%A0+la+situation+de+handicap+NNF.pdf" xr:uid="{85C39618-C574-4EEC-8C06-0BC340D4273B}"/>
     <hyperlink ref="D7" r:id="rId14" xr:uid="{E88B21CF-4C2B-47AB-B153-EB4D68F183C9}"/>
     <hyperlink ref="D9" r:id="rId15" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Entreprise%20au%20sein%20de%20Nokia%20Networks%20France%20(16%20d%c3%a9cembre%202025).pdf" xr:uid="{BF514F36-2459-4883-A6C8-AB19CDC9D51E}"/>
     <hyperlink ref="D27" r:id="rId16" xr:uid="{4293582A-4729-404B-A1F9-27BD5C6AE9EF}"/>
@@ -2809,11 +2827,12 @@
     <hyperlink ref="D17" r:id="rId23" xr:uid="{29A2B983-F112-4EE6-9B44-0F1CB988C6C1}"/>
     <hyperlink ref="D10" r:id="rId24" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Accord%20d'entreprise%20relatif%20au%20Plan%20d'Epargne%20Retraite%20d'Entreprise%20Collectif%20PERCOL%20(16%20d%c3%a9cembre%202025).pdf" xr:uid="{ADB6C391-B664-442C-84BE-32EB612092D0}"/>
     <hyperlink ref="D8" r:id="rId25" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Accord%20collectif%20portant%20sur%20une%20Rupture%20Conventionnelle%20Collective%20(RCC)%20au%20sein%20de%20Nokia%20Networks%20France%20(compress%c3%a9).pdf" xr:uid="{CDF018D6-A914-4E6F-BC99-C9BC7058618D}"/>
-    <hyperlink ref="O22" r:id="rId26" xr:uid="{795404A2-F15F-4A6A-94CF-0EC12677A11E}"/>
+    <hyperlink ref="P22" r:id="rId26" xr:uid="{795404A2-F15F-4A6A-94CF-0EC12677A11E}"/>
     <hyperlink ref="D23" r:id="rId27" display="https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents%2FHR%20Regions%2FEurope%20South%2FFrance%2FArchive%2FArchives%2FAccords%20Nokia%2FAccord%20harmonisation%20taux%20variable%20cible%20salari%C3%A9s%20non%20sales%20du%2019%20d%C3%A9cembre%202023%2Epdf" xr:uid="{FDD5D552-019A-4567-AF33-C61EE56F7820}"/>
+    <hyperlink ref="D21" r:id="rId28" xr:uid="{2522EABD-D1D8-4D0A-8D29-FE52786A9FF3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId28"/>
+  <pageSetup orientation="portrait" r:id="rId29"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
   </headerFooter>
@@ -2834,10 +2853,31 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
+    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
+    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
+      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
+      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -3108,30 +3148,9 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
-    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
-    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
-      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
-      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3185,14 +3204,25 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
+    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3212,21 +3242,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
-    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add the AUXAD agreement and align the page with the latest Excel sync.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2415" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C22E56B-621D-46D5-938F-717FA532B371}"/>
+  <xr:revisionPtr revIDLastSave="2503" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{903CCD27-DD50-4B71-AADE-96FB1B9F3E41}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="327">
   <si>
     <t>Accord ou négociation</t>
   </si>
@@ -121,12 +121,6 @@
     <t>CET</t>
   </si>
   <si>
-    <t>GEPP – PV de désaccord</t>
-  </si>
-  <si>
-    <t>Partage de la valeur – PV de désaccord</t>
-  </si>
-  <si>
     <t>Intéressement 2025-2028</t>
   </si>
   <si>
@@ -139,12 +133,6 @@
     <t>Remboursement santé</t>
   </si>
   <si>
-    <t>NAO 2025 – PV de désaccord</t>
-  </si>
-  <si>
-    <t>NAO 2023 – PV de désaccord</t>
-  </si>
-  <si>
     <t>RCC 2026 n°2</t>
   </si>
   <si>
@@ -160,9 +148,6 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20am%C3%A9nagement%20temps%20travail%20NPS%202024.pdf</t>
   </si>
   <si>
-    <t>NAO 2024 – PV de désaccord</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/GEPP%20PV%20de%20d%C3%A9saccord%20mis%20%C3%A0%20signature.pdf</t>
   </si>
   <si>
@@ -355,21 +340,9 @@
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2023_p04_signature.jpg</t>
   </si>
   <si>
-    <t>Pas d'accord majoritaire ; PV signé par la DRH et les DSC CFDT, CFE-CGC et CGT. (autre source, à vérifier)</t>
-  </si>
-  <si>
-    <t>Compteur &gt; 900 jours. (autre source, à vérifier)</t>
-  </si>
-  <si>
     <t>Comité Groupe France (NNF, ASN, RFS).</t>
   </si>
   <si>
-    <t>Dénoncé en 2025 (sortie d'ASN, fermeture de RFS). (autre source, à vérifier)</t>
-  </si>
-  <si>
-    <t>Contestation des nombreux 0 % d'augmentation. (source : tract, à vérifier)</t>
-  </si>
-  <si>
     <t>autre source (email, teams, sharepoint)</t>
   </si>
   <si>
@@ -421,9 +394,6 @@
     <t>Politique handicap NNF : rôles des acteurs (managers, santé au travail, service social, Mission handicap). Cotisations retraite prises en charge à 100 % en temps partiel choisi.</t>
   </si>
   <si>
-    <t>Pas d'augmentation générale. Augmentations individuelles 2,15 % (promotions incluses) au 01/04/2026. Primes de transport : zone 1 9 €, zone 2 12 €, zone 3 60 €.</t>
-  </si>
-  <si>
     <t>Modifie l'article 2.5 « Réponse apportée au salarié » (départs volontaires), suite aux observations de l'inspection du travail.</t>
   </si>
   <si>
@@ -439,18 +409,12 @@
     <t>PERCOL propre à NNF : gestion libre ou pilotée, abondement, transfert collectif des avoirs.</t>
   </si>
   <si>
-    <t>Pas d'accord sur la GEPP.</t>
-  </si>
-  <si>
     <t>Ouverture après 6 mois de présence. Monétisation 1 fois par an (juin), 10 jours max. 5e semaine non monétisable.</t>
   </si>
   <si>
     <t>Enveloppe max = 4 % de la masse salariale selon CA (50 %), brevets/publications (25 %), mobilité durable (25 %). Répartition 50 % présence, 50 % salaire.</t>
   </si>
   <si>
-    <t>Pas d'accord sur les salaires 2025.</t>
-  </si>
-  <si>
     <t>Aide à l'équipement de 300 € (note de frais, sous 6 mois). Indemnité de télétravail de 4 € à 4,40 €, sans indexation.</t>
   </si>
   <si>
@@ -466,9 +430,6 @@
     <t>Mise en conformité avec la convention de la métallurgie : cadres → groupes F à I, non-cadres → groupes A à E.</t>
   </si>
   <si>
-    <t>Pas d'accord sur les salaires 2024.</t>
-  </si>
-  <si>
     <t>Bonus cible aligné au 01/01/2024 sur le taux Nokia du Job Grade : JG5-6 5 %, JG7 7,5 %, JG8 10 %, JG9 12,5 %, JG10 15 %, JG11 20 %, JG12 25 %, JG13 30 %.</t>
   </si>
   <si>
@@ -481,9 +442,6 @@
     <t>173 départs volontaires max. Congé de mobilité, parcours retraite, aides formation/création/mobilité. Pas de licenciement contraint.</t>
   </si>
   <si>
-    <t>Pas d'accord. Enveloppe unilatérale : 3,21 % cadres, 5 % non-cadres.</t>
-  </si>
-  <si>
     <t>Référent égalité, objectif d'embauches de femmes, 80 % des managers formés, revue de l'ASR.</t>
   </si>
   <si>
@@ -751,15 +709,6 @@
     <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2023_PV_desaccord_p10_signature.jpg</t>
   </si>
   <si>
-    <t>Vote AG extra 04/12/2025 : 0 pour / 17 contre / 4 abst. (21 votants) (autre source)</t>
-  </si>
-  <si>
-    <t>Vote AG extra 04/12/2025 : 0 pour / 15 contre / 6 abst. (21 votants) (autre source)</t>
-  </si>
-  <si>
-    <t>Vote AG extra 24/03/2025 : signature décidée, 24 votants dont 3 procurations (autre source)</t>
-  </si>
-  <si>
     <t>Abondement concentré sur les actions Nokia, rémunération « TTC », exonérations de cotisations ; préférence pour un 13e mois cotisé.</t>
   </si>
   <si>
@@ -781,33 +730,12 @@
     <t>Mesures insuffisantes et trop individualisées. Demande intersyndicale des statistiques réelles d'application.</t>
   </si>
   <si>
-    <t>Signature unanime.</t>
-  </si>
-  <si>
-    <t>Accord signé par toutes les OS représentatives.</t>
-  </si>
-  <si>
-    <t>Accord signé par toutes les OS : augmentation du nombre de DS par OS sur NPS (5 DS pour la CGT).</t>
-  </si>
-  <si>
-    <t>Régime AUXAD : contrepartie obtenue, prise en charge de la mutuelle à 60 % par l'employeur (contre 50 %) et +1 % de masse salariale dans la formule d'intéressement.</t>
-  </si>
-  <si>
-    <t>Accord RCC initial non signé non plus. RCC signée le 19/12/2025 par la CFDT et la CFE-CGC ; avenant signé le 15/01/2026 ; nouvelle demande de validation à l'administration le 21/01/2026.</t>
-  </si>
-  <si>
     <t>Débat interne : le DSC voulait d'abord ne pas signer pour « faire front » avec les autres OS ; signature finalement décidée, le gain pour les salariés étant jugé « énorme ».</t>
   </si>
   <si>
-    <t>Nouvelle réduction d'effectifs : 231 suppressions de postes en 2024. (autre source, non retrouvé dans le PDF qui indique 347 maximum) Signé par toutes les OS, y compris la CFTC.</t>
-  </si>
-  <si>
     <t>Version présentée comme finale le 29/11/2023 ; AG CGT le 01/12/2023 avec vote consolidé NPS + Lannion.</t>
   </si>
   <si>
-    <t>Version finale transmise le 03/07/2023, mise à la signature le 04/07/2023 à Massy ; jusqu'à 173 départs volontaires.</t>
-  </si>
-  <si>
     <t>accord majoritaire</t>
   </si>
   <si>
@@ -817,9 +745,6 @@
     <t>Décision unilatérale : prime négociée seulement si bénéfice net fiscal &gt; 15 % du CA France.</t>
   </si>
   <si>
-    <t>Unité syndicale initiale contre ce « chantage », puis signature isolée de la CFDT majoritaire.</t>
-  </si>
-  <si>
     <t>Aucune solution pour les salariés aux compteurs d'heures positifs (remise à zéro = heures non payées, non cotisées).</t>
   </si>
   <si>
@@ -835,69 +760,27 @@
     <t>Vote CGT commun NNF (accord-cadre nouvelle CCN) : 21 votants, 13 pour, 2 contre, 6 abstentions (NPS 5/2/4, Lannion 8/0/2). Tracts : « Et toi alors, t'es coté combien ? », « Mais pourquoi tant de (M)N ? », « MN : des couleuvres ou des spaghettis ».</t>
   </si>
   <si>
-    <t>L'avocat du CSE-C a obtenu ce que la Direction proposait en échange d'une signature ; fin d'une injustice pour ~400 salariés sous le taux nominal de leur grade.</t>
-  </si>
-  <si>
-    <t>Signature unanime des OS. Source : communication intersyndicale.</t>
-  </si>
-  <si>
-    <t>Signé le 12/04/2023 par la CFDT et la CFE-CGC seulement. Vote dans les 2 syndicats (Lannion et IDF).</t>
-  </si>
-  <si>
     <t>Débat/vote en AG extra le 15/07/2026. Slogan du tract : « RCC 2026, c'est toujours non ».</t>
   </si>
   <si>
-    <t>La Direction (M. Cudot) refuse toute modification du texte et exige une réponse avant le 10/07/2026 12h. Signature électronique de toutes les OS le 13/07/2026 (2e procédure, les pages n'ayant pas été paraphées au 1er essai). Risque relevé en interne qu'un échange de mails remplace une vraie négociation.</t>
-  </si>
-  <si>
     <t>Vote en AG extraordinaire du 21/05/2026. La CFE-CGC signe après le vote de ses adhérents mais juge l'accord « nettement insuffisant » (« handiwashing ») ; sa signature plus celle d'une autre OS permet l'application de l'accord. Méthode jugée déloyale (bilatérales « en coulisses »), relations tendues.</t>
   </si>
   <si>
-    <t>Confirmation par courriel. Signature CGT annoncée le 26/01/2026 après débat/vote des syndiqués ; R1 le 19/01, réunion finale le 23/01/2026. Négociation accélérée en 7 jours, peu de lecture des statistiques ; « chantage à la signature » évoqué en débat.</t>
-  </si>
-  <si>
-    <t>Accord signé le 19/12/2025 par la CFDT (adhérents majoritairement pour) et la CFE-CGC, sans la CGT. AG extra le 17/11/2025, débat/vote le 18/12/2025. Slogan : « le bon chiffre c'est zéro ».</t>
-  </si>
-  <si>
     <t>Débat/vote en AG extra fin juin 2025. Négociation précipitée : dernier round supprimé, pas de texte final avant le vote.</t>
   </si>
   <si>
-    <t>Enveloppe d'environ 2 % (0,68 % après inflation). Signature CFDT isolée, non majoritaire. (autre source, à vérifier) Action : blocage des calendriers (~600 salariés).</t>
-  </si>
-  <si>
-    <t>Vote AG extra 11-12/02/2025 : 14 pour / 14 contre / 2 abst. (NPS 8/7/1, Lannion 6/7/1) ; égalité = contre (autre source) Accord initial signé par la CFTC et la CFDT ; la CFTC n'étant plus représentative, la Direction avait besoin de la signature CFE-CGC ou CGT (« chantage affectif »). Rapport de force jugé suffisant pour obtenir plus.</t>
-  </si>
-  <si>
     <t>Une seule réunion de négociation (31/05/2024). La CFE-CGC refuse d'abord de signer le PV (ses positions n'y sont pas reprises) ; la Direction ajoute ses revendications le 31/07/2024. La CGT maintient son refus de signer le PV. PV de désaccord à durée déterminée : nouvelle négociation possible après un an. Négociation jugée déloyale : la Direction voulait « cocher la case ».</t>
   </si>
   <si>
-    <t>Mobilisation intersyndicale CFDT / CFE-CGC / CGT en mars 2024. (source : tract, à vérifier) Actions : communiqué de presse, lettre à l'inspection du travail sur la loyauté des négociations, déconnexion à 16h / calendriers.</t>
-  </si>
-  <si>
     <t>Modalités électorales (vote électronique, calendrier, collèges, nombre de sièges, répartition H/F) négociées en commun avec Paris-Saclay et jugées conformes.</t>
   </si>
   <si>
     <t>Modalités électorales (vote électronique, calendrier, collèges, nombre de sièges, répartition H/F, effectifs de référence) jugées conformes.</t>
   </si>
   <si>
-    <t>Contenu : la restauration sort des ASC des CSE-E et passe en gestion Direction (budget ASC modifié, commission restauration redéfinie). Avis favorable de toutes les OS sur le projet.</t>
-  </si>
-  <si>
     <t>Contre : pas de budget spécifique ni d'heures de délégation pour les référents ; mission handicap réduite à 1 personne nommée par la Direction ; élus non associés aux décisions (commission paritaire supprimée, simple bilan annuel) ; maintien dans l'emploi en recul par rapport à 2021 ; jours d'absence sur demande avec justificatif. Demandes CGT non retenues : rôle formalisé de la CSSCT, secrétaire CSSCT dans la mission handicap, lien AGEFIPH, mesures contre le plafond de verre (bac+2/3). Pour : sans accord, seulement le minimum légal (ni aide de 200 €, ni jours de congé) ; CSSCT associée aux études de poste ; TPC prolongeable au-delà de 5 ans avec retraite et prévoyance à 100 %.</t>
   </si>
   <si>
-    <t>Prorogation technique des mandats CSE-E Lannion (17/11 → 06/12/2026) pour aligner les élections sur celles de Paris-Saclay ; aucun enjeu de fond défavorable.</t>
-  </si>
-  <si>
-    <t>Pour : enveloppe portée de 1,85 % à 2,15 % (+0,30 point) conditionnée à la signature, avec hausse des primes de transport (vélo 400 → 500 €, indemnité kilométrique) et des primes d'intervention (forfait 265 € au lieu de 250 €) ; mobilisation jugée difficile. Contre : aucune augmentation générale ; revendications CGT refusées (rattrapage de 5 % depuis 2021 + 4 %) ; individualisation ; les femmes restent moins augmentées, écart plus fort à Lannion.</t>
-  </si>
-  <si>
-    <t>Avenant de procédure (article 2.5, suite aux observations de l'inspection du travail) à une RCC que la CGT n'a pas signée.</t>
-  </si>
-  <si>
-    <t>Fixation des ponts : 1 JRTT/JRS collectif le 15/05/2026 et journée de solidarité le 25/05/2026 ; accord technique sans recul.</t>
-  </si>
-  <si>
     <t>Pour : souplesse pour les salariés, jour supplémentaire à Lannion. Contre : monétisation des congés (repos transformé en argent), 5e semaine exclue mais logique banalisée.</t>
   </si>
   <si>
@@ -910,12 +793,6 @@
     <t>Pour : 1 jour de repos supplémentaire pour tous, aligné sur Paris-Saclay. Contre : prime de crèche (80 €/mois jusqu'aux 4 ans de l'enfant) fermée aux nouveaux entrants au 01/01/2026, congés familiaux supprimés ; risque de préparer un établissement unique NPS + Lannion.</t>
   </si>
   <si>
-    <t>Pour : indemnité +10 % (4 € → 4,40 €), maintien de l'accord, aide à l'équipement de 300 € plus favorable que le dispositif corporate. Contre : pas d'indexation, aide non renouvelable, hausse financée par les sommes non utilisées ; accord initial non signé par la CGT.</t>
-  </si>
-  <si>
-    <t>Fixation des ponts et de la journée de solidarité 2025 ; accord technique sans recul.</t>
-  </si>
-  <si>
     <t>Versement conditionné à un bénéfice net fiscal &gt; 15 % du CA, inatteignable vu le déficit comptable de NNF (héritage Alcatel-Lucent, R&amp;D sous-facturée à la maison mère) : aucune prime possible en pratique. Revendication : du salaire fixe plutôt que des primes.</t>
   </si>
   <si>
@@ -925,9 +802,6 @@
     <t>Contre : nouvelle classification, fiches emplois et cotation des postes ; fin de la reconnaissance des diplômes et de l'expérience, salaire lié au poste, perte possible du statut cadre. Pour : CCN imposée par la branche, l'accord-cadre en encadre la mise en place dans l'entreprise.</t>
   </si>
   <si>
-    <t>Fixation des ponts et de la journée de solidarité 2024 ; accord technique sans recul.</t>
-  </si>
-  <si>
     <t>Correction demandée par la CGT obtenue (« salaire fixe » au lieu de « salaire de base »).</t>
   </si>
   <si>
@@ -937,15 +811,6 @@
     <t>Pour : quelques actions (formation des managers, candidature féminine recherchée pour les postes de management). Contre : pas d'enveloppe budgétaire spécifique, aucune amélioration proposée par la CGT retenue.</t>
   </si>
   <si>
-    <t>Fixation des ponts et de la journée de solidarité 2023 ; accord technique sans recul.</t>
-  </si>
-  <si>
-    <t>Augmentation des moyens syndicaux (nombre de DS par OS à Lannion).</t>
-  </si>
-  <si>
-    <t>Augmentation des moyens syndicaux (5 DS pour la CGT sur NPS).</t>
-  </si>
-  <si>
     <t>Accord sur le régime de remboursement des frais de santé, sans recul identifié.</t>
   </si>
   <si>
@@ -956,13 +821,235 @@
   </si>
   <si>
     <t>Jusqu'à 421 suppressions de postes non justifiées par la charge de travail ; RCC à répétition ; ni garantie d'emploi ni embauche ; externalisations et perte de compétences ; critères de substitution ; pression au volontariat.</t>
+  </si>
+  <si>
+    <t>GEPP</t>
+  </si>
+  <si>
+    <t>NAO 2025</t>
+  </si>
+  <si>
+    <t>Partage de la valeur</t>
+  </si>
+  <si>
+    <t>NAO 2024</t>
+  </si>
+  <si>
+    <t>NAO 2023</t>
+  </si>
+  <si>
+    <t>Pas d'accord : la Direction refuse tout plan d'embauche (« 1 départ = 1 embauche »). Mesures unilatérales pour 3 ans : forums métiers et mobilité internationale ; prime de mobilité inter-région de 10 000 € brut, déménagement jusqu'à 5 000 € HT et 1 jour de congé ; priorité au recrutement interne et aux jeunes diplômés ; TPC seniors prolongeable au-delà de 5 ans avec retraite et prévoyance à 100 % ; entretiens de début et de cours de mandat pour les élus. Suivi annuel en CSE-C.</t>
+  </si>
+  <si>
+    <t>accord collectif relatif aux évolutions du régime AUXAD -VF.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/BDESENNF-CSE-C/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FBDESENNF%2DCSE%2DC%2FShared%20Documents%2F05a%2E%20CSE%2DC%2FCSE%2DC%202025%2F03%2DCSE%2DC%20extraordinaire%209%20avril%202025%2Faccord%20collectif%20relatif%20aux%20%C3%A9volutions%20du%20r%C3%A9gime%20AUXAD%20%2DVF%2Epdf</t>
+  </si>
+  <si>
+    <t>Évolutions du régime AUXAD</t>
+  </si>
+  <si>
+    <t>Le règlement de la retraite supplémentaire AUXAD (anciens hauts salaires Alcatel, rémunération &gt; 8 PASS, environ 250 ayants droit) devient accord collectif dans sa version du 01/10/2021 : valeur du point figée à celle du 30/09/2021, sans revalorisation. Objectif : sécuriser le régime face aux recours de retraités (jurisprudence Cass. 19/01/2022). Engagement de négocier avant toute évolution. Durée indéterminée. Contreparties : mutuelle prise en charge à 60 % (au lieu de 50 %) et intéressement à 4 % de la masse salariale (au lieu de 3 %).</t>
+  </si>
+  <si>
+    <t>Pour : gain substantiel pour les salariés (mutuelle 60/40 à vie, intéressement 4 % MS), autofinancé par la fin de l'indexation d'une retraite chapeau de très hauts salaires. Contre : contreparties qui ne font qu'aligner sur les pratiques du marché ; aucune contrepartie salariale ; gain principal sur l'intéressement, limité à 4 ans.</t>
+  </si>
+  <si>
+    <t>La Direction (M. Cudot) refuse toute modification du texte et exige une réponse avant le 10/07/2026 12h. Signature électronique le 13/07/2026 (2e procédure, les pages n'ayant pas été paraphées au 1er essai). Avis favorable de toutes les OS sur le projet. Risque relevé en interne qu'un échange de mails remplace une vraie négociation.</t>
+  </si>
+  <si>
+    <t>Favorable au transfert de la restauration à la Direction.</t>
+  </si>
+  <si>
+    <t>Accord technique, aucun enjeu de fond défavorable.</t>
+  </si>
+  <si>
+    <t>Pas d'augmentation générale. Augmentations individuelles 2,15 % des TTC (promotions incluses ; GPP et Unexplained Pay Gap maintenus) au 01/04/2026. Primes de transport au 01/04/2026 : zone 1 9 €, zone 2 12 €, zone 3 60 €. Forfait vélo porté de 400 € à 500 €/an (60 €/mois, 0,36 €/km). Astreinte 265 € (+6 %), ticket astreinte 22 € ; travail de nuit 140 € (&lt;5 h) / 280 € (&gt;5 h), nuit de WE 160 € / 320 €, samedi 320 €. Expire le 30/04/2027.</t>
+  </si>
+  <si>
+    <t>Avenant du 15/01/2026 ; nouvelle demande de validation à l'administration le 21/01/2026.</t>
+  </si>
+  <si>
+    <t>Avenant de procédure sans contenu nouveau ; opposition maintenue à la RCC elle-même.</t>
+  </si>
+  <si>
+    <t>Accord technique sans recul.</t>
+  </si>
+  <si>
+    <t>CFDT : adhérents majoritairement pour. AG extra le 17/11/2025, débat/vote le 18/12/2025. Slogan : « le bon chiffre c'est zéro ».</t>
+  </si>
+  <si>
+    <t>Vote AG extra 04/12/2025 : 0 pour / 17 contre / 4 abst. (21 votants).</t>
+  </si>
+  <si>
+    <t>Vote AG extra 04/12/2025 : 0 pour / 15 contre / 6 abst. (21 votants).</t>
+  </si>
+  <si>
+    <t>PV de désaccord signé par la DRH et les DSC CFDT, CFE-CGC et CGT (à vérifier). La CFDT et la CGT refusent de signer un accord sans plan d'embauche.</t>
+  </si>
+  <si>
+    <t>Pour : prise en charge employeur portée à 60 % (contre 50 %), gain jugé très important pour les salariés ; contrepartie de l'accord AUXAD.</t>
+  </si>
+  <si>
+    <t>Vote AG extra 24/03/2025 (24 votants dont 3 procurations).</t>
+  </si>
+  <si>
+    <t>Pas d'accord majoritaire. Mesures unilatérales : budget d'augmentations individuelles de 2 % des TTC, pas d'augmentation générale ; GPP et Unexplained Pay Gap maintenus. Primes de transport +5 % au 01/07/2025 : zone 1 7,98 €, zone 2 10,93 €, zone 3 57,45 €. Expire le 30/06/2026.</t>
+  </si>
+  <si>
+    <t>Réunions des 17/12/2024, 27/01, 03/03 et 12/03/2025 ; PV de désaccord du 27/03/2025 ; accord séparé signé par la seule CFDT (20/03/2025), non majoritaire. Action : blocage des calendriers (~600 salariés).</t>
+  </si>
+  <si>
+    <t>Unité syndicale initiale contre ce « chantage », rompue par la CFDT (majoritaire).</t>
+  </si>
+  <si>
+    <t>Vote AG extra 11-12/02/2025 : 14 pour / 14 contre / 2 abst. (NPS 8/7/1, Lannion 6/7/1) ; égalité = contre. Accord initial signé par la CFTC et la CFDT ; la CFTC n'étant plus représentative, la Direction avait besoin de la signature CFE-CGC ou CGT (« chantage affectif »). Rapport de force jugé suffisant pour obtenir plus.</t>
+  </si>
+  <si>
+    <t>Pour : indemnité +10 % (4 € → 4,40 €), maintien de l'accord, aide à l'équipement de 300 € plus favorable que le dispositif corporate. Contre : pas d'indexation, aide non renouvelable, hausse financée par les sommes non utilisées.</t>
+  </si>
+  <si>
+    <t>Compteur &gt; 900 jours (à vérifier).</t>
+  </si>
+  <si>
+    <t>Nouvelle réduction d'effectifs : 231 suppressions de postes en 2024 (non retrouvé dans le PDF, qui indique 347 maximum).</t>
+  </si>
+  <si>
+    <t>Pas d'accord. Enveloppe unilatérale relevée de 0,66 point à 1,81 % des TTC, uniquement en augmentations individuelles ; GPP et Unexplained Pay Gap maintenus. Primes de transport et IK voiture inchangées. Expire le 30/06/2025.</t>
+  </si>
+  <si>
+    <t>Réunions des 06/12/2023, 25/01 et 08/02/2024, puis PV de désaccord ; réouverture le 02/04/2024 ; avenant au PV du 09/04/2024. Mobilisation intersyndicale CFDT / CFE-CGC / CGT en mars 2024 (source : tract, à vérifier). Actions : communiqué de presse, lettre à l'inspection du travail sur la loyauté des négociations, déconnexion à 16h / calendriers.</t>
+  </si>
+  <si>
+    <t>Dénoncé en 2025 (sortie d'ASN, fermeture de RFS) (à vérifier).</t>
+  </si>
+  <si>
+    <t>Version finale transmise le 03/07/2023, mise à la signature le 04/07/2023 à Massy.</t>
+  </si>
+  <si>
+    <t>Pas d'accord. Mesures unilatérales au 01/07/2023 : augmentations individuelles 3,21 % des TTC pour les JG 6 et plus, 5 % pour les JG 5 et moins ; GPP et Unexplained Pay Gap maintenus. Primes de transport +5 % ; prime vélo portée à 500 €/an (60 €/mois) ; IK vélo +40 % à 0,35 €/km. Expire le 30/06/2024.</t>
+  </si>
+  <si>
+    <t>Réunions des 24/03, 29/03 et 05/04/2023 ; PV de désaccord du 12/04/2023. Contestation des nombreux 0 % d'augmentation (source : tract, à vérifier).</t>
+  </si>
+  <si>
+    <t>Vote dans les 2 syndicats (Lannion et IDF).</t>
+  </si>
+  <si>
+    <t>Favorable : renforcement des moyens syndicaux (2 DS par OS à Lannion).</t>
+  </si>
+  <si>
+    <t>Favorable : renforcement des moyens syndicaux (5 DS pour la CGT sur NPS).</t>
+  </si>
+  <si>
+    <t>Règles de remplissage de la feuille accords</t>
+  </si>
+  <si>
+    <t>Pour : enveloppe portée de 1,85 % à 2,15 % (+0,30 point), hausse des primes de transport (vélo 400 → 500 €, indemnité kilométrique) et des primes d'intervention (forfait 265 € au lieu de 250 €). Contre : aucune augmentation générale ; revendications CGT refusées (rattrapage de 5 % depuis 2021 + 4 %) ; individualisation ; les femmes restent moins augmentées, écart plus fort à Lannion.</t>
+  </si>
+  <si>
+    <t>Confirmation par courriel. Débat/vote des syndiqués avant le 26/01/2026 ; R1 le 19/01, réunion finale le 23/01/2026 ; accord fait à Massy le 27/01/2026. Négociation accélérée en 7 jours, peu de lecture des statistiques ; +0,30 point conditionné à la signature (« chantage à la signature ») ; mobilisation jugée difficile.</t>
+  </si>
+  <si>
+    <t>Fin d'une injustice pour ~400 salariés sous le taux nominal de leur grade.</t>
+  </si>
+  <si>
+    <t>Source : communication intersyndicale. Résultat obtenu par l'avocat du CSE-C (ce que la Direction proposait en échange d'une signature).</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_accord_collectif_relatif_aux_evolutions_du_regime_AUXAD_VF_p06_signature.jpg</t>
+  </si>
+  <si>
+    <t>Vote AG extra CGT du 27/03/2025 : « La CGT signe l'accord AUXAD et ses contreparties ». Réunions des 13/02 et 28/03/2025 ; courriel Direction du 31/03/2025 (mise à la signature au 09/04/2025) ; info-consultation CSE-C extraordinaire du 09/04/2025. Argumentaire AG CGT (mars 2025). Négociation au pas de course, quasi exclusivement en bilatérales DSC, opacité sur les sommes provisionnées.</t>
+  </si>
+  <si>
+    <t>Colonne</t>
+  </si>
+  <si>
+    <t>Règle</t>
+  </si>
+  <si>
+    <t>Général</t>
+  </si>
+  <si>
+    <t>Colonnes repérées par leur en-tête, jamais par leur lettre (l'ordre peut changer). Lignes triées par date décroissante.</t>
+  </si>
+  <si>
+    <t>Pas de redondance entre colonnes : chaque info n'apparaît qu'à un seul endroit.</t>
+  </si>
+  <si>
+    <t>Phrases courtes et factuelles, en français. Dates au format jj/mm/aaaa.</t>
+  </si>
+  <si>
+    <t>Une valeur non confirmée = « À vérifier ». Une valeur sans objet = « - ».</t>
+  </si>
+  <si>
+    <t>année, site</t>
+  </si>
+  <si>
+    <t>Année de l'accord ; site = NNF, NPS ou LAN.</t>
+  </si>
+  <si>
+    <t>Titre court, objet seul. Ajouter l'année quand l'objet se répète (NAO, RCC, aménagement du temps de travail).</t>
+  </si>
+  <si>
+    <t>URL accord, file name accord</t>
+  </si>
+  <si>
+    <t>Plusieurs documents : URLs séparées par des virgules, noms de fichier dans le même ordre. Le nom de fichier est le nom exact. Pas de %2F dans le chemin.</t>
+  </si>
+  <si>
+    <t>Date finale lue dans le PDF (signature, validation ou page de garde), en vraie date au format jj/mm/aaaa. Vide = -. Date uniquement dans cette colonne.</t>
+  </si>
+  <si>
+    <t>TRUE = accord ; FALSE = pas d'accord (PV de désaccord) ; À vérifier sinon.</t>
+  </si>
+  <si>
+    <t>CGT, CFDT, CFE-CGC, CFTC</t>
+  </si>
+  <si>
+    <t>TRUE = signature confirmée ; FALSE = non signataire ; À vérifier ; - = OS non concernée. Seul endroit où figure le statut signé / non signé.</t>
+  </si>
+  <si>
+    <t>Pas d'accord (PV de désaccord) : aucune signature d'accord collectif.</t>
+  </si>
+  <si>
+    <t>URL de la capture de la page de signature (dossier captures_signatures). Vide si pas de capture.</t>
+  </si>
+  <si>
+    <t>Format unique : « p.X : signatures de la Direction, de la CFDT, de la CFE-CGC et de la CGT. » en nommant les organisations visibles et toute absence (« ; aucune signature de la CGT »).</t>
+  </si>
+  <si>
+    <t>Pas de noms de personnes, pas de nom de fichier, pas de date, pas de vote AG, pas de courriel : aucune info parasite.</t>
+  </si>
+  <si>
+    <t>Signaler une version non signée. PV de désaccord : « PV de désaccord valide unilatéralement ; aucun accord collectif n’a été signé. »</t>
+  </si>
+  <si>
+    <t>Résumé court du fond uniquement (mesures, chiffres, dates d'effet, durée). Aucune info méta (réunions, votes, signatures, procédure, sources).</t>
+  </si>
+  <si>
+    <t>Analyse de fond de la CGT uniquement (pour / contre, revendications). Pas de statut signé / non signé, pas de vote, pas de déroulé. Affichée après le résumé, préfixée « Position CGT : ».</t>
+  </si>
+  <si>
+    <t>Toutes les infos méta : réunions, votes AG, déroulé et méthode de négociation, courriels, positions des autres OS, mentions à vérifier. Notes de travail, non reprises dans l'index.</t>
+  </si>
+  <si>
+    <t>Titre du tract. Plusieurs tracts : un titre par ligne, dans l'ordre des URLs. - = pas de tract.</t>
+  </si>
+  <si>
+    <t>URL tract, file name tract</t>
+  </si>
+  <si>
+    <t>URL absolue et encodée. Le nom du fichier tract doit correspondre à la fin de l'URL tract.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1013,13 +1100,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="7">
@@ -1107,7 +1208,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1139,19 +1240,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1169,59 +1264,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="27">
     <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1299,39 +1378,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFD8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1378,6 +1425,112 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFD8A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1661,25 +1814,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr defaultColWidth="12.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" style="19" customWidth="1"/>
-    <col min="3" max="3" width="41.28515625" style="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.28515625" style="17" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" style="17" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" style="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37.5703125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42.42578125" style="19" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" style="19" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" style="19" customWidth="1"/>
-    <col min="8" max="10" width="9.28515625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.28515625" style="19" customWidth="1"/>
-    <col min="12" max="12" width="26.42578125" style="20" customWidth="1"/>
-    <col min="13" max="13" width="49.5703125" style="19" customWidth="1"/>
-    <col min="14" max="16" width="57.140625" style="19" customWidth="1"/>
-    <col min="17" max="17" width="36.28515625" style="19" customWidth="1"/>
-    <col min="18" max="18" width="36.85546875" style="20" customWidth="1"/>
-    <col min="19" max="19" width="32.28515625" style="19" customWidth="1"/>
-    <col min="20" max="16384" width="12.140625" style="19"/>
+    <col min="5" max="5" width="42.42578125" style="17" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" style="17" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="17" customWidth="1"/>
+    <col min="8" max="10" width="9.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.28515625" style="17" customWidth="1"/>
+    <col min="12" max="12" width="26.42578125" style="18" customWidth="1"/>
+    <col min="13" max="13" width="49.5703125" style="17" customWidth="1"/>
+    <col min="14" max="16" width="57.140625" style="17" customWidth="1"/>
+    <col min="17" max="17" width="36.28515625" style="17" customWidth="1"/>
+    <col min="18" max="18" width="36.85546875" style="18" customWidth="1"/>
+    <col min="19" max="19" width="32.28515625" style="17" customWidth="1"/>
+    <col min="20" max="16384" width="12.140625" style="17"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" x14ac:dyDescent="0.25">
@@ -1693,16 +1846,16 @@
         <v>0</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>10</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>248</v>
+        <v>224</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>1</v>
@@ -1714,31 +1867,31 @@
         <v>3</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>249</v>
+        <v>225</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="P1" s="8" t="s">
         <v>11</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="90" x14ac:dyDescent="0.25">
@@ -1749,10 +1902,10 @@
         <v>13</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>40</v>
+        <v>23</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>35</v>
       </c>
       <c r="E2" s="11" t="str" cm="1">
         <f t="array" ref="E2">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D2,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -1778,26 +1931,26 @@
         <f>IF(OR(B2="NNF",B2="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M2)))</f>
         <v>-</v>
       </c>
-      <c r="L2" s="21" t="s">
-        <v>69</v>
+      <c r="L2" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="N2" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="O2" s="14" t="s">
-        <v>260</v>
-      </c>
-      <c r="P2" s="14" t="s">
-        <v>295</v>
-      </c>
-      <c r="Q2" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="R2" s="21" t="s">
-        <v>46</v>
+        <v>190</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q2" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="R2" s="19" t="s">
+        <v>41</v>
       </c>
       <c r="S2" s="11" t="str" cm="1">
         <f t="array" ref="S2">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R2,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -1809,13 +1962,13 @@
         <v>2026</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>168</v>
+        <v>144</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>154</v>
       </c>
       <c r="E3" s="11" t="str" cm="1">
         <f t="array" ref="E3">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D3,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -1839,26 +1992,24 @@
         <v>1</v>
       </c>
       <c r="K3" s="13" t="str">
-        <f t="shared" ref="K3:K40" si="0">IF(OR(B3="NNF",B3="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M3)))</f>
+        <f>IF(OR(B3="NNF",B3="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M3)))</f>
         <v>-</v>
       </c>
-      <c r="L3" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>202</v>
-      </c>
-      <c r="N3" s="14" t="s">
+      <c r="L3" s="19" t="s">
         <v>178</v>
       </c>
-      <c r="O3" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="P3" s="19" t="s">
-        <v>270</v>
-      </c>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="21"/>
+      <c r="M3" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="N3" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="O3" s="11"/>
+      <c r="P3" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="19"/>
       <c r="S3" s="11"/>
     </row>
     <row r="4" spans="1:19" ht="45" x14ac:dyDescent="0.25">
@@ -1869,10 +2020,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>169</v>
+        <v>145</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>155</v>
       </c>
       <c r="E4" s="11" t="str" cm="1">
         <f t="array" ref="E4">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D4,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -1896,26 +2047,24 @@
         <v>1</v>
       </c>
       <c r="K4" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L4" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="M4" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="N4" s="14" t="s">
+        <f>IF(OR(B4="NNF",B4="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M4)))</f>
+        <v>1</v>
+      </c>
+      <c r="L4" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="O4" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="P4" s="19" t="s">
-        <v>271</v>
-      </c>
-      <c r="Q4" s="17"/>
-      <c r="R4" s="21"/>
+      <c r="M4" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="N4" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="11"/>
+      <c r="P4" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="19"/>
       <c r="S4" s="11"/>
     </row>
     <row r="5" spans="1:19" ht="90" x14ac:dyDescent="0.25">
@@ -1926,10 +2075,10 @@
         <v>13</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>109</v>
+        <v>60</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>100</v>
       </c>
       <c r="E5" s="11" t="str" cm="1">
         <f t="array" ref="E5">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D5,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -1952,28 +2101,28 @@
         <v>1</v>
       </c>
       <c r="K5" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B5="NNF",B5="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M5)))</f>
         <v>-</v>
       </c>
-      <c r="L5" s="21" t="s">
-        <v>70</v>
+      <c r="L5" s="19" t="s">
+        <v>65</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="N5" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="O5" s="14" t="s">
-        <v>261</v>
-      </c>
-      <c r="P5" s="14" t="s">
-        <v>272</v>
-      </c>
-      <c r="Q5" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R5" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="N5" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="Q5" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R5" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S5" s="11" t="str" cm="1">
@@ -1991,10 +2140,10 @@
       <c r="C6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="E6" s="15" t="str" cm="1">
+      <c r="D6" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="10" t="str" cm="1">
         <f t="array" ref="E6">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D6,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v>Accord d'entreprise relatif à la situation de handicap NNF.pdf</v>
       </c>
@@ -2015,31 +2164,31 @@
         <v>1</v>
       </c>
       <c r="K6" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B6="NNF",B6="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M6)))</f>
         <v>-</v>
       </c>
-      <c r="L6" s="21" t="s">
-        <v>190</v>
+      <c r="L6" s="19" t="s">
+        <v>176</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="P6" s="19" t="s">
-        <v>273</v>
-      </c>
-      <c r="Q6" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="R6" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="S6" s="15" t="str" cm="1">
+        <v>233</v>
+      </c>
+      <c r="P6" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q6" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="R6" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="S6" s="10" t="str" cm="1">
         <f t="array" ref="S6">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R6,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v/>
       </c>
@@ -2049,13 +2198,13 @@
         <v>2026</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>176</v>
+        <v>149</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>162</v>
       </c>
       <c r="E7" s="11" t="str" cm="1">
         <f t="array" ref="E7">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D7,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2079,24 +2228,24 @@
         <v>1</v>
       </c>
       <c r="K7" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B7="NNF",B7="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M7)))</f>
         <v>-</v>
       </c>
-      <c r="L7" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="M7" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="N7" s="14" t="s">
+      <c r="L7" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="O7" s="14"/>
-      <c r="P7" s="19" t="s">
-        <v>274</v>
-      </c>
-      <c r="Q7" s="17"/>
-      <c r="R7" s="21"/>
+      <c r="M7" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="N7" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="O7" s="11"/>
+      <c r="P7" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="19"/>
       <c r="S7" s="11"/>
     </row>
     <row r="8" spans="1:19" ht="120" x14ac:dyDescent="0.25">
@@ -2107,10 +2256,10 @@
         <v>13</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>110</v>
+        <v>54</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>101</v>
       </c>
       <c r="E8" s="11" t="str" cm="1">
         <f t="array" ref="E8">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D8,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2134,28 +2283,28 @@
         <v>1</v>
       </c>
       <c r="K8" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B8="NNF",B8="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M8)))</f>
         <v>-</v>
       </c>
-      <c r="L8" s="21" t="s">
-        <v>71</v>
+      <c r="L8" s="19" t="s">
+        <v>66</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="N8" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="O8" s="14" t="s">
-        <v>263</v>
-      </c>
-      <c r="P8" s="19" t="s">
-        <v>275</v>
-      </c>
-      <c r="Q8" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R8" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="P8" s="21" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q8" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R8" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S8" s="11" t="str" cm="1">
@@ -2163,7 +2312,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="10">
         <v>2026</v>
       </c>
@@ -2171,10 +2320,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>66</v>
+        <v>53</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>61</v>
       </c>
       <c r="E9" s="11" t="str" cm="1">
         <f t="array" ref="E9">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D9,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2197,28 +2346,28 @@
         <v>1</v>
       </c>
       <c r="K9" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B9="NNF",B9="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M9)))</f>
         <v>-</v>
       </c>
-      <c r="L9" s="21" t="s">
-        <v>72</v>
+      <c r="L9" s="19" t="s">
+        <v>67</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>207</v>
-      </c>
-      <c r="N9" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="O9" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="P9" s="14" t="s">
-        <v>276</v>
-      </c>
-      <c r="Q9" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R9" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q9" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R9" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S9" s="11" t="str" cm="1">
@@ -2234,12 +2383,12 @@
         <v>14</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="15" t="str" cm="1">
+        <v>52</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="10" t="str" cm="1">
         <f t="array" ref="E10">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D10,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v>Accord Aménagement Temps Travail NPS 2026 (19 décembre 2025).pdf</v>
       </c>
@@ -2260,29 +2409,29 @@
         <v>1</v>
       </c>
       <c r="K10" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L10" s="21" t="s">
-        <v>73</v>
+        <f>IF(OR(B10="NNF",B10="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M10)))</f>
+        <v>1</v>
+      </c>
+      <c r="L10" s="19" t="s">
+        <v>68</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="Q10" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="R10" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="S10" s="15" t="str" cm="1">
+        <v>270</v>
+      </c>
+      <c r="Q10" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="R10" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="S10" s="10" t="str" cm="1">
         <f t="array" ref="S10">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R10,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v/>
       </c>
@@ -2295,10 +2444,10 @@
         <v>13</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>111</v>
+        <v>51</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>102</v>
       </c>
       <c r="E11" s="11" t="str" cm="1">
         <f t="array" ref="E11">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D11,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2321,29 +2470,29 @@
         <v>1</v>
       </c>
       <c r="K11" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B11="NNF",B11="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M11)))</f>
         <v>-</v>
       </c>
-      <c r="L11" s="21" t="s">
-        <v>74</v>
+      <c r="L11" s="19" t="s">
+        <v>69</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="N11" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="O11" s="14" t="s">
-        <v>264</v>
-      </c>
-      <c r="P11" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="Q11" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="R11" s="21" t="s">
-        <v>47</v>
+        <v>195</v>
+      </c>
+      <c r="N11" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="O11" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="P11" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q11" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="R11" s="19" t="s">
+        <v>42</v>
       </c>
       <c r="S11" s="11" t="str" cm="1">
         <f t="array" ref="S11">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R11,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2360,8 +2509,8 @@
       <c r="C12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="21" t="s">
-        <v>112</v>
+      <c r="D12" s="19" t="s">
+        <v>103</v>
       </c>
       <c r="E12" s="11" t="str" cm="1">
         <f t="array" ref="E12">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D12,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2384,28 +2533,28 @@
         <v>1</v>
       </c>
       <c r="K12" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B12="NNF",B12="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M12)))</f>
         <v>-</v>
       </c>
-      <c r="L12" s="21" t="s">
-        <v>75</v>
+      <c r="L12" s="19" t="s">
+        <v>70</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="N12" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="O12" s="14" t="s">
-        <v>229</v>
-      </c>
-      <c r="P12" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="Q12" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R12" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="N12" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="P12" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q12" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R12" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S12" s="11" t="str" cm="1">
@@ -2423,8 +2572,8 @@
       <c r="C13" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="21" t="s">
-        <v>113</v>
+      <c r="D13" s="19" t="s">
+        <v>104</v>
       </c>
       <c r="E13" s="11" t="str" cm="1">
         <f t="array" ref="E13">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D13,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2447,28 +2596,28 @@
         <v>1</v>
       </c>
       <c r="K13" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B13="NNF",B13="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M13)))</f>
         <v>-</v>
       </c>
-      <c r="L13" s="21" t="s">
-        <v>76</v>
+      <c r="L13" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>211</v>
-      </c>
-      <c r="N13" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="O13" s="14" t="s">
-        <v>230</v>
-      </c>
-      <c r="P13" s="14" t="s">
-        <v>233</v>
-      </c>
-      <c r="Q13" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R13" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="N13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="O13" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="P13" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q13" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R13" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S13" s="11" t="str" cm="1">
@@ -2476,7 +2625,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
         <v>2025</v>
       </c>
@@ -2484,10 +2633,10 @@
         <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>33</v>
+        <v>253</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>28</v>
       </c>
       <c r="E14" s="11" t="str" cm="1">
         <f t="array" ref="E14">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D14,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2509,29 +2658,29 @@
         <v>8</v>
       </c>
       <c r="K14" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B14="NNF",B14="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M14)))</f>
         <v>-</v>
       </c>
-      <c r="L14" s="21" t="s">
-        <v>224</v>
+      <c r="L14" s="19" t="s">
+        <v>210</v>
       </c>
       <c r="M14" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="N14" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="O14" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="P14" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q14" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="R14" s="21" t="s">
-        <v>48</v>
+        <v>83</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="O14" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="P14" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q14" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="R14" s="19" t="s">
+        <v>43</v>
       </c>
       <c r="S14" s="11" t="str" cm="1">
         <f t="array" ref="S14">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R14,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2549,7 +2698,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E15" s="11" t="str" cm="1">
         <f t="array" ref="E15">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D15,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2573,28 +2722,28 @@
         <v>1</v>
       </c>
       <c r="K15" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B15="NNF",B15="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M15)))</f>
         <v>-</v>
       </c>
-      <c r="L15" s="21" t="s">
-        <v>77</v>
+      <c r="L15" s="19" t="s">
+        <v>72</v>
       </c>
       <c r="M15" s="12" t="s">
-        <v>212</v>
-      </c>
-      <c r="N15" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="O15" s="14" t="s">
-        <v>265</v>
-      </c>
-      <c r="P15" s="14" t="s">
-        <v>278</v>
-      </c>
-      <c r="Q15" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R15" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="N15" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="O15" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="P15" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q15" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R15" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S15" s="11" t="str" cm="1">
@@ -2602,7 +2751,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A16" s="10">
         <v>2025</v>
       </c>
@@ -2610,21 +2759,19 @@
         <v>13</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="E16" s="11" t="str" cm="1">
-        <f t="array" ref="E16">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D16,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Avenant frais de santé (9 avril 2025).pdf</v>
+        <v>261</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>259</v>
       </c>
       <c r="F16" s="12">
         <f>DATE(2025,4,9)</f>
         <v>45756</v>
       </c>
       <c r="G16" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C16)),TRUE,IF(AND(B16="LAN",I16=TRUE),TRUE,IF(AND(B16="NPS",I16=TRUE,K16=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H16:J16,TRUE),_xlpm.av,COUNTIF(H16:J16,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
         <v>1</v>
       </c>
       <c r="H16" s="13" t="b">
@@ -2636,30 +2783,35 @@
       <c r="J16" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K16" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="L16" s="21" t="s">
-        <v>196</v>
-      </c>
-      <c r="M16" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="N16" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="O16" s="14" t="s">
-        <v>244</v>
-      </c>
-      <c r="P16" s="14" t="s">
-        <v>242</v>
-      </c>
-      <c r="Q16" s="17"/>
-      <c r="R16" s="21"/>
-      <c r="S16" s="11"/>
-    </row>
-    <row r="17" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="K16" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="M16" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="N16" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="O16" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="P16" s="15" t="s">
+        <v>263</v>
+      </c>
+      <c r="Q16" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R16" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="S16" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="10">
         <v>2025</v>
       </c>
@@ -2667,17 +2819,18 @@
         <v>13</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>114</v>
+        <v>148</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>161</v>
       </c>
       <c r="E17" s="11" t="str" cm="1">
         <f t="array" ref="E17">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D17,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord d'intéressement 2025-2028.pdf</v>
+        <v>Avenant frais de santé (9 avril 2025).pdf</v>
       </c>
       <c r="F17" s="12">
-        <v>45744</v>
+        <f>DATE(2025,4,9)</f>
+        <v>45756</v>
       </c>
       <c r="G17" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C17)),TRUE,IF(AND(B17="LAN",I17=TRUE),TRUE,IF(AND(B17="NPS",I17=TRUE,K17=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H17:J17,TRUE),_xlpm.av,COUNTIF(H17:J17,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -2693,36 +2846,29 @@
         <v>1</v>
       </c>
       <c r="K17" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B17="NNF",B17="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M17)))</f>
         <v>-</v>
       </c>
-      <c r="L17" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="M17" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="N17" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="O17" s="14" t="s">
-        <v>231</v>
-      </c>
-      <c r="P17" s="14" t="s">
-        <v>279</v>
-      </c>
-      <c r="Q17" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R17" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="S17" s="11" t="str" cm="1">
-        <f t="array" ref="S17">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R17,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="L17" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="N17" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="O17" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="P17" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="19"/>
+      <c r="S17" s="11"/>
+    </row>
+    <row r="18" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="10">
         <v>2025</v>
       </c>
@@ -2730,58 +2876,59 @@
         <v>13</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>44</v>
+        <v>19</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="E18" s="11" t="str" cm="1">
         <f t="array" ref="E18">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D18,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Procès verbal NAO (désaccord) 2025 (27 mars 2025).pdf</v>
+        <v>Accord d'intéressement 2025-2028.pdf</v>
       </c>
       <c r="F18" s="12">
-        <v>45743</v>
+        <v>45744</v>
       </c>
       <c r="G18" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H18" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I18" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J18" s="13" t="s">
-        <v>8</v>
+        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C18)),TRUE,IF(AND(B18="LAN",I18=TRUE),TRUE,IF(AND(B18="NPS",I18=TRUE,K18=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H18:J18,TRUE),_xlpm.av,COUNTIF(H18:J18,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <v>1</v>
+      </c>
+      <c r="H18" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" s="13" t="b">
+        <v>1</v>
       </c>
       <c r="K18" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B18="NNF",B18="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M18)))</f>
         <v>-</v>
       </c>
-      <c r="L18" s="21" t="s">
-        <v>225</v>
+      <c r="L18" s="19" t="s">
+        <v>73</v>
       </c>
       <c r="M18" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="N18" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="O18" s="14" t="s">
-        <v>266</v>
-      </c>
-      <c r="P18" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="Q18" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="R18" s="21" t="s">
-        <v>49</v>
+      <c r="N18" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="O18" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="P18" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q18" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R18" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="S18" s="11" t="str" cm="1">
         <f t="array" ref="S18">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R18,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>tract-salaires-2025.pdf</v>
+        <v/>
       </c>
     </row>
     <row r="19" spans="1:19" ht="75" x14ac:dyDescent="0.25">
@@ -2789,74 +2936,79 @@
         <v>2025</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>188</v>
+        <v>13</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>173</v>
+        <v>254</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>39</v>
       </c>
       <c r="E19" s="11" t="str" cm="1">
         <f t="array" ref="E19">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D19,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Avenant Accord ARTT Lannion 20 03 2025.pdf</v>
+        <v>Procès verbal NAO (désaccord) 2025 (27 mars 2025).pdf</v>
       </c>
       <c r="F19" s="12">
-        <f>DATE(2025,3,20)</f>
-        <v>45736</v>
+        <v>45743</v>
       </c>
       <c r="G19" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C19)),TRUE,IF(AND(B19="LAN",I19=TRUE),TRUE,IF(AND(B19="NPS",I19=TRUE,K19=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H19:J19,TRUE),_xlpm.av,COUNTIF(H19:J19,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
-        <v>1</v>
-      </c>
-      <c r="H19" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I19" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="J19" s="13" t="b">
-        <v>0</v>
+      <c r="H19" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I19" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>8</v>
       </c>
       <c r="K19" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B19="NNF",B19="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M19)))</f>
         <v>-</v>
       </c>
-      <c r="L19" s="21" t="s">
-        <v>194</v>
-      </c>
-      <c r="M19" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="N19" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="O19" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="P19" s="14" t="s">
-        <v>281</v>
-      </c>
-      <c r="Q19" s="17"/>
-      <c r="R19" s="21"/>
-      <c r="S19" s="11"/>
-    </row>
-    <row r="20" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="L19" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="M19" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="N19" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="O19" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="P19" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q19" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="R19" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="S19" s="11" t="str" cm="1">
+        <f t="array" ref="S19">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R19,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v>tract-salaires-2025.pdf</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="10">
         <v>2025</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>174</v>
+        <v>146</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>159</v>
       </c>
       <c r="E20" s="11" t="str" cm="1">
         <f t="array" ref="E20">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D20,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Avenant Accord Horaire Variable Lannion 20 03 2025.pdf</v>
+        <v>Avenant Accord ARTT Lannion 20 03 2025.pdf</v>
       </c>
       <c r="F20" s="12">
         <f>DATE(2025,3,20)</f>
@@ -2876,47 +3028,48 @@
         <v>0</v>
       </c>
       <c r="K20" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B20="NNF",B20="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M20)))</f>
         <v>-</v>
       </c>
-      <c r="L20" s="21" t="s">
-        <v>195</v>
-      </c>
-      <c r="M20" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="N20" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="O20" s="14" t="s">
-        <v>253</v>
-      </c>
-      <c r="P20" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="Q20" s="17"/>
-      <c r="R20" s="21"/>
+      <c r="L20" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="N20" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="O20" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="P20" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="19"/>
       <c r="S20" s="11"/>
     </row>
-    <row r="21" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="10">
         <v>2025</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>13</v>
+        <v>174</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>115</v>
+        <v>147</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>160</v>
       </c>
       <c r="E21" s="11" t="str" cm="1">
         <f t="array" ref="E21">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D21,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Avenant accord télétravail avril 2022.pdf</v>
+        <v>Avenant Accord Horaire Variable Lannion 20 03 2025.pdf</v>
       </c>
       <c r="F21" s="12">
-        <v>45712</v>
+        <f>DATE(2025,3,20)</f>
+        <v>45736</v>
       </c>
       <c r="G21" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C21)),TRUE,IF(AND(B21="LAN",I21=TRUE),TRUE,IF(AND(B21="NPS",I21=TRUE,K21=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H21:J21,TRUE),_xlpm.av,COUNTIF(H21:J21,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -2929,64 +3082,57 @@
         <v>1</v>
       </c>
       <c r="J21" s="13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B21="NNF",B21="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M21)))</f>
         <v>-</v>
       </c>
-      <c r="L21" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="M21" s="12" t="s">
-        <v>207</v>
-      </c>
-      <c r="N21" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="O21" s="14" t="s">
-        <v>267</v>
-      </c>
-      <c r="P21" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="Q21" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="R21" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="S21" s="11" t="str" cm="1">
-        <f t="array" ref="S21">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R21,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>tract-avenant-TL-v2.pdf</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="L21" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="M21" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="N21" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="O21" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="P21" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q21" s="15"/>
+      <c r="R21" s="19"/>
+      <c r="S21" s="11"/>
+    </row>
+    <row r="22" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
         <v>2025</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="E22" s="15" t="str" cm="1">
+        <v>56</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" s="11" t="str" cm="1">
         <f t="array" ref="E22">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D22,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord 2025 NPS - aménagement temps de travail (20 janvier 2025).pdf</v>
-      </c>
-      <c r="F22" s="16">
-        <v>45677</v>
+        <v>Avenant accord télétravail avril 2022.pdf</v>
+      </c>
+      <c r="F22" s="12">
+        <v>45712</v>
       </c>
       <c r="G22" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C22)),TRUE,IF(AND(B22="LAN",I22=TRUE),TRUE,IF(AND(B22="NPS",I22=TRUE,K22=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H22:J22,TRUE),_xlpm.av,COUNTIF(H22:J22,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
         <v>1</v>
       </c>
       <c r="H22" s="13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" s="13" t="b">
         <v>1</v>
@@ -2994,53 +3140,55 @@
       <c r="J22" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K22" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L22" s="21" t="s">
-        <v>191</v>
-      </c>
-      <c r="M22" s="16" t="s">
-        <v>216</v>
-      </c>
-      <c r="N22" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="O22" s="10"/>
-      <c r="P22" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="Q22" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="R22" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="S22" s="15" t="str" cm="1">
+      <c r="K22" s="13" t="str">
+        <f>IF(OR(B22="NNF",B22="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M22)))</f>
+        <v>-</v>
+      </c>
+      <c r="L22" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="M22" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="N22" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="O22" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="P22" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="Q22" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="R22" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="S22" s="11" t="str" cm="1">
         <f t="array" ref="S22">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R22,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+        <v>tract-avenant-TL-v2.pdf</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="10">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="E23" s="11" t="str" cm="1">
+        <v>57</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="10" t="str" cm="1">
         <f t="array" ref="E23">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D23,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord don de jours 14 novembre 2024.pdf</v>
-      </c>
-      <c r="F23" s="12">
-        <v>45610</v>
+        <v>Accord 2025 NPS - aménagement temps de travail (20 janvier 2025).pdf</v>
+      </c>
+      <c r="F23" s="14">
+        <v>45677</v>
       </c>
       <c r="G23" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C23)),TRUE,IF(AND(B23="LAN",I23=TRUE),TRUE,IF(AND(B23="NPS",I23=TRUE,K23=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H23:J23,TRUE),_xlpm.av,COUNTIF(H23:J23,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -3055,37 +3203,35 @@
       <c r="J23" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K23" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="L23" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="M23" s="12" t="s">
+      <c r="K23" s="13" t="b">
+        <f>IF(OR(B23="NNF",B23="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M23)))</f>
+        <v>1</v>
+      </c>
+      <c r="L23" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="M23" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="N23" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="O23" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="P23" s="14" t="s">
-        <v>235</v>
-      </c>
-      <c r="Q23" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R23" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="S23" s="11" t="str" cm="1">
+      <c r="N23" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="Q23" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="R23" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="S23" s="10" t="str" cm="1">
         <f t="array" ref="S23">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R23,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="10">
         <v>2024</v>
       </c>
@@ -3093,53 +3239,54 @@
         <v>13</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>106</v>
+        <v>6</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>37</v>
       </c>
       <c r="E24" s="11" t="str" cm="1">
         <f t="array" ref="E24">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D24,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>PV désaccord Partage de la valeur VS.pdf</v>
+        <v>Accord don de jours 14 novembre 2024.pdf</v>
       </c>
       <c r="F24" s="12">
-        <v>45538</v>
+        <v>45610</v>
       </c>
       <c r="G24" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H24" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I24" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J24" s="13" t="s">
-        <v>8</v>
+        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C24)),TRUE,IF(AND(B24="LAN",I24=TRUE),TRUE,IF(AND(B24="NPS",I24=TRUE,K24=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H24:J24,TRUE),_xlpm.av,COUNTIF(H24:J24,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <v>1</v>
+      </c>
+      <c r="H24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J24" s="13" t="b">
+        <v>1</v>
       </c>
       <c r="K24" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B24="NNF",B24="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M24)))</f>
         <v>-</v>
       </c>
-      <c r="L24" s="21" t="s">
-        <v>226</v>
+      <c r="L24" s="19" t="s">
+        <v>75</v>
       </c>
       <c r="M24" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="N24" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="O24" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="P24" s="14" t="s">
-        <v>284</v>
-      </c>
-      <c r="Q24" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R24" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="N24" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="O24" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="P24" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q24" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R24" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S24" s="11" t="str" cm="1">
@@ -3147,67 +3294,66 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A25" s="10">
         <v>2024</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>38</v>
+        <v>255</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>97</v>
       </c>
       <c r="E25" s="11" t="str" cm="1">
         <f t="array" ref="E25">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D25,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord RCC 2024 (19 avril 2024).pdf</v>
+        <v>PV désaccord Partage de la valeur VS.pdf</v>
       </c>
       <c r="F25" s="12">
-        <v>45401</v>
+        <v>45538</v>
       </c>
       <c r="G25" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C25)),TRUE,IF(AND(B25="LAN",I25=TRUE),TRUE,IF(AND(B25="NPS",I25=TRUE,K25=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H25:J25,TRUE),_xlpm.av,COUNTIF(H25:J25,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
-        <v>1</v>
-      </c>
-      <c r="H25" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="J25" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="K25" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L25" s="21" t="s">
-        <v>81</v>
+        <v>0</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I25" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="K25" s="13" t="str">
+        <f>IF(OR(B25="NNF",B25="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M25)))</f>
+        <v>-</v>
+      </c>
+      <c r="L25" s="19" t="s">
+        <v>212</v>
       </c>
       <c r="M25" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="N25" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="O25" s="14" t="s">
-        <v>245</v>
-      </c>
-      <c r="P25" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="Q25" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="R25" s="21" t="s">
-        <v>51</v>
+        <v>83</v>
+      </c>
+      <c r="N25" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="O25" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="P25" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="Q25" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R25" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="S25" s="11" t="str" cm="1">
         <f t="array" ref="S25">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R25,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>tract_bilan_rcc24_v4.pdf</v>
+        <v/>
       </c>
     </row>
     <row r="26" spans="1:19" ht="60" x14ac:dyDescent="0.25">
@@ -3215,125 +3361,125 @@
         <v>2024</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>43</v>
+        <v>7</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>33</v>
       </c>
       <c r="E26" s="11" t="str" cm="1">
         <f t="array" ref="E26">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D26,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v>Accord RCC 2024 (19 avril 2024).pdf</v>
+      </c>
+      <c r="F26" s="12">
+        <v>45401</v>
+      </c>
+      <c r="G26" s="13" t="b">
+        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C26)),TRUE,IF(AND(B26="LAN",I26=TRUE),TRUE,IF(AND(B26="NPS",I26=TRUE,K26=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H26:J26,TRUE),_xlpm.av,COUNTIF(H26:J26,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <v>1</v>
+      </c>
+      <c r="H26" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26" s="13" t="b">
+        <f>IF(OR(B26="NNF",B26="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M26)))</f>
+        <v>1</v>
+      </c>
+      <c r="L26" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="M26" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="N26" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="O26" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="P26" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="Q26" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="R26" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="S26" s="11" t="str" cm="1">
+        <f t="array" ref="S26">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R26,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v>tract_bilan_rcc24_v4.pdf</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+      <c r="A27" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" s="11" t="str" cm="1">
+        <f t="array" ref="E27">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D27,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v>Avenant Procès-verbal de désaccord NAO 2024 (9 avril 2024).pdf</v>
       </c>
-      <c r="F26" s="12">
+      <c r="F27" s="12">
         <f>DATE(2024,4,9)</f>
         <v>45391</v>
       </c>
-      <c r="G26" s="13" t="b">
+      <c r="G27" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H26" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J26" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="K26" s="13" t="str">
-        <f t="shared" si="0"/>
+      <c r="H27" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I27" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J27" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="K27" s="13" t="str">
+        <f>IF(OR(B27="NNF",B27="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M27)))</f>
         <v>-</v>
       </c>
-      <c r="L26" s="21" t="s">
-        <v>227</v>
-      </c>
-      <c r="M26" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="N26" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="O26" s="14" t="s">
-        <v>269</v>
-      </c>
-      <c r="P26" s="14" t="s">
+      <c r="L27" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="M27" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="N27" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="O27" s="11" t="s">
         <v>285</v>
       </c>
-      <c r="Q26" s="17" t="s">
-        <v>155</v>
-      </c>
-      <c r="R26" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="S26" s="11" t="str" cm="1">
-        <f t="array" ref="S26">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R26,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>tract_retour_salaires_2024_v1.pdf</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="10">
-        <v>2024</v>
-      </c>
-      <c r="B27" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="E27" s="11" t="str" cm="1">
-        <f t="array" ref="E27">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D27,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord CGF.pdf</v>
-      </c>
-      <c r="F27" s="12">
-        <v>45366</v>
-      </c>
-      <c r="G27" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C27)),TRUE,IF(AND(B27="LAN",I27=TRUE),TRUE,IF(AND(B27="NPS",I27=TRUE,K27=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H27:J27,TRUE),_xlpm.av,COUNTIF(H27:J27,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
-        <v>1</v>
-      </c>
-      <c r="H27" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I27" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="J27" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="K27" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="L27" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="M27" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="N27" s="14" t="s">
+      <c r="P27" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="Q27" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="R27" s="19" t="s">
         <v>99</v>
-      </c>
-      <c r="O27" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="P27" s="14" t="s">
-        <v>236</v>
-      </c>
-      <c r="Q27" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R27" s="21" t="s">
-        <v>8</v>
       </c>
       <c r="S27" s="11" t="str" cm="1">
         <f t="array" ref="S27">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R27,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v/>
+        <v>tract_retour_salaires_2024_v1.pdf</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3341,21 +3487,20 @@
         <v>2024</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>188</v>
+        <v>13</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>170</v>
+        <v>20</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>34</v>
       </c>
       <c r="E28" s="11" t="str" cm="1">
         <f t="array" ref="E28">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D28,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord Etablissement NNF Lannion Mise en place accord cadre nouvelle CCN du 7 mars 2024.pdf</v>
+        <v>Accord CGF.pdf</v>
       </c>
       <c r="F28" s="12">
-        <f>DATE(2024,3,7)</f>
-        <v>45358</v>
+        <v>45366</v>
       </c>
       <c r="G28" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C28)),TRUE,IF(AND(B28="LAN",I28=TRUE),TRUE,IF(AND(B28="NPS",I28=TRUE,K28=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H28:J28,TRUE),_xlpm.av,COUNTIF(H28:J28,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -3371,48 +3516,55 @@
         <v>1</v>
       </c>
       <c r="K28" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B28="NNF",B28="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M28)))</f>
         <v>-</v>
       </c>
-      <c r="L28" s="21" t="s">
-        <v>198</v>
-      </c>
-      <c r="M28" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="N28" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="O28" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="P28" s="19" t="s">
+      <c r="L28" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="M28" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="N28" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="O28" s="11" t="s">
         <v>286</v>
       </c>
-      <c r="Q28" s="17"/>
-      <c r="R28" s="21"/>
-      <c r="S28" s="11"/>
+      <c r="P28" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q28" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R28" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="S28" s="11" t="str" cm="1">
+        <f t="array" ref="S28">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R28,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v/>
+      </c>
     </row>
     <row r="29" spans="1:19" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10">
         <v>2024</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>14</v>
+        <v>174</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>30</v>
+        <v>150</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>156</v>
       </c>
       <c r="E29" s="11" t="str" cm="1">
         <f t="array" ref="E29">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D29,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord cadre NPS nouvelle convention collective- 2024 signé.pdf</v>
+        <v>Accord Etablissement NNF Lannion Mise en place accord cadre nouvelle CCN du 7 mars 2024.pdf</v>
       </c>
       <c r="F29" s="12">
-        <f>DATE(2024,2,29)</f>
-        <v>45351</v>
+        <f>DATE(2024,3,7)</f>
+        <v>45358</v>
       </c>
       <c r="G29" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C29)),TRUE,IF(AND(B29="LAN",I29=TRUE),TRUE,IF(AND(B29="NPS",I29=TRUE,K29=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H29:J29,TRUE),_xlpm.av,COUNTIF(H29:J29,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -3427,113 +3579,114 @@
       <c r="J29" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K29" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L29" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="M29" s="12" t="s">
-        <v>218</v>
-      </c>
-      <c r="N29" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="O29" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="P29" s="19" t="s">
-        <v>286</v>
-      </c>
-      <c r="Q29" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="R29" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="S29" s="11" t="str" cm="1">
-        <f t="array" ref="S29">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R29,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>ncc cotation 3.pdf</v>
-      </c>
+      <c r="K29" s="13" t="str">
+        <f>IF(OR(B29="NNF",B29="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M29)))</f>
+        <v>-</v>
+      </c>
+      <c r="L29" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="M29" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="N29" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="O29" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="P29" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="19"/>
+      <c r="S29" s="11"/>
     </row>
     <row r="30" spans="1:19" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10">
         <v>2024</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>171</v>
+        <v>58</v>
+      </c>
+      <c r="D30" s="19" t="s">
+        <v>26</v>
       </c>
       <c r="E30" s="11" t="str" cm="1">
         <f t="array" ref="E30">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D30,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v>Accord cadre NPS nouvelle convention collective- 2024 signé.pdf</v>
+      </c>
+      <c r="F30" s="12">
+        <f>DATE(2024,2,29)</f>
+        <v>45351</v>
+      </c>
+      <c r="G30" s="13" t="b">
+        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C30)),TRUE,IF(AND(B30="LAN",I30=TRUE),TRUE,IF(AND(B30="NPS",I30=TRUE,K30=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H30:J30,TRUE),_xlpm.av,COUNTIF(H30:J30,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <v>1</v>
+      </c>
+      <c r="H30" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K30" s="13" t="b">
+        <f>IF(OR(B30="NNF",B30="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M30)))</f>
+        <v>1</v>
+      </c>
+      <c r="L30" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="M30" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="N30" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="O30" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="P30" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q30" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="R30" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="S30" s="11" t="str" cm="1">
+        <f t="array" ref="S30">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R30,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v>ncc cotation 3.pdf</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+      <c r="A31" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="E31" s="11" t="str" cm="1">
+        <f t="array" ref="E31">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D31,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v>Accord collectif mise en place CCN.pdf</v>
       </c>
-      <c r="F30" s="12">
+      <c r="F31" s="12">
         <f>DATE(2024,2,15)</f>
         <v>45337</v>
       </c>
-      <c r="G30" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C30)),TRUE,IF(AND(B30="LAN",I30=TRUE),TRUE,IF(AND(B30="NPS",I30=TRUE,K30=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H30:J30,TRUE),_xlpm.av,COUNTIF(H30:J30,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
-        <v>1</v>
-      </c>
-      <c r="H30" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I30" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="J30" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="K30" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="L30" s="21" t="s">
-        <v>199</v>
-      </c>
-      <c r="M30" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="N30" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="O30" s="14" t="s">
-        <v>256</v>
-      </c>
-      <c r="P30" s="19" t="s">
-        <v>286</v>
-      </c>
-      <c r="Q30" s="17"/>
-      <c r="R30" s="21"/>
-      <c r="S30" s="11"/>
-    </row>
-    <row r="31" spans="1:19" ht="45" x14ac:dyDescent="0.25">
-      <c r="A31" s="10">
-        <v>2023</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="E31" s="11" t="str" cm="1">
-        <f t="array" ref="E31">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D31,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord harmonisation taux variable cible salariés non sales du 19 décembre 2023.pdf</v>
-      </c>
-      <c r="F31" s="12">
-        <v>45279</v>
-      </c>
       <c r="G31" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C31)),TRUE,IF(AND(B31="LAN",I31=TRUE),TRUE,IF(AND(B31="NPS",I31=TRUE,K31=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H31:J31,TRUE),_xlpm.av,COUNTIF(H31:J31,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
         <v>1</v>
@@ -3548,54 +3701,47 @@
         <v>1</v>
       </c>
       <c r="K31" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B31="NNF",B31="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M31)))</f>
         <v>-</v>
       </c>
-      <c r="L31" s="21" t="s">
+      <c r="L31" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="M31" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="M31" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="N31" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O31" s="14" t="s">
-        <v>258</v>
-      </c>
-      <c r="P31" s="14" t="s">
-        <v>257</v>
-      </c>
-      <c r="Q31" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R31" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="S31" s="11" t="str" cm="1">
-        <f t="array" ref="S31">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R31,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v/>
-      </c>
+      <c r="N31" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="O31" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="P31" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q31" s="15"/>
+      <c r="R31" s="19"/>
+      <c r="S31" s="11"/>
     </row>
     <row r="32" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="10">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>31</v>
+        <v>59</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>98</v>
       </c>
       <c r="E32" s="11" t="str" cm="1">
         <f t="array" ref="E32">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D32,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord aménagement temps travail NPS 2024.pdf</v>
+        <v>Accord harmonisation taux variable cible salariés non sales du 19 décembre 2023.pdf</v>
       </c>
       <c r="F32" s="12">
-        <v>45268</v>
+        <v>45279</v>
       </c>
       <c r="G32" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C32)),TRUE,IF(AND(B32="LAN",I32=TRUE),TRUE,IF(AND(B32="NPS",I32=TRUE,K32=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H32:J32,TRUE),_xlpm.av,COUNTIF(H32:J32,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -3610,29 +3756,29 @@
       <c r="J32" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K32" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L32" s="21" t="s">
-        <v>68</v>
+      <c r="K32" s="13" t="str">
+        <f>IF(OR(B32="NNF",B32="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M32)))</f>
+        <v>-</v>
+      </c>
+      <c r="L32" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="N32" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="O32" s="14" t="s">
-        <v>237</v>
-      </c>
-      <c r="P32" s="19" t="s">
-        <v>287</v>
-      </c>
-      <c r="Q32" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R32" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="N32" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="O32" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="P32" s="21" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q32" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R32" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S32" s="11" t="str" cm="1">
@@ -3640,26 +3786,25 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="10">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>37</v>
+        <v>55</v>
+      </c>
+      <c r="D33" s="19" t="s">
+        <v>27</v>
       </c>
       <c r="E33" s="11" t="str" cm="1">
         <f t="array" ref="E33">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D33,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord de substitution non cadres - 30 novembre 2023.pdf</v>
+        <v>Accord aménagement temps travail NPS 2024.pdf</v>
       </c>
       <c r="F33" s="12">
-        <f>DATE(2023,11,30)</f>
-        <v>45260</v>
+        <v>45268</v>
       </c>
       <c r="G33" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C33)),TRUE,IF(AND(B33="LAN",I33=TRUE),TRUE,IF(AND(B33="NPS",I33=TRUE,K33=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H33:J33,TRUE),_xlpm.av,COUNTIF(H33:J33,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -3674,29 +3819,29 @@
       <c r="J33" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K33" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="L33" s="21" t="s">
-        <v>83</v>
+      <c r="K33" s="13" t="b">
+        <f>IF(OR(B33="NNF",B33="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M33)))</f>
+        <v>1</v>
+      </c>
+      <c r="L33" s="19" t="s">
+        <v>63</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="N33" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="O33" s="14" t="s">
-        <v>246</v>
-      </c>
-      <c r="P33" s="14" t="s">
-        <v>288</v>
-      </c>
-      <c r="Q33" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R33" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="N33" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="O33" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="P33" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="Q33" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R33" s="19" t="s">
         <v>8</v>
       </c>
       <c r="S33" s="11" t="str" cm="1">
@@ -3704,7 +3849,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="10">
         <v>2023</v>
       </c>
@@ -3712,17 +3857,18 @@
         <v>13</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="21" t="s">
-        <v>36</v>
+        <v>21</v>
+      </c>
+      <c r="D34" s="19" t="s">
+        <v>32</v>
       </c>
       <c r="E34" s="11" t="str" cm="1">
         <f t="array" ref="E34">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D34,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord RCC 2023.pdf</v>
+        <v>Accord de substitution non cadres - 30 novembre 2023.pdf</v>
       </c>
       <c r="F34" s="12">
-        <v>45111</v>
+        <f>DATE(2023,11,30)</f>
+        <v>45260</v>
       </c>
       <c r="G34" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C34)),TRUE,IF(AND(B34="LAN",I34=TRUE),TRUE,IF(AND(B34="NPS",I34=TRUE,K34=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H34:J34,TRUE),_xlpm.av,COUNTIF(H34:J34,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -3735,39 +3881,39 @@
         <v>1</v>
       </c>
       <c r="J34" s="13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B34="NNF",B34="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M34)))</f>
         <v>-</v>
       </c>
-      <c r="L34" s="21" t="s">
-        <v>84</v>
+      <c r="L34" s="19" t="s">
+        <v>78</v>
       </c>
       <c r="M34" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="N34" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="O34" s="14" t="s">
-        <v>247</v>
-      </c>
-      <c r="P34" s="14" t="s">
-        <v>289</v>
-      </c>
-      <c r="Q34" s="17" t="s">
-        <v>156</v>
-      </c>
-      <c r="R34" s="21" t="s">
-        <v>53</v>
+        <v>87</v>
+      </c>
+      <c r="N34" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="O34" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="P34" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q34" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R34" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="S34" s="11" t="str" cm="1">
         <f t="array" ref="S34">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R34,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Tract Volontariat RCC.pdf</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="10">
         <v>2023</v>
       </c>
@@ -3775,61 +3921,62 @@
         <v>13</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>41</v>
+        <v>5</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>31</v>
       </c>
       <c r="E35" s="11" t="str" cm="1">
         <f t="array" ref="E35">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D35,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>NAO 2023 - PV désaccord.pdf</v>
+        <v>Accord RCC 2023.pdf</v>
       </c>
       <c r="F35" s="12">
-        <v>45028</v>
+        <v>45111</v>
       </c>
       <c r="G35" s="13" t="b">
+        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C35)),TRUE,IF(AND(B35="LAN",I35=TRUE),TRUE,IF(AND(B35="NPS",I35=TRUE,K35=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H35:J35,TRUE),_xlpm.av,COUNTIF(H35:J35,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <v>1</v>
+      </c>
+      <c r="H35" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I35" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J35" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H35" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I35" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J35" s="13" t="s">
-        <v>8</v>
-      </c>
       <c r="K35" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B35="NNF",B35="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M35)))</f>
         <v>-</v>
       </c>
-      <c r="L35" s="21" t="s">
-        <v>228</v>
+      <c r="L35" s="19" t="s">
+        <v>79</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="N35" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="O35" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="P35" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q35" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="R35" s="21" t="s">
-        <v>54</v>
+        <v>206</v>
+      </c>
+      <c r="N35" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="O35" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="P35" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="Q35" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="R35" s="19" t="s">
+        <v>48</v>
       </c>
       <c r="S35" s="11" t="str" cm="1">
         <f t="array" ref="S35">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R35,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Tract brèves de printemps.pdf</v>
-      </c>
-    </row>
-    <row r="36" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+        <v>Tract Volontariat RCC.pdf</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A36" s="10">
         <v>2023</v>
       </c>
@@ -3837,87 +3984,86 @@
         <v>13</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D36" s="21" t="s">
-        <v>34</v>
+        <v>257</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="E36" s="11" t="str" cm="1">
         <f t="array" ref="E36">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D36,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord égalité professionnelle.pdf</v>
+        <v>NAO 2023 - PV désaccord.pdf</v>
       </c>
       <c r="F36" s="12">
         <v>45028</v>
       </c>
       <c r="G36" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C36)),TRUE,IF(AND(B36="LAN",I36=TRUE),TRUE,IF(AND(B36="NPS",I36=TRUE,K36=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H36:J36,TRUE),_xlpm.av,COUNTIF(H36:J36,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
-        <v>1</v>
-      </c>
-      <c r="H36" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="I36" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="J36" s="13" t="b">
-        <v>1</v>
+      <c r="H36" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I36" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J36" s="13" t="s">
+        <v>8</v>
       </c>
       <c r="K36" s="13" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(OR(B36="NNF",B36="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M36)))</f>
         <v>-</v>
       </c>
-      <c r="L36" s="21" t="s">
-        <v>94</v>
+      <c r="L36" s="19" t="s">
+        <v>214</v>
       </c>
       <c r="M36" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="N36" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="O36" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="P36" s="11" t="s">
         <v>221</v>
       </c>
-      <c r="N36" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="O36" s="14" t="s">
-        <v>259</v>
-      </c>
-      <c r="P36" s="14" t="s">
-        <v>290</v>
-      </c>
-      <c r="Q36" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="R36" s="21" t="s">
-        <v>54</v>
+      <c r="Q36" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="R36" s="19" t="s">
+        <v>49</v>
       </c>
       <c r="S36" s="11" t="str" cm="1">
         <f t="array" ref="S36">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R36,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v>Tract brèves de printemps.pdf</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A37" s="10">
         <v>2023</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="D37" s="21" t="s">
-        <v>189</v>
+        <v>4</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="E37" s="11" t="str" cm="1">
         <f t="array" ref="E37">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D37,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord aménagement temps travail NPS 2023.pdf</v>
+        <v>Accord égalité professionnelle.pdf</v>
       </c>
       <c r="F37" s="12">
-        <v>44967</v>
+        <v>45028</v>
       </c>
       <c r="G37" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C37)),TRUE,IF(AND(B37="LAN",I37=TRUE),TRUE,IF(AND(B37="NPS",I37=TRUE,K37=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H37:J37,TRUE),_xlpm.av,COUNTIF(H37:J37,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
         <v>1</v>
       </c>
       <c r="H37" s="13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I37" s="13" t="b">
         <v>1</v>
@@ -3925,34 +4071,34 @@
       <c r="J37" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K37" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L37" s="21" t="s">
-        <v>96</v>
+      <c r="K37" s="13" t="str">
+        <f>IF(OR(B37="NNF",B37="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M37)))</f>
+        <v>-</v>
+      </c>
+      <c r="L37" s="19" t="s">
+        <v>89</v>
       </c>
       <c r="M37" s="12" t="s">
-        <v>216</v>
-      </c>
-      <c r="N37" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="O37" s="14" t="s">
-        <v>239</v>
-      </c>
-      <c r="P37" s="19" t="s">
-        <v>291</v>
-      </c>
-      <c r="Q37" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R37" s="21" t="s">
-        <v>8</v>
+        <v>207</v>
+      </c>
+      <c r="N37" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="O37" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="P37" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="Q37" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="R37" s="19" t="s">
+        <v>49</v>
       </c>
       <c r="S37" s="11" t="str" cm="1">
         <f t="array" ref="S37">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R37,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v/>
+        <v>Tract brèves de printemps.pdf</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="30" x14ac:dyDescent="0.25">
@@ -3960,21 +4106,20 @@
         <v>2023</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>188</v>
+        <v>14</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="D38" s="21" t="s">
-        <v>177</v>
+        <v>90</v>
+      </c>
+      <c r="D38" s="19" t="s">
+        <v>175</v>
       </c>
       <c r="E38" s="11" t="str" cm="1">
         <f t="array" ref="E38">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D38,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord nombre délégués syndicaux Lannion 24 janvier 2023.pdf</v>
+        <v>Accord aménagement temps travail NPS 2023.pdf</v>
       </c>
       <c r="F38" s="12">
-        <f>DATE(2023,1,24)</f>
-        <v>44950</v>
+        <v>44967</v>
       </c>
       <c r="G38" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C38)),TRUE,IF(AND(B38="LAN",I38=TRUE),TRUE,IF(AND(B38="NPS",I38=TRUE,K38=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H38:J38,TRUE),_xlpm.av,COUNTIF(H38:J38,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -3989,47 +4134,54 @@
       <c r="J38" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K38" s="13" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
-      </c>
-      <c r="L38" s="21" t="s">
-        <v>201</v>
+      <c r="K38" s="13" t="b">
+        <f>IF(OR(B38="NNF",B38="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M38)))</f>
+        <v>1</v>
+      </c>
+      <c r="L38" s="19" t="s">
+        <v>91</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="N38" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="O38" s="14"/>
-      <c r="P38" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="Q38" s="17"/>
-      <c r="R38" s="21"/>
-      <c r="S38" s="11"/>
+        <v>202</v>
+      </c>
+      <c r="N38" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="O38" s="11"/>
+      <c r="P38" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="Q38" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R38" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="S38" s="11" t="str" cm="1">
+        <f t="array" ref="S38">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R38,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v/>
+      </c>
     </row>
     <row r="39" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="10">
         <v>2023</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>14</v>
+        <v>174</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="D39" s="21" t="s">
-        <v>172</v>
+        <v>153</v>
+      </c>
+      <c r="D39" s="19" t="s">
+        <v>163</v>
       </c>
       <c r="E39" s="11" t="str" cm="1">
         <f t="array" ref="E39">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D39,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
-        <v>Accord augmentation nombre délégués syndicaux NPS 2023.pdf</v>
+        <v>Accord nombre délégués syndicaux Lannion 24 janvier 2023.pdf</v>
       </c>
       <c r="F39" s="12">
-        <f>DATE(2023,1,23)</f>
-        <v>44949</v>
+        <f>DATE(2023,1,24)</f>
+        <v>44950</v>
       </c>
       <c r="G39" s="13" t="b">
         <f>IF(ISNUMBER(SEARCH("PV de désaccord",C39)),TRUE,IF(AND(B39="LAN",I39=TRUE),TRUE,IF(AND(B39="NPS",I39=TRUE,K39=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H39:J39,TRUE),_xlpm.av,COUNTIF(H39:J39,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
@@ -4044,27 +4196,25 @@
       <c r="J39" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="K39" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="L39" s="21" t="s">
-        <v>200</v>
+      <c r="K39" s="13" t="str">
+        <f>IF(OR(B39="NNF",B39="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M39)))</f>
+        <v>-</v>
+      </c>
+      <c r="L39" s="19" t="s">
+        <v>187</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>223</v>
-      </c>
-      <c r="N39" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="O39" s="14" t="s">
-        <v>241</v>
-      </c>
-      <c r="P39" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="Q39" s="17"/>
-      <c r="R39" s="21"/>
+        <v>208</v>
+      </c>
+      <c r="N39" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="O39" s="11"/>
+      <c r="P39" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="Q39" s="15"/>
+      <c r="R39" s="19"/>
       <c r="S39" s="11"/>
     </row>
     <row r="40" spans="1:19" ht="30" x14ac:dyDescent="0.25">
@@ -4072,186 +4222,247 @@
         <v>2023</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D40" s="21" t="s">
-        <v>35</v>
+        <v>152</v>
+      </c>
+      <c r="D40" s="19" t="s">
+        <v>158</v>
       </c>
       <c r="E40" s="11" t="str" cm="1">
         <f t="array" ref="E40">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D40,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+        <v>Accord augmentation nombre délégués syndicaux NPS 2023.pdf</v>
+      </c>
+      <c r="F40" s="12">
+        <f>DATE(2023,1,23)</f>
+        <v>44949</v>
+      </c>
+      <c r="G40" s="13" t="b">
+        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C40)),TRUE,IF(AND(B40="LAN",I40=TRUE),TRUE,IF(AND(B40="NPS",I40=TRUE,K40=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H40:J40,TRUE),_xlpm.av,COUNTIF(H40:J40,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <v>1</v>
+      </c>
+      <c r="H40" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J40" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K40" s="13" t="b">
+        <f>IF(OR(B40="NNF",B40="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M40)))</f>
+        <v>1</v>
+      </c>
+      <c r="L40" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="M40" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="N40" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="O40" s="11"/>
+      <c r="P40" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="Q40" s="15"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="11"/>
+    </row>
+    <row r="41" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="10">
+        <v>2023</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D41" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="E41" s="11" t="str" cm="1">
+        <f t="array" ref="E41">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D41,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v>Accord remboursement santé - 2023.pdf</v>
       </c>
-      <c r="F40" s="12">
+      <c r="F41" s="12">
         <f>DATE(2022,11,17)</f>
         <v>44882</v>
       </c>
-      <c r="G40" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C40)),TRUE,IF(AND(B40="LAN",I40=TRUE),TRUE,IF(AND(B40="NPS",I40=TRUE,K40=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H40:J40,TRUE),_xlpm.av,COUNTIF(H40:J40,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
-        <v>1</v>
-      </c>
-      <c r="H40" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I40" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="J40" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="K40" s="13" t="str">
-        <f t="shared" si="0"/>
+      <c r="G41" s="13" t="b">
+        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C41)),TRUE,IF(AND(B41="LAN",I41=TRUE),TRUE,IF(AND(B41="NPS",I41=TRUE,K41=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H41:J41,TRUE),_xlpm.av,COUNTIF(H41:J41,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <v>1</v>
+      </c>
+      <c r="H41" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I41" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J41" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K41" s="13" t="str">
+        <f>IF(OR(B41="NNF",B41="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M41)))</f>
         <v>-</v>
       </c>
-      <c r="L40" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="M40" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="N40" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="O40" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="P40" s="17" t="s">
-        <v>294</v>
-      </c>
-      <c r="Q40" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="R40" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="S40" s="11" t="str" cm="1">
-        <f t="array" ref="S40">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R40,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
+      <c r="L41" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="M41" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="N41" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="O41" s="11"/>
+      <c r="P41" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q41" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R41" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="S41" s="11" t="str" cm="1">
+        <f t="array" ref="S41">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R41,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S30" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U40">
-    <sortCondition descending="1" ref="F2:F40"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S41">
+    <sortCondition descending="1" ref="F2:F41"/>
   </sortState>
-  <conditionalFormatting sqref="Q3:R4 Q6:R8 Q28:R30 Q37:R37 Q32:R32 L2:R2 L33:R36 L9:R27 L32:O32 L31:R31 L37:O37 L28:O30 L6:O8 L5:R5 L3:O4 A2:K40 L38:R40">
-    <cfRule type="containsText" dxfId="21" priority="19" operator="containsText" text="vérifier">
+  <conditionalFormatting sqref="D2:D41">
+    <cfRule type="expression" dxfId="26" priority="45">
+      <formula>LEN(TRIM($D2))=0</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="25" priority="46" operator="containsText" text="CGT39">
+      <formula>NOT(ISERROR(SEARCH("CGT39",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="24" priority="47" operator="containsText" text="BDESE">
+      <formula>NOT(ISERROR(SEARCH("BDESE",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="23" priority="48" operator="containsText" text="HRLibrary">
+      <formula>NOT(ISERROR(SEARCH("HRLibrary",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="22" priority="49" operator="containsText" text="NokiaNetworksFrance">
+      <formula>NOT(ISERROR(SEARCH("NokiaNetworksFrance",D2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G35">
+    <cfRule type="expression" dxfId="21" priority="6">
+      <formula>G35=TRUE</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="20" priority="7">
+      <formula>G35=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:L30">
+    <cfRule type="expression" dxfId="19" priority="39">
+      <formula>G2=TRUE</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="40">
+      <formula>G2=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G31:L40">
+    <cfRule type="expression" dxfId="17" priority="8">
+      <formula>G31=TRUE</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="9">
+      <formula>G31=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L30">
+    <cfRule type="containsText" dxfId="15" priority="10" operator="containsText" text="vérifier">
+      <formula>NOT(ISERROR(SEARCH("vérifier",L30)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="14" priority="11" operator="containsText" text="préciser">
+      <formula>NOT(ISERROR(SEARCH("préciser",L30)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="12">
+      <formula>L30=TRUE</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="13">
+      <formula>L30=FALSE</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="11" priority="14" operator="containsText" text="retrouver">
+      <formula>NOT(ISERROR(SEARCH("retrouver",L30)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L28:O30 A2:K40 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 L2:R2 L3:O4 Q3:R4 L5:R5 L6:O8 Q6:R8 L9:R27 Q28:R30 Q32:R32 Q37:R37">
+    <cfRule type="containsText" dxfId="10" priority="24" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="21" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="9" priority="26" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:L30">
-    <cfRule type="expression" dxfId="19" priority="34">
-      <formula>G2=TRUE</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="35">
-      <formula>G2=FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q3:R4 Q6:R8 Q28:R30 Q37:R37 Q32:R32 L2:R2 L33:R36 L9:R27 L32:O32 L31:R31 L37:O37 L28:O30 L6:O8 L5:R5 L3:O4 A2:K40 L38:R40">
-    <cfRule type="containsText" dxfId="17" priority="39" operator="containsText" text="retrouver">
+  <conditionalFormatting sqref="L2:R2 A2:K40 L3:O4 L5:R5 L6:O8 L9:R27 L28:O30 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 Q3:R4 Q6:R8 Q28:R30 Q32:R32 Q37:R37">
+    <cfRule type="containsText" dxfId="8" priority="44" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D40">
-    <cfRule type="expression" dxfId="16" priority="40">
-      <formula>LEN(TRIM($D2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D40">
-    <cfRule type="containsText" dxfId="15" priority="41" operator="containsText" text="CGT39">
-      <formula>NOT(ISERROR(SEARCH("CGT39",D2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D40">
-    <cfRule type="containsText" dxfId="14" priority="42" operator="containsText" text="BDESE">
-      <formula>NOT(ISERROR(SEARCH("BDESE",D2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D40">
-    <cfRule type="containsText" dxfId="13" priority="43" operator="containsText" text="HRLibrary">
-      <formula>NOT(ISERROR(SEARCH("HRLibrary",D2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D40">
-    <cfRule type="containsText" dxfId="12" priority="44" operator="containsText" text="NokiaNetworksFrance">
-      <formula>NOT(ISERROR(SEARCH("NokiaNetworksFrance",D2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S40">
-    <cfRule type="containsText" dxfId="11" priority="13" operator="containsText" text="vérifier">
+  <conditionalFormatting sqref="S2:S41">
+    <cfRule type="containsText" dxfId="7" priority="18" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",S2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="14" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="6" priority="19" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",S2)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S40">
-    <cfRule type="containsText" dxfId="9" priority="15" operator="containsText" text="retrouver">
+    <cfRule type="containsText" dxfId="5" priority="20" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",S2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L30">
-    <cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="vérifier">
-      <formula>NOT(ISERROR(SEARCH("vérifier",L30)))</formula>
+  <conditionalFormatting sqref="G41:L41">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>G41=TRUE</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="6" operator="containsText" text="préciser">
-      <formula>NOT(ISERROR(SEARCH("préciser",L30)))</formula>
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>G41=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L30">
-    <cfRule type="expression" dxfId="6" priority="7">
-      <formula>L30=TRUE</formula>
+  <conditionalFormatting sqref="A41:R41">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="vérifier">
+      <formula>NOT(ISERROR(SEARCH("vérifier",A41)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="8">
-      <formula>L30=FALSE</formula>
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="préciser">
+      <formula>NOT(ISERROR(SEARCH("préciser",A41)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L30">
-    <cfRule type="containsText" dxfId="4" priority="9" operator="containsText" text="retrouver">
-      <formula>NOT(ISERROR(SEARCH("retrouver",L30)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G31:L40">
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>G31=TRUE</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
-      <formula>G31=FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G35">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>G35=TRUE</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>G35=FALSE</formula>
+  <conditionalFormatting sqref="A41:R41">
+    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="retrouver">
+      <formula>NOT(ISERROR(SEARCH("retrouver",A41)))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/2026%20protocole%20accord%20pr%C3%A9%C3%A9ctoral%20LANNION%20sign%C3%A9.pdf" xr:uid="{3DEBA908-9DCC-4C09-BA3C-6496E30376B0}"/>
     <hyperlink ref="D4" r:id="rId2" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/2026%20protocole%20accord%20pr%C3%A9%C3%A9lectoral%20sign%C3%A9.pdf" xr:uid="{6FEC8F61-3E2E-4A39-8E55-E655F5C98EDB}"/>
-    <hyperlink ref="D19" r:id="rId3" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Avenant%20Accord%20ARTT%20Lannion%2020%2003%202025.pdf?d=w41b9a9b002484645baa30299d81f4cd9&amp;csf=1&amp;web=1&amp;e=CBBk7K" xr:uid="{DDDE2E99-60A1-4C85-8E8A-A082CBA4D9C2}"/>
-    <hyperlink ref="D20" r:id="rId4" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Avenant%20Accord%20Horaire%20Variable%20Lannion%2020%2003%202025.pdf?d=w0708203cc5384f55a34496c60e3be8c7&amp;csf=1&amp;web=1&amp;e=HcRWx3" xr:uid="{AD1B6036-A480-400F-BCAB-0625286A7D7B}"/>
-    <hyperlink ref="D16" r:id="rId5" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Avenant%20frais%20de%20sant%C3%A9%20(9%20avril%202025).pdf?d=w3ab9353536cb49678646454b636bb215&amp;csf=1&amp;web=1&amp;e=HFDFvw" xr:uid="{DB05645A-2A6B-4BAF-9B88-01F85B98CAEE}"/>
+    <hyperlink ref="D20" r:id="rId3" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Avenant%20Accord%20ARTT%20Lannion%2020%2003%202025.pdf?d=w41b9a9b002484645baa30299d81f4cd9&amp;csf=1&amp;web=1&amp;e=CBBk7K" xr:uid="{DDDE2E99-60A1-4C85-8E8A-A082CBA4D9C2}"/>
+    <hyperlink ref="D21" r:id="rId4" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Avenant%20Accord%20Horaire%20Variable%20Lannion%2020%2003%202025.pdf?d=w0708203cc5384f55a34496c60e3be8c7&amp;csf=1&amp;web=1&amp;e=HcRWx3" xr:uid="{AD1B6036-A480-400F-BCAB-0625286A7D7B}"/>
+    <hyperlink ref="D17" r:id="rId5" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202025/Avenant%20frais%20de%20sant%C3%A9%20(9%20avril%202025).pdf?d=w3ab9353536cb49678646454b636bb215&amp;csf=1&amp;web=1&amp;e=HFDFvw" xr:uid="{DB05645A-2A6B-4BAF-9B88-01F85B98CAEE}"/>
     <hyperlink ref="D7" r:id="rId6" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/Accord%20Etablissement%20Prorogation%20des%20Mandats%20CSE-E%20Lannion.pdf?d=w43ddbf8e1efb416daa39a1aba4d23da2&amp;csf=1&amp;web=1&amp;e=Awv1cc" xr:uid="{CC014E71-AD12-4209-901B-BCFE08D7C6AF}"/>
-    <hyperlink ref="D30" r:id="rId7" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20collectif%20mise%20en%20place%20CCN.pdf" xr:uid="{65FF0241-4E2B-41E4-9A3A-2A553B2FC4F7}"/>
-    <hyperlink ref="D28" r:id="rId8" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20Etablissement%20NNF%20Lannion%20Mise%20en%20place%20accord%20cadre%20nouvelle%20CCN%20du%207%20mars%202024.pdf" xr:uid="{EAC5F39B-7E23-4F8C-A956-D1A23AD59037}"/>
-    <hyperlink ref="D39" r:id="rId9" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20augmentation%20nombre%20d%C3%A9l%C3%A9gu%C3%A9s%20syndicaux%20NPS%202023.pdf" xr:uid="{7AAC36A3-6D0B-4195-B33D-3DBFC7518375}"/>
-    <hyperlink ref="D38" r:id="rId10" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20nombre%20d%C3%A9l%C3%A9gu%C3%A9s%20syndicaux%20Lannion%2024%20janvier%202023.pdf?d=w7f99dd8365c6418eb22acb63a8ac44b2&amp;csf=1&amp;web=1&amp;e=nOfza5" xr:uid="{F1E97C35-916D-446B-B83F-9D8E27B48A78}"/>
-    <hyperlink ref="D37" r:id="rId11" xr:uid="{3CA5F90A-37A0-47B4-A593-00FA1CC25A3A}"/>
-    <hyperlink ref="D22" r:id="rId12" xr:uid="{953BDEB9-68F0-45C1-BEE6-C570830B2425}"/>
-    <hyperlink ref="L19" r:id="rId13" xr:uid="{9553D652-6925-4255-8B66-56354E6BF3B1}"/>
-    <hyperlink ref="L20" r:id="rId14" xr:uid="{0B7E48E3-FDDE-4B3A-A09C-DE4FFC8D13AF}"/>
-    <hyperlink ref="D24" r:id="rId15" xr:uid="{35FF18B8-C1F8-4ACB-AC18-C9B1639EB410}"/>
+    <hyperlink ref="D31" r:id="rId7" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20collectif%20mise%20en%20place%20CCN.pdf" xr:uid="{65FF0241-4E2B-41E4-9A3A-2A553B2FC4F7}"/>
+    <hyperlink ref="D29" r:id="rId8" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20Etablissement%20NNF%20Lannion%20Mise%20en%20place%20accord%20cadre%20nouvelle%20CCN%20du%207%20mars%202024.pdf" xr:uid="{EAC5F39B-7E23-4F8C-A956-D1A23AD59037}"/>
+    <hyperlink ref="D40" r:id="rId9" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20augmentation%20nombre%20d%C3%A9l%C3%A9gu%C3%A9s%20syndicaux%20NPS%202023.pdf" xr:uid="{7AAC36A3-6D0B-4195-B33D-3DBFC7518375}"/>
+    <hyperlink ref="D39" r:id="rId10" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20nombre%20d%C3%A9l%C3%A9gu%C3%A9s%20syndicaux%20Lannion%2024%20janvier%202023.pdf?d=w7f99dd8365c6418eb22acb63a8ac44b2&amp;csf=1&amp;web=1&amp;e=nOfza5" xr:uid="{F1E97C35-916D-446B-B83F-9D8E27B48A78}"/>
+    <hyperlink ref="D38" r:id="rId11" xr:uid="{3CA5F90A-37A0-47B4-A593-00FA1CC25A3A}"/>
+    <hyperlink ref="D23" r:id="rId12" xr:uid="{953BDEB9-68F0-45C1-BEE6-C570830B2425}"/>
+    <hyperlink ref="L20" r:id="rId13" xr:uid="{9553D652-6925-4255-8B66-56354E6BF3B1}"/>
+    <hyperlink ref="L21" r:id="rId14" xr:uid="{0B7E48E3-FDDE-4B3A-A09C-DE4FFC8D13AF}"/>
+    <hyperlink ref="D25" r:id="rId15" xr:uid="{35FF18B8-C1F8-4ACB-AC18-C9B1639EB410}"/>
     <hyperlink ref="L14" r:id="rId16" xr:uid="{BA92569F-D437-4A24-9A1C-EDBCBE27EBE4}"/>
+    <hyperlink ref="D16" r:id="rId17" display="https://nokia.sharepoint.com/sites/BDESENNF-CSE-C/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FBDESENNF%2DCSE%2DC%2FShared%20Documents%2F05a%2E%20CSE%2DC%2FCSE%2DC%202025%2F03%2DCSE%2DC%20extraordinaire%209%20avril%202025%2Faccord%20collectif%20relatif%20aux%20%C3%A9volutions%20du%20r%C3%A9gime%20AUXAD%20%2DVF%2Epdf" xr:uid="{22171004-D3FC-446C-9F9D-36C128A50C34}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId17"/>
+  <pageSetup orientation="portrait" r:id="rId18"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
   </headerFooter>
@@ -4260,9 +4471,188 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{527E1360-D0DF-42E4-8989-040F8979EEC8}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="12.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="32.42578125" customWidth="1"/>
+    <col min="2" max="2" width="118.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>293</v>
+      </c>
+      <c r="B1" s="22"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="24" t="s">
+        <v>300</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="22" t="s">
+        <v>307</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>310</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="22" t="s">
+        <v>314</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="22" t="s">
+        <v>314</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="22" t="s">
+        <v>325</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>326</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
@@ -4280,23 +4670,61 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
-    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
-    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
-      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
-      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -4567,59 +4995,21 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
+    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
+    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
+      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
+      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4631,17 +5021,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
-    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4661,18 +5056,13 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
+    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Sync disagreement signatories and the latest summaries and CGT positions from Excel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2503" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{903CCD27-DD50-4B71-AADE-96FB1B9F3E41}"/>
+  <xr:revisionPtr revIDLastSave="2548" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAAB38F6-12CA-4BA0-8EE1-6D90B4F40EBD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="328">
   <si>
     <t>Accord ou négociation</t>
   </si>
@@ -244,9 +244,6 @@
     <t>Harmonisation du taux de bonus</t>
   </si>
   <si>
-    <t>Avenant CSE</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Avenant%20RCC%202025.pdf</t>
   </si>
   <si>
@@ -388,9 +385,6 @@
     <t>195 suppressions de postes. Volontariat ouvert à tous les salariés du 01/09 au 30/09/2026.</t>
   </si>
   <si>
-    <t>La restauration sort des ASC des CSE d'établissement et passe à la Direction ; budget ASC et commission restauration revus.</t>
-  </si>
-  <si>
     <t>Politique handicap NNF : rôles des acteurs (managers, santé au travail, service social, Mission handicap). Cotisations retraite prises en charge à 100 % en temps partiel choisi.</t>
   </si>
   <si>
@@ -715,9 +709,6 @@
     <t>Retraite par capitalisation contre la répartition, perte de cotisations sociales ; préférence pour un 13e mois cotisé.</t>
   </si>
   <si>
-    <t>Pas d'engagement d'embauche ni de remplacement des départs, garanties insuffisantes sur les activités en France.</t>
-  </si>
-  <si>
     <t>Soutien à l'élargissement, demande d'un seuil préservant les congés des aidants.</t>
   </si>
   <si>
@@ -742,9 +733,6 @@
     <t>CFTC</t>
   </si>
   <si>
-    <t>Décision unilatérale : prime négociée seulement si bénéfice net fiscal &gt; 15 % du CA France.</t>
-  </si>
-  <si>
     <t>Aucune solution pour les salariés aux compteurs d'heures positifs (remise à zéro = heures non payées, non cotisées).</t>
   </si>
   <si>
@@ -778,12 +766,6 @@
     <t>Modalités électorales (vote électronique, calendrier, collèges, nombre de sièges, répartition H/F, effectifs de référence) jugées conformes.</t>
   </si>
   <si>
-    <t>Contre : pas de budget spécifique ni d'heures de délégation pour les référents ; mission handicap réduite à 1 personne nommée par la Direction ; élus non associés aux décisions (commission paritaire supprimée, simple bilan annuel) ; maintien dans l'emploi en recul par rapport à 2021 ; jours d'absence sur demande avec justificatif. Demandes CGT non retenues : rôle formalisé de la CSSCT, secrétaire CSSCT dans la mission handicap, lien AGEFIPH, mesures contre le plafond de verre (bac+2/3). Pour : sans accord, seulement le minimum légal (ni aide de 200 €, ni jours de congé) ; CSSCT associée aux études de poste ; TPC prolongeable au-delà de 5 ans avec retraite et prévoyance à 100 %.</t>
-  </si>
-  <si>
-    <t>Pour : souplesse pour les salariés, jour supplémentaire à Lannion. Contre : monétisation des congés (repos transformé en argent), 5e semaine exclue mais logique banalisée.</t>
-  </si>
-  <si>
     <t>Mêmes bases que l'accord précédent, qui a donné de bons niveaux d'intéressement ; part de la masse salariale dans la formule portée de 3 % à 4 %, en contrepartie de la signature AUXAD.</t>
   </si>
   <si>
@@ -793,9 +775,6 @@
     <t>Pour : 1 jour de repos supplémentaire pour tous, aligné sur Paris-Saclay. Contre : prime de crèche (80 €/mois jusqu'aux 4 ans de l'enfant) fermée aux nouveaux entrants au 01/01/2026, congés familiaux supprimés ; risque de préparer un établissement unique NPS + Lannion.</t>
   </si>
   <si>
-    <t>Versement conditionné à un bénéfice net fiscal &gt; 15 % du CA, inatteignable vu le déficit comptable de NNF (héritage Alcatel-Lucent, R&amp;D sous-facturée à la maison mère) : aucune prime possible en pratique. Revendication : du salaire fixe plutôt que des primes.</t>
-  </si>
-  <si>
     <t>Augmentations bien inférieures à l'inflation, d'où une baisse des salaires réels ; pas de mesure générale ; NAO suivie d'une RCC (357 suppressions, dont 1/3 en R&amp;D).</t>
   </si>
   <si>
@@ -805,24 +784,12 @@
     <t>Correction demandée par la CGT obtenue (« salaire fixe » au lieu de « salaire de base »).</t>
   </si>
   <si>
-    <t>Pour : volontariat, mesures individuelles correctes, éviter un PSE à moyen terme. Points d'alerte : pressions au volontariat, affaiblissement des équipes, absence de garanties sur les activités en France, lien RCC / absence d'augmentation.</t>
-  </si>
-  <si>
     <t>Pour : quelques actions (formation des managers, candidature féminine recherchée pour les postes de management). Contre : pas d'enveloppe budgétaire spécifique, aucune amélioration proposée par la CGT retenue.</t>
   </si>
   <si>
     <t>Accord sur le régime de remboursement des frais de santé, sans recul identifié.</t>
   </si>
   <si>
-    <t>RCC devenue un outil récurrent (2e de 2026) ; suppressions de postes sans embauche ni garantie d'emploi (la CGT demandait une garantie jusqu'au 31/12/2027) ; volontariat élargi à tous les salariés, d'où une pression sur les non-volontaires ; OS exclues de la commission de validation ; ni stratégie industrielle ni pérennité des sites traitées.</t>
-  </si>
-  <si>
-    <t>Pour : mesures individuelles de départ jugées correctes et alternative à un PSE. Contre (bilan a posteriori) : délocalisations, perte de savoir-faire, charge de travail, RPS, externalisations.</t>
-  </si>
-  <si>
-    <t>Jusqu'à 421 suppressions de postes non justifiées par la charge de travail ; RCC à répétition ; ni garantie d'emploi ni embauche ; externalisations et perte de compétences ; critères de substitution ; pression au volontariat.</t>
-  </si>
-  <si>
     <t>GEPP</t>
   </si>
   <si>
@@ -838,9 +805,6 @@
     <t>NAO 2023</t>
   </si>
   <si>
-    <t>Pas d'accord : la Direction refuse tout plan d'embauche (« 1 départ = 1 embauche »). Mesures unilatérales pour 3 ans : forums métiers et mobilité internationale ; prime de mobilité inter-région de 10 000 € brut, déménagement jusqu'à 5 000 € HT et 1 jour de congé ; priorité au recrutement interne et aux jeunes diplômés ; TPC seniors prolongeable au-delà de 5 ans avec retraite et prévoyance à 100 % ; entretiens de début et de cours de mandat pour les élus. Suivi annuel en CSE-C.</t>
-  </si>
-  <si>
     <t>accord collectif relatif aux évolutions du régime AUXAD -VF.pdf</t>
   </si>
   <si>
@@ -850,24 +814,9 @@
     <t>Évolutions du régime AUXAD</t>
   </si>
   <si>
-    <t>Le règlement de la retraite supplémentaire AUXAD (anciens hauts salaires Alcatel, rémunération &gt; 8 PASS, environ 250 ayants droit) devient accord collectif dans sa version du 01/10/2021 : valeur du point figée à celle du 30/09/2021, sans revalorisation. Objectif : sécuriser le régime face aux recours de retraités (jurisprudence Cass. 19/01/2022). Engagement de négocier avant toute évolution. Durée indéterminée. Contreparties : mutuelle prise en charge à 60 % (au lieu de 50 %) et intéressement à 4 % de la masse salariale (au lieu de 3 %).</t>
-  </si>
-  <si>
-    <t>Pour : gain substantiel pour les salariés (mutuelle 60/40 à vie, intéressement 4 % MS), autofinancé par la fin de l'indexation d'une retraite chapeau de très hauts salaires. Contre : contreparties qui ne font qu'aligner sur les pratiques du marché ; aucune contrepartie salariale ; gain principal sur l'intéressement, limité à 4 ans.</t>
-  </si>
-  <si>
-    <t>La Direction (M. Cudot) refuse toute modification du texte et exige une réponse avant le 10/07/2026 12h. Signature électronique le 13/07/2026 (2e procédure, les pages n'ayant pas été paraphées au 1er essai). Avis favorable de toutes les OS sur le projet. Risque relevé en interne qu'un échange de mails remplace une vraie négociation.</t>
-  </si>
-  <si>
-    <t>Favorable au transfert de la restauration à la Direction.</t>
-  </si>
-  <si>
     <t>Accord technique, aucun enjeu de fond défavorable.</t>
   </si>
   <si>
-    <t>Pas d'augmentation générale. Augmentations individuelles 2,15 % des TTC (promotions incluses ; GPP et Unexplained Pay Gap maintenus) au 01/04/2026. Primes de transport au 01/04/2026 : zone 1 9 €, zone 2 12 €, zone 3 60 €. Forfait vélo porté de 400 € à 500 €/an (60 €/mois, 0,36 €/km). Astreinte 265 € (+6 %), ticket astreinte 22 € ; travail de nuit 140 € (&lt;5 h) / 280 € (&gt;5 h), nuit de WE 160 € / 320 €, samedi 320 €. Expire le 30/04/2027.</t>
-  </si>
-  <si>
     <t>Avenant du 15/01/2026 ; nouvelle demande de validation à l'administration le 21/01/2026.</t>
   </si>
   <si>
@@ -895,9 +844,6 @@
     <t>Vote AG extra 24/03/2025 (24 votants dont 3 procurations).</t>
   </si>
   <si>
-    <t>Pas d'accord majoritaire. Mesures unilatérales : budget d'augmentations individuelles de 2 % des TTC, pas d'augmentation générale ; GPP et Unexplained Pay Gap maintenus. Primes de transport +5 % au 01/07/2025 : zone 1 7,98 €, zone 2 10,93 €, zone 3 57,45 €. Expire le 30/06/2026.</t>
-  </si>
-  <si>
     <t>Réunions des 17/12/2024, 27/01, 03/03 et 12/03/2025 ; PV de désaccord du 27/03/2025 ; accord séparé signé par la seule CFDT (20/03/2025), non majoritaire. Action : blocage des calendriers (~600 salariés).</t>
   </si>
   <si>
@@ -913,9 +859,6 @@
     <t>Compteur &gt; 900 jours (à vérifier).</t>
   </si>
   <si>
-    <t>Nouvelle réduction d'effectifs : 231 suppressions de postes en 2024 (non retrouvé dans le PDF, qui indique 347 maximum).</t>
-  </si>
-  <si>
     <t>Pas d'accord. Enveloppe unilatérale relevée de 0,66 point à 1,81 % des TTC, uniquement en augmentations individuelles ; GPP et Unexplained Pay Gap maintenus. Primes de transport et IK voiture inchangées. Expire le 30/06/2025.</t>
   </si>
   <si>
@@ -946,9 +889,6 @@
     <t>Règles de remplissage de la feuille accords</t>
   </si>
   <si>
-    <t>Pour : enveloppe portée de 1,85 % à 2,15 % (+0,30 point), hausse des primes de transport (vélo 400 → 500 €, indemnité kilométrique) et des primes d'intervention (forfait 265 € au lieu de 250 €). Contre : aucune augmentation générale ; revendications CGT refusées (rattrapage de 5 % depuis 2021 + 4 %) ; individualisation ; les femmes restent moins augmentées, écart plus fort à Lannion.</t>
-  </si>
-  <si>
     <t>Confirmation par courriel. Débat/vote des syndiqués avant le 26/01/2026 ; R1 le 19/01, réunion finale le 23/01/2026 ; accord fait à Massy le 27/01/2026. Négociation accélérée en 7 jours, peu de lecture des statistiques ; +0,30 point conditionné à la signature (« chantage à la signature ») ; mobilisation jugée difficile.</t>
   </si>
   <si>
@@ -1043,6 +983,69 @@
   </si>
   <si>
     <t>URL absolue et encodée. Le nom du fichier tract doit correspondre à la fin de l'URL tract.</t>
+  </si>
+  <si>
+    <t>Cette RCC n'est que la phase 3 de la RCC 2026 n°1 : le constat d'un outil devenu récurrent était déjà posé, en toute logique c'est toujours non. Suppressions de postes sans embauche ni garantie d'emploi (garantie demandée jusqu'au 31/12/2027) ; volontariat élargi à tous les salariés, d'où une pression sur les non-volontaires ; OS exclues de la commission de validation ; ni stratégie industrielle ni pérennité des sites.</t>
+  </si>
+  <si>
+    <t>Pour : gains concrets au-delà du minimum légal, surtout le temps partiel choisi (TPC) prolongeable au-delà de 5 ans avec retraite et prévoyance prises en charge à 100 % ; aide de 200 € et jours de congé dédiés ; CSSCT associée aux études de poste. Contre : pas de moyens dédiés aux référents, élus écartés du pilotage (commission paritaire supprimée).</t>
+  </si>
+  <si>
+    <t>Avenant CSE Restauration</t>
+  </si>
+  <si>
+    <t>PV de désaccord valide unilatéralement ; accord séparé signé par la seule CFDT, non majoritaire ; aucune signature de la CFE-CGC ni de la CGT.</t>
+  </si>
+  <si>
+    <t>Pas d'accord majoritaire. Mesures unilatérales : budget d'augmentations individuelles de 2 % des TTC, sans augmentation générale ; GPP et Unexplained Pay Gap maintenus ; primes de transport revalorisées de 5 %.</t>
+  </si>
+  <si>
+    <t>Trop c'est trop : la CGT a fait preuve de flexibilité et de pragmatisme en accompagnant les deux RCC précédentes (2023, 2024), un dispositif qui échange une signature contre la garantie du volontariat. La Direction semble désormais vouloir se faire un PSE en 4 fois, sans frais : ce sera sans nous. Jusqu'à 421 suppressions de postes non justifiées par la charge de travail ; ni garantie d'emploi ni embauche ; externalisations et perte de compétences ; pression au volontariat.</t>
+  </si>
+  <si>
+    <t>Accord technique : il formalise une délégation de la restauration à la Direction déjà en place, sans enjeu de fond défavorable.</t>
+  </si>
+  <si>
+    <t>Nokia n'a jamais eu l'intention d'aboutir à un accord : la négociation obligatoire a été menée pour la forme. Pas d'engagement d'embauche ni de remplacement des départs, garanties insuffisantes sur les activités en France.</t>
+  </si>
+  <si>
+    <t>Choix pragmatique tranché assez facilement pour la première édition de ce dispositif, qui garantissait le volontariat en échange de la signature d'un accord majoritaire. Solide sur ses convictions, la CGT sait aussi faire preuve de pragmatisme quand le contexte le permet : volontariat, mesures individuelles correctes, éviter un PSE à moyen terme. Points d'alerte : pressions au volontariat, affaiblissement des équipes, absence de garanties sur les activités en France, lien RCC / absence d'augmentation.</t>
+  </si>
+  <si>
+    <t>Deuxième RCC acceptée car la pyramide des âges et le contexte le permettaient encore (départs volontaires majoritairement en fin de carrière) ; mesures individuelles de départ jugées correctes, alternative à un PSE. Bilan a posteriori critique : délocalisations, perte de savoir-faire, charge de travail, RPS, externalisations.</t>
+  </si>
+  <si>
+    <t>Après de longs débats internes, la CGT vote finalement la signature. Nouvelle réduction d'effectifs : 231 suppressions de postes en 2024 (non retrouvé dans le PDF, qui indique 347 maximum).</t>
+  </si>
+  <si>
+    <t>Contre : la CGT se méfie quand la Direction propose d'« augmenter » les salariés avec leur propre argent (monétisation des congés, repos transformé en argent) ; 5e semaine exclue mais logique banalisée. Points positifs reconnus : souplesse pour les salariés, jour supplémentaire à Lannion.</t>
+  </si>
+  <si>
+    <t>Pas d'augmentation générale. Augmentations individuelles de 2,15 % au 01/04/2026. Primes de transport, forfait vélo (500 €/an) et primes d'astreinte et de nuit revalorisées.</t>
+  </si>
+  <si>
+    <t>Compromis assumé : loin de nos revendications, mais 2,15 % reste bon à prendre et les salariés en ont besoin. La CGT sait faire des compromis. Limites : aucune augmentation générale, individualisation.</t>
+  </si>
+  <si>
+    <t>Négociation obligatoire tous les 3 ans, sans obligation d'aboutir. Pas d'accord : la Direction refuse tout plan d'embauche. Mesures unilatérales pour 3 ans : aides à la mobilité, priorité au recrutement interne, TPC seniors prolongeable avec retraite et prévoyance à 100 %.</t>
+  </si>
+  <si>
+    <t>La retraite supplémentaire AUXAD (anciens hauts salaires Alcatel, environ 250 ayants droit) devient un accord collectif, avec une valeur du point figée sans revalorisation. Contreparties : mutuelle prise en charge à 60 % et intéressement porté à 4 % de la masse salariale.</t>
+  </si>
+  <si>
+    <t>Signature négociée en échange de deux gains pour tous les salariés : frais de santé mieux pris en charge (60 %) et meilleur intéressement (4 %). Limites : aucune contrepartie salariale, gain sur l'intéressement limité à 4 ans.</t>
+  </si>
+  <si>
+    <t>Négociation obligatoire, sans obligation d'aboutir. Pas d'accord : prime versée seulement si le bénéfice net fiscal dépasse 15 % du CA France.</t>
+  </si>
+  <si>
+    <t>Comme pour la GEPP, négociation menée pour la forme : Nokia n'a jamais cherché d'accord. Seuil inatteignable vu le déficit de NNF, donc aucune prime en pratique. Revendication : du salaire fixe plutôt que des primes.</t>
+  </si>
+  <si>
+    <t>Suite à la baisse des dépenses de restauration depuis le COVID (confinements, télétravail), qui a réduit la contribution ASC versée aux CSE-E, Nokia verse une indemnité transactionnelle de 145 000 € (protocole via le CSE-C, répartie au prorata des effectifs NPS/Lannion) pour solder les années antérieures à 2026. L'avenant sort la restauration des ASC et encadre la délégation à la Direction, qui assume tous les coûts et rend compte de la facturation et du budget à une commission restauration par CSE-E.</t>
+  </si>
+  <si>
+    <t>La Direction (M. Cudot) refuse toute modification du texte et exige une réponse avant le 10/07/2026 12h. Signature électronique le 13/07/2026 (2e procédure, les pages n'ayant pas été paraphées au 1er essai). Avis favorable de toutes les OS sur le projet. Risque relevé en interne qu'un échange de mails remplace une vraie négociation. Estimations du manque à percevoir (réunion Direction/DSC/Syndex, 01/10/2025) : ≈ 800 k€ pour Syndex (Paris-Saclay seul, base masse salariale N) contre ≈ 200 k€ pour la Direction (deux sites, base N-1). CSE-E Paris-Saclay du 24/03/2026 : mandat au CSE-C pour transiger à 145 000 € (unanimité, 25 voix).</t>
   </si>
 </sst>
 </file>
@@ -1208,7 +1211,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1267,12 +1270,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1287,7 +1284,29 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="29">
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1331,30 +1350,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1531,6 +1526,30 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1846,16 +1865,16 @@
         <v>0</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>10</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>1</v>
@@ -1867,7 +1886,7 @@
         <v>3</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L1" s="9" t="s">
         <v>50</v>
@@ -1876,25 +1895,25 @@
         <v>24</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P1" s="8" t="s">
         <v>11</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="10">
         <v>2026</v>
       </c>
@@ -1915,7 +1934,7 @@
         <v>46219</v>
       </c>
       <c r="G2" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C2)),TRUE,IF(AND(B2="LAN",I2=TRUE),TRUE,IF(AND(B2="NPS",I2=TRUE,K2=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H2:J2,TRUE),_xlpm.av,COUNTIF(H2:J2,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" ref="G2:G13" si="0">IF(ISNUMBER(SEARCH("PV de désaccord",C2)),TRUE,IF(AND(B2="LAN",I2=TRUE),TRUE,IF(AND(B2="NPS",I2=TRUE,K2=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H2:J2,TRUE),_xlpm.av,COUNTIF(H2:J2,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
         <v>1</v>
       </c>
       <c r="H2" s="13" t="b">
@@ -1928,26 +1947,26 @@
         <v>1</v>
       </c>
       <c r="K2" s="13" t="str">
-        <f>IF(OR(B2="NNF",B2="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M2)))</f>
+        <f t="shared" ref="K2:K15" si="1">IF(OR(B2="NNF",B2="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M2)))</f>
         <v>-</v>
       </c>
       <c r="L2" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>250</v>
+        <v>307</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="R2" s="19" t="s">
         <v>41</v>
@@ -1962,13 +1981,13 @@
         <v>2026</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E3" s="11" t="str" cm="1">
         <f t="array" ref="E3">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D3,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -1979,7 +1998,7 @@
         <v>46218</v>
       </c>
       <c r="G3" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C3)),TRUE,IF(AND(B3="LAN",I3=TRUE),TRUE,IF(AND(B3="NPS",I3=TRUE,K3=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H3:J3,TRUE),_xlpm.av,COUNTIF(H3:J3,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H3" s="13" t="b">
@@ -1992,21 +2011,21 @@
         <v>1</v>
       </c>
       <c r="K3" s="13" t="str">
-        <f>IF(OR(B3="NNF",B3="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M3)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="O3" s="11"/>
       <c r="P3" s="17" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="Q3" s="15"/>
       <c r="R3" s="19"/>
@@ -2020,10 +2039,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E4" s="11" t="str" cm="1">
         <f t="array" ref="E4">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D4,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2034,7 +2053,7 @@
         <v>46218</v>
       </c>
       <c r="G4" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C4)),TRUE,IF(AND(B4="LAN",I4=TRUE),TRUE,IF(AND(B4="NPS",I4=TRUE,K4=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H4:J4,TRUE),_xlpm.av,COUNTIF(H4:J4,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H4" s="13" t="b">
@@ -2047,27 +2066,27 @@
         <v>1</v>
       </c>
       <c r="K4" s="13" t="b">
-        <f>IF(OR(B4="NNF",B4="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M4)))</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="O4" s="11"/>
-      <c r="P4" s="21" t="s">
-        <v>237</v>
+      <c r="P4" s="17" t="s">
+        <v>233</v>
       </c>
       <c r="Q4" s="15"/>
       <c r="R4" s="19"/>
       <c r="S4" s="11"/>
     </row>
-    <row r="5" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="165" x14ac:dyDescent="0.25">
       <c r="A5" s="10">
         <v>2026</v>
       </c>
@@ -2075,10 +2094,10 @@
         <v>13</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>60</v>
+        <v>309</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E5" s="11" t="str" cm="1">
         <f t="array" ref="E5">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D5,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2088,7 +2107,7 @@
         <v>46212</v>
       </c>
       <c r="G5" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C5)),TRUE,IF(AND(B5="LAN",I5=TRUE),TRUE,IF(AND(B5="NPS",I5=TRUE,K5=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H5:J5,TRUE),_xlpm.av,COUNTIF(H5:J5,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H5" s="13" t="b">
@@ -2101,23 +2120,23 @@
         <v>1</v>
       </c>
       <c r="K5" s="13" t="str">
-        <f>IF(OR(B5="NNF",B5="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M5)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>108</v>
+        <v>326</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>264</v>
+        <v>327</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>265</v>
+        <v>313</v>
       </c>
       <c r="Q5" s="15" t="s">
         <v>8</v>
@@ -2130,7 +2149,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="180" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="10">
         <v>2026</v>
       </c>
@@ -2141,7 +2160,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E6" s="10" t="str" cm="1">
         <f t="array" ref="E6">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D6,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2151,7 +2170,7 @@
         <v>46192</v>
       </c>
       <c r="G6" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C6)),TRUE,IF(AND(B6="LAN",I6=TRUE),TRUE,IF(AND(B6="NPS",I6=TRUE,K6=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H6:J6,TRUE),_xlpm.av,COUNTIF(H6:J6,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H6" s="13" t="b">
@@ -2164,23 +2183,23 @@
         <v>1</v>
       </c>
       <c r="K6" s="13" t="str">
-        <f>IF(OR(B6="NNF",B6="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M6)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L6" s="19" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="P6" s="17" t="s">
-        <v>238</v>
+        <v>308</v>
       </c>
       <c r="Q6" s="16" t="s">
         <v>8</v>
@@ -2198,13 +2217,13 @@
         <v>2026</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E7" s="11" t="str" cm="1">
         <f t="array" ref="E7">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D7,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2215,7 +2234,7 @@
         <v>46160</v>
       </c>
       <c r="G7" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C7)),TRUE,IF(AND(B7="LAN",I7=TRUE),TRUE,IF(AND(B7="NPS",I7=TRUE,K7=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H7:J7,TRUE),_xlpm.av,COUNTIF(H7:J7,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H7" s="13" t="b">
@@ -2228,27 +2247,27 @@
         <v>1</v>
       </c>
       <c r="K7" s="13" t="str">
-        <f>IF(OR(B7="NNF",B7="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M7)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O7" s="11"/>
       <c r="P7" s="17" t="s">
-        <v>266</v>
+        <v>250</v>
       </c>
       <c r="Q7" s="15"/>
       <c r="R7" s="19"/>
       <c r="S7" s="11"/>
     </row>
-    <row r="8" spans="1:19" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="10">
         <v>2026</v>
       </c>
@@ -2259,7 +2278,7 @@
         <v>54</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E8" s="11" t="str" cm="1">
         <f t="array" ref="E8">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D8,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2270,7 +2289,7 @@
         <v>46046</v>
       </c>
       <c r="G8" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C8)),TRUE,IF(AND(B8="LAN",I8=TRUE),TRUE,IF(AND(B8="NPS",I8=TRUE,K8=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H8:J8,TRUE),_xlpm.av,COUNTIF(H8:J8,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H8" s="13" t="b">
@@ -2283,23 +2302,23 @@
         <v>1</v>
       </c>
       <c r="K8" s="13" t="str">
-        <f>IF(OR(B8="NNF",B8="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M8)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>267</v>
+        <v>319</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>295</v>
-      </c>
-      <c r="P8" s="21" t="s">
-        <v>294</v>
+        <v>275</v>
+      </c>
+      <c r="P8" s="17" t="s">
+        <v>320</v>
       </c>
       <c r="Q8" s="15" t="s">
         <v>8</v>
@@ -2323,7 +2342,7 @@
         <v>53</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E9" s="11" t="str" cm="1">
         <f t="array" ref="E9">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D9,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2333,7 +2352,7 @@
         <v>46037</v>
       </c>
       <c r="G9" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C9)),TRUE,IF(AND(B9="LAN",I9=TRUE),TRUE,IF(AND(B9="NPS",I9=TRUE,K9=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H9:J9,TRUE),_xlpm.av,COUNTIF(H9:J9,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H9" s="13" t="b">
@@ -2346,23 +2365,23 @@
         <v>1</v>
       </c>
       <c r="K9" s="13" t="str">
-        <f>IF(OR(B9="NNF",B9="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M9)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L9" s="19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="Q9" s="15" t="s">
         <v>8</v>
@@ -2396,7 +2415,7 @@
         <v>46010</v>
       </c>
       <c r="G10" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C10)),TRUE,IF(AND(B10="LAN",I10=TRUE),TRUE,IF(AND(B10="NPS",I10=TRUE,K10=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H10:J10,TRUE),_xlpm.av,COUNTIF(H10:J10,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H10" s="13" t="b">
@@ -2409,21 +2428,21 @@
         <v>1</v>
       </c>
       <c r="K10" s="13" t="b">
-        <f>IF(OR(B10="NNF",B10="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M10)))</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="L10" s="19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="Q10" s="16" t="s">
         <v>8</v>
@@ -2436,7 +2455,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="135" x14ac:dyDescent="0.25">
       <c r="A11" s="10">
         <v>2026</v>
       </c>
@@ -2447,7 +2466,7 @@
         <v>51</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E11" s="11" t="str" cm="1">
         <f t="array" ref="E11">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D11,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2457,7 +2476,7 @@
         <v>46010</v>
       </c>
       <c r="G11" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C11)),TRUE,IF(AND(B11="LAN",I11=TRUE),TRUE,IF(AND(B11="NPS",I11=TRUE,K11=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H11:J11,TRUE),_xlpm.av,COUNTIF(H11:J11,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H11" s="13" t="b">
@@ -2470,26 +2489,26 @@
         <v>1</v>
       </c>
       <c r="K11" s="13" t="str">
-        <f>IF(OR(B11="NNF",B11="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M11)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L11" s="19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="N11" s="11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="O11" s="11" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="P11" s="11" t="s">
-        <v>252</v>
+        <v>312</v>
       </c>
       <c r="Q11" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="R11" s="19" t="s">
         <v>42</v>
@@ -2510,7 +2529,7 @@
         <v>17</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E12" s="11" t="str" cm="1">
         <f t="array" ref="E12">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D12,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2520,7 +2539,7 @@
         <v>46007</v>
       </c>
       <c r="G12" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C12)),TRUE,IF(AND(B12="LAN",I12=TRUE),TRUE,IF(AND(B12="NPS",I12=TRUE,K12=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H12:J12,TRUE),_xlpm.av,COUNTIF(H12:J12,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H12" s="13" t="b">
@@ -2533,23 +2552,23 @@
         <v>1</v>
       </c>
       <c r="K12" s="13" t="str">
-        <f>IF(OR(B12="NNF",B12="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M12)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="N12" s="11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="O12" s="11" t="s">
-        <v>272</v>
+        <v>255</v>
       </c>
       <c r="P12" s="11" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="Q12" s="15" t="s">
         <v>8</v>
@@ -2573,7 +2592,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E13" s="11" t="str" cm="1">
         <f t="array" ref="E13">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D13,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2583,7 +2602,7 @@
         <v>46007</v>
       </c>
       <c r="G13" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C13)),TRUE,IF(AND(B13="LAN",I13=TRUE),TRUE,IF(AND(B13="NPS",I13=TRUE,K13=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H13:J13,TRUE),_xlpm.av,COUNTIF(H13:J13,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H13" s="13" t="b">
@@ -2596,23 +2615,23 @@
         <v>1</v>
       </c>
       <c r="K13" s="13" t="str">
-        <f>IF(OR(B13="NNF",B13="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M13)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L13" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="N13" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>273</v>
+        <v>256</v>
       </c>
       <c r="P13" s="11" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="Q13" s="15" t="s">
         <v>8</v>
@@ -2625,7 +2644,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="120" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
         <v>2025</v>
       </c>
@@ -2633,7 +2652,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="D14" s="19" t="s">
         <v>28</v>
@@ -2648,36 +2667,36 @@
       <c r="G14" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I14" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J14" s="13" t="s">
-        <v>8</v>
+      <c r="H14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" s="13" t="b">
+        <v>0</v>
       </c>
       <c r="K14" s="13" t="str">
-        <f>IF(OR(B14="NNF",B14="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M14)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L14" s="19" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="M14" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>258</v>
+        <v>321</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>274</v>
+        <v>257</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>217</v>
+        <v>314</v>
       </c>
       <c r="Q14" s="15" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R14" s="19" t="s">
         <v>43</v>
@@ -2687,7 +2706,7 @@
         <v>tract_rcc_2026.pdf</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="10">
         <v>2025</v>
       </c>
@@ -2722,23 +2741,23 @@
         <v>1</v>
       </c>
       <c r="K15" s="13" t="str">
-        <f>IF(OR(B15="NNF",B15="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M15)))</f>
+        <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="L15" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M15" s="12" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="P15" s="11" t="s">
-        <v>239</v>
+        <v>318</v>
       </c>
       <c r="Q15" s="15" t="s">
         <v>8</v>
@@ -2751,7 +2770,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="150" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="10">
         <v>2025</v>
       </c>
@@ -2759,13 +2778,13 @@
         <v>13</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="F16" s="12">
         <f>DATE(2025,4,9)</f>
@@ -2787,19 +2806,19 @@
         <v>8</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="M16" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>262</v>
+        <v>322</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="P16" s="15" t="s">
-        <v>263</v>
+        <v>323</v>
       </c>
       <c r="Q16" s="15" t="s">
         <v>8</v>
@@ -2819,10 +2838,10 @@
         <v>13</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E17" s="11" t="str" cm="1">
         <f t="array" ref="E17">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D17,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2846,23 +2865,23 @@
         <v>1</v>
       </c>
       <c r="K17" s="13" t="str">
-        <f>IF(OR(B17="NNF",B17="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M17)))</f>
+        <f t="shared" ref="K17:K41" si="2">IF(OR(B17="NNF",B17="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M17)))</f>
         <v>-</v>
       </c>
       <c r="L17" s="19" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>275</v>
+        <v>258</v>
       </c>
       <c r="Q17" s="15"/>
       <c r="R17" s="19"/>
@@ -2879,7 +2898,7 @@
         <v>19</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E18" s="11" t="str" cm="1">
         <f t="array" ref="E18">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D18,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2902,23 +2921,23 @@
         <v>1</v>
       </c>
       <c r="K18" s="13" t="str">
-        <f>IF(OR(B18="NNF",B18="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M18)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L18" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="O18" s="11" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="P18" s="11" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="Q18" s="15" t="s">
         <v>8</v>
@@ -2931,7 +2950,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="10">
         <v>2025</v>
       </c>
@@ -2939,7 +2958,7 @@
         <v>13</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="D19" s="19" t="s">
         <v>39</v>
@@ -2954,36 +2973,36 @@
       <c r="G19" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H19" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I19" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J19" s="13" t="s">
-        <v>8</v>
+      <c r="H19" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" s="13" t="b">
+        <v>0</v>
       </c>
       <c r="K19" s="13" t="str">
-        <f>IF(OR(B19="NNF",B19="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M19)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L19" s="19" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>83</v>
+        <v>310</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>277</v>
+        <v>311</v>
       </c>
       <c r="O19" s="11" t="s">
-        <v>278</v>
+        <v>260</v>
       </c>
       <c r="P19" s="11" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="Q19" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="R19" s="19" t="s">
         <v>44</v>
@@ -2998,13 +3017,13 @@
         <v>2025</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E20" s="11" t="str" cm="1">
         <f t="array" ref="E20">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D20,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3028,23 +3047,23 @@
         <v>0</v>
       </c>
       <c r="K20" s="13" t="str">
-        <f>IF(OR(B20="NNF",B20="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M20)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L20" s="19" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N20" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="O20" s="11" t="s">
-        <v>279</v>
+        <v>261</v>
       </c>
       <c r="P20" s="11" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="Q20" s="15"/>
       <c r="R20" s="19"/>
@@ -3055,13 +3074,13 @@
         <v>2025</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E21" s="11" t="str" cm="1">
         <f t="array" ref="E21">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D21,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3085,23 +3104,23 @@
         <v>0</v>
       </c>
       <c r="K21" s="13" t="str">
-        <f>IF(OR(B21="NNF",B21="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M21)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L21" s="19" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="N21" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="P21" s="11" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="Q21" s="15"/>
       <c r="R21" s="19"/>
@@ -3118,7 +3137,7 @@
         <v>56</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E22" s="11" t="str" cm="1">
         <f t="array" ref="E22">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D22,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3141,26 +3160,26 @@
         <v>1</v>
       </c>
       <c r="K22" s="13" t="str">
-        <f>IF(OR(B22="NNF",B22="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M22)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L22" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M22" s="12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="N22" s="11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="O22" s="11" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="P22" s="11" t="s">
-        <v>281</v>
+        <v>263</v>
       </c>
       <c r="Q22" s="15" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="R22" s="19" t="s">
         <v>45</v>
@@ -3180,8 +3199,8 @@
       <c r="C23" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D23" s="20" t="s">
-        <v>96</v>
+      <c r="D23" s="19" t="s">
+        <v>95</v>
       </c>
       <c r="E23" s="10" t="str" cm="1">
         <f t="array" ref="E23">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D23,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3204,21 +3223,21 @@
         <v>1</v>
       </c>
       <c r="K23" s="13" t="b">
-        <f>IF(OR(B23="NNF",B23="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M23)))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L23" s="19" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="O23" s="10"/>
       <c r="P23" s="10" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="Q23" s="16" t="s">
         <v>8</v>
@@ -3265,23 +3284,23 @@
         <v>1</v>
       </c>
       <c r="K24" s="13" t="str">
-        <f>IF(OR(B24="NNF",B24="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M24)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L24" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M24" s="12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="N24" s="11" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>282</v>
+        <v>264</v>
       </c>
       <c r="P24" s="11" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="Q24" s="15" t="s">
         <v>8</v>
@@ -3302,10 +3321,10 @@
         <v>13</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>255</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>97</v>
+        <v>244</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>96</v>
       </c>
       <c r="E25" s="11" t="str" cm="1">
         <f t="array" ref="E25">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D25,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3317,33 +3336,33 @@
       <c r="G25" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H25" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I25" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J25" s="13" t="s">
-        <v>8</v>
+      <c r="H25" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" s="13" t="b">
+        <v>0</v>
       </c>
       <c r="K25" s="13" t="str">
-        <f>IF(OR(B25="NNF",B25="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M25)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L25" s="19" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="M25" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>226</v>
+        <v>324</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="P25" s="11" t="s">
-        <v>243</v>
+        <v>325</v>
       </c>
       <c r="Q25" s="15" t="s">
         <v>8</v>
@@ -3356,7 +3375,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A26" s="10">
         <v>2024</v>
       </c>
@@ -3390,26 +3409,26 @@
         <v>1</v>
       </c>
       <c r="K26" s="13" t="b">
-        <f>IF(OR(B26="NNF",B26="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M26)))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L26" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N26" s="11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>283</v>
+        <v>317</v>
       </c>
       <c r="P26" s="11" t="s">
-        <v>251</v>
+        <v>316</v>
       </c>
       <c r="Q26" s="15" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="R26" s="19" t="s">
         <v>46</v>
@@ -3427,7 +3446,7 @@
         <v>13</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="D27" s="19" t="s">
         <v>38</v>
@@ -3443,39 +3462,39 @@
       <c r="G27" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H27" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J27" s="13" t="s">
-        <v>8</v>
+      <c r="H27" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J27" s="13" t="b">
+        <v>0</v>
       </c>
       <c r="K27" s="13" t="str">
-        <f>IF(OR(B27="NNF",B27="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M27)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L27" s="19" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="M27" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N27" s="11" t="s">
-        <v>284</v>
+        <v>265</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>285</v>
+        <v>266</v>
       </c>
       <c r="P27" s="11" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="Q27" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="R27" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="S27" s="11" t="str" cm="1">
         <f t="array" ref="S27">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R27,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3503,7 +3522,7 @@
         <v>45366</v>
       </c>
       <c r="G28" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C28)),TRUE,IF(AND(B28="LAN",I28=TRUE),TRUE,IF(AND(B28="NPS",I28=TRUE,K28=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H28:J28,TRUE),_xlpm.av,COUNTIF(H28:J28,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" ref="G28:G35" si="3">IF(ISNUMBER(SEARCH("PV de désaccord",C28)),TRUE,IF(AND(B28="LAN",I28=TRUE),TRUE,IF(AND(B28="NPS",I28=TRUE,K28=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H28:J28,TRUE),_xlpm.av,COUNTIF(H28:J28,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
         <v>1</v>
       </c>
       <c r="H28" s="13" t="b">
@@ -3516,23 +3535,23 @@
         <v>1</v>
       </c>
       <c r="K28" s="13" t="str">
-        <f>IF(OR(B28="NNF",B28="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M28)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L28" s="19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M28" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N28" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>286</v>
-      </c>
-      <c r="P28" s="21" t="s">
-        <v>219</v>
+        <v>267</v>
+      </c>
+      <c r="P28" s="17" t="s">
+        <v>216</v>
       </c>
       <c r="Q28" s="15" t="s">
         <v>8</v>
@@ -3550,13 +3569,13 @@
         <v>2024</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E29" s="11" t="str" cm="1">
         <f t="array" ref="E29">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D29,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3567,7 +3586,7 @@
         <v>45358</v>
       </c>
       <c r="G29" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C29)),TRUE,IF(AND(B29="LAN",I29=TRUE),TRUE,IF(AND(B29="NPS",I29=TRUE,K29=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H29:J29,TRUE),_xlpm.av,COUNTIF(H29:J29,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H29" s="13" t="b">
@@ -3580,23 +3599,23 @@
         <v>1</v>
       </c>
       <c r="K29" s="13" t="str">
-        <f>IF(OR(B29="NNF",B29="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M29)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L29" s="19" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="M29" s="11" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="P29" s="17" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="Q29" s="15"/>
       <c r="R29" s="19"/>
@@ -3624,7 +3643,7 @@
         <v>45351</v>
       </c>
       <c r="G30" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C30)),TRUE,IF(AND(B30="LAN",I30=TRUE),TRUE,IF(AND(B30="NPS",I30=TRUE,K30=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H30:J30,TRUE),_xlpm.av,COUNTIF(H30:J30,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H30" s="13" t="b">
@@ -3637,26 +3656,26 @@
         <v>1</v>
       </c>
       <c r="K30" s="13" t="b">
-        <f>IF(OR(B30="NNF",B30="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M30)))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L30" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M30" s="12" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="N30" s="11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="P30" s="17" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="Q30" s="15" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="R30" s="19" t="s">
         <v>47</v>
@@ -3674,10 +3693,10 @@
         <v>13</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E31" s="11" t="str" cm="1">
         <f t="array" ref="E31">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D31,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3688,7 +3707,7 @@
         <v>45337</v>
       </c>
       <c r="G31" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C31)),TRUE,IF(AND(B31="LAN",I31=TRUE),TRUE,IF(AND(B31="NPS",I31=TRUE,K31=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H31:J31,TRUE),_xlpm.av,COUNTIF(H31:J31,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H31" s="13" t="b">
@@ -3701,23 +3720,23 @@
         <v>1</v>
       </c>
       <c r="K31" s="13" t="str">
-        <f>IF(OR(B31="NNF",B31="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M31)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L31" s="19" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M31" s="11" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="P31" s="11" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="Q31" s="15"/>
       <c r="R31" s="19"/>
@@ -3734,7 +3753,7 @@
         <v>59</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E32" s="11" t="str" cm="1">
         <f t="array" ref="E32">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D32,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3744,7 +3763,7 @@
         <v>45279</v>
       </c>
       <c r="G32" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C32)),TRUE,IF(AND(B32="LAN",I32=TRUE),TRUE,IF(AND(B32="NPS",I32=TRUE,K32=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H32:J32,TRUE),_xlpm.av,COUNTIF(H32:J32,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H32" s="13" t="b">
@@ -3757,23 +3776,23 @@
         <v>1</v>
       </c>
       <c r="K32" s="13" t="str">
-        <f>IF(OR(B32="NNF",B32="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M32)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N32" s="11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>297</v>
-      </c>
-      <c r="P32" s="21" t="s">
-        <v>296</v>
+        <v>277</v>
+      </c>
+      <c r="P32" s="17" t="s">
+        <v>276</v>
       </c>
       <c r="Q32" s="15" t="s">
         <v>8</v>
@@ -3807,7 +3826,7 @@
         <v>45268</v>
       </c>
       <c r="G33" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C33)),TRUE,IF(AND(B33="LAN",I33=TRUE),TRUE,IF(AND(B33="NPS",I33=TRUE,K33=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H33:J33,TRUE),_xlpm.av,COUNTIF(H33:J33,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H33" s="13" t="b">
@@ -3820,23 +3839,23 @@
         <v>1</v>
       </c>
       <c r="K33" s="13" t="b">
-        <f>IF(OR(B33="NNF",B33="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M33)))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L33" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="N33" s="11" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="P33" s="11" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="Q33" s="15" t="s">
         <v>8</v>
@@ -3871,7 +3890,7 @@
         <v>45260</v>
       </c>
       <c r="G34" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C34)),TRUE,IF(AND(B34="LAN",I34=TRUE),TRUE,IF(AND(B34="NPS",I34=TRUE,K34=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H34:J34,TRUE),_xlpm.av,COUNTIF(H34:J34,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H34" s="13" t="b">
@@ -3884,23 +3903,23 @@
         <v>1</v>
       </c>
       <c r="K34" s="13" t="str">
-        <f>IF(OR(B34="NNF",B34="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M34)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L34" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M34" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N34" s="11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="P34" s="11" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="Q34" s="15" t="s">
         <v>8</v>
@@ -3913,7 +3932,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" ht="135" x14ac:dyDescent="0.25">
       <c r="A35" s="10">
         <v>2023</v>
       </c>
@@ -3934,7 +3953,7 @@
         <v>45111</v>
       </c>
       <c r="G35" s="13" t="b">
-        <f>IF(ISNUMBER(SEARCH("PV de désaccord",C35)),TRUE,IF(AND(B35="LAN",I35=TRUE),TRUE,IF(AND(B35="NPS",I35=TRUE,K35=TRUE),TRUE,_xlfn.LET(_xlpm.ok,COUNTIF(H35:J35,TRUE),_xlpm.av,COUNTIF(H35:J35,"À vérifier"),IF(_xlpm.ok&gt;=2,TRUE,IF(_xlpm.ok+_xlpm.av&gt;=2,"À vérifier",FALSE))))))</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="H35" s="13" t="b">
@@ -3947,26 +3966,26 @@
         <v>0</v>
       </c>
       <c r="K35" s="13" t="str">
-        <f>IF(OR(B35="NNF",B35="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M35)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L35" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="N35" s="11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>287</v>
+        <v>268</v>
       </c>
       <c r="P35" s="11" t="s">
-        <v>247</v>
+        <v>315</v>
       </c>
       <c r="Q35" s="15" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="R35" s="19" t="s">
         <v>48</v>
@@ -3984,7 +4003,7 @@
         <v>13</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="D36" s="19" t="s">
         <v>36</v>
@@ -3999,36 +4018,36 @@
       <c r="G36" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H36" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I36" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J36" s="13" t="s">
-        <v>8</v>
+      <c r="H36" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J36" s="13" t="b">
+        <v>0</v>
       </c>
       <c r="K36" s="13" t="str">
-        <f>IF(OR(B36="NNF",B36="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M36)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L36" s="19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M36" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N36" s="11" t="s">
-        <v>288</v>
+        <v>269</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>289</v>
+        <v>270</v>
       </c>
       <c r="P36" s="11" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="Q36" s="15" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="R36" s="19" t="s">
         <v>49</v>
@@ -4072,26 +4091,26 @@
         <v>1</v>
       </c>
       <c r="K37" s="13" t="str">
-        <f>IF(OR(B37="NNF",B37="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M37)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L37" s="19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M37" s="12" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="N37" s="11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="P37" s="21" t="s">
-        <v>248</v>
+        <v>271</v>
+      </c>
+      <c r="P37" s="17" t="s">
+        <v>240</v>
       </c>
       <c r="Q37" s="15" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="R37" s="19" t="s">
         <v>49</v>
@@ -4109,10 +4128,10 @@
         <v>14</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E38" s="11" t="str" cm="1">
         <f t="array" ref="E38">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D38,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4135,21 +4154,21 @@
         <v>1</v>
       </c>
       <c r="K38" s="13" t="b">
-        <f>IF(OR(B38="NNF",B38="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M38)))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L38" s="19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="N38" s="11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="O38" s="11"/>
       <c r="P38" s="11" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="Q38" s="15" t="s">
         <v>8</v>
@@ -4167,13 +4186,13 @@
         <v>2023</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E39" s="11" t="str" cm="1">
         <f t="array" ref="E39">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D39,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4197,21 +4216,21 @@
         <v>1</v>
       </c>
       <c r="K39" s="13" t="str">
-        <f>IF(OR(B39="NNF",B39="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M39)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L39" s="19" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="O39" s="11"/>
       <c r="P39" s="11" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="Q39" s="15"/>
       <c r="R39" s="19"/>
@@ -4225,10 +4244,10 @@
         <v>14</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E40" s="11" t="str" cm="1">
         <f t="array" ref="E40">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D40,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4252,21 +4271,21 @@
         <v>1</v>
       </c>
       <c r="K40" s="13" t="b">
-        <f>IF(OR(B40="NNF",B40="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M40)))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L40" s="19" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="M40" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="O40" s="11"/>
       <c r="P40" s="15" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="Q40" s="15"/>
       <c r="R40" s="19"/>
@@ -4307,21 +4326,21 @@
         <v>1</v>
       </c>
       <c r="K41" s="13" t="str">
-        <f>IF(OR(B41="NNF",B41="LAN"),"-",ISNUMBER(SEARCH("de la CFTC",M41)))</f>
+        <f t="shared" si="2"/>
         <v>-</v>
       </c>
       <c r="L41" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M41" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="O41" s="11"/>
       <c r="P41" s="15" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="Q41" s="15" t="s">
         <v>8</v>
@@ -4339,107 +4358,113 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S41">
     <sortCondition descending="1" ref="F2:F41"/>
   </sortState>
+  <conditionalFormatting sqref="A41:R41">
+    <cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="vérifier">
+      <formula>NOT(ISERROR(SEARCH("vérifier",A41)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="27" priority="6" operator="containsText" text="préciser">
+      <formula>NOT(ISERROR(SEARCH("préciser",A41)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="26" priority="7" operator="containsText" text="retrouver">
+      <formula>NOT(ISERROR(SEARCH("retrouver",A41)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D2:D41">
-    <cfRule type="expression" dxfId="26" priority="45">
+    <cfRule type="expression" dxfId="25" priority="47">
       <formula>LEN(TRIM($D2))=0</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="46" operator="containsText" text="CGT39">
+    <cfRule type="containsText" dxfId="24" priority="48" operator="containsText" text="CGT39">
       <formula>NOT(ISERROR(SEARCH("CGT39",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="47" operator="containsText" text="BDESE">
+    <cfRule type="containsText" dxfId="23" priority="49" operator="containsText" text="BDESE">
       <formula>NOT(ISERROR(SEARCH("BDESE",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="48" operator="containsText" text="HRLibrary">
+    <cfRule type="containsText" dxfId="22" priority="50" operator="containsText" text="HRLibrary">
       <formula>NOT(ISERROR(SEARCH("HRLibrary",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="49" operator="containsText" text="NokiaNetworksFrance">
+    <cfRule type="containsText" dxfId="21" priority="51" operator="containsText" text="NokiaNetworksFrance">
       <formula>NOT(ISERROR(SEARCH("NokiaNetworksFrance",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G35">
-    <cfRule type="expression" dxfId="21" priority="6">
+    <cfRule type="expression" dxfId="20" priority="8">
       <formula>G35=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="7">
+    <cfRule type="expression" dxfId="19" priority="9">
       <formula>G35=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:L30">
-    <cfRule type="expression" dxfId="19" priority="39">
+    <cfRule type="expression" dxfId="6" priority="41">
       <formula>G2=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="40">
+    <cfRule type="expression" dxfId="5" priority="42">
       <formula>G2=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G31:L40">
-    <cfRule type="expression" dxfId="17" priority="8">
+    <cfRule type="expression" dxfId="18" priority="10">
       <formula>G31=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="9">
+    <cfRule type="expression" dxfId="17" priority="11">
       <formula>G31=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G41:L41">
+    <cfRule type="expression" dxfId="16" priority="3">
+      <formula>G41=TRUE</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="4">
+      <formula>G41=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L30">
-    <cfRule type="containsText" dxfId="15" priority="10" operator="containsText" text="vérifier">
+    <cfRule type="containsText" dxfId="14" priority="12" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",L30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="11" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="13" priority="13" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",L30)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="12">
+    <cfRule type="expression" dxfId="12" priority="14">
       <formula>L30=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="13">
+    <cfRule type="expression" dxfId="11" priority="15">
       <formula>L30=FALSE</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="14" operator="containsText" text="retrouver">
+    <cfRule type="containsText" dxfId="10" priority="16" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",L30)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L28:O30 A2:K40 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 L2:R2 L3:O4 Q3:R4 L5:R5 L6:O8 Q6:R8 L9:R27 Q28:R30 Q32:R32 Q37:R37">
-    <cfRule type="containsText" dxfId="10" priority="24" operator="containsText" text="vérifier">
+  <conditionalFormatting sqref="L28:O30 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 L2:R2 L3:O4 Q3:R4 L5:R5 L6:O8 Q6:R8 L9:R27 Q28:R30 Q32:R32 Q37:R37 A2:K40">
+    <cfRule type="containsText" dxfId="4" priority="26" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="26" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="3" priority="28" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:R2 A2:K40 L3:O4 L5:R5 L6:O8 L9:R27 L28:O30 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 Q3:R4 Q6:R8 Q28:R30 Q32:R32 Q37:R37">
-    <cfRule type="containsText" dxfId="8" priority="44" operator="containsText" text="retrouver">
+  <conditionalFormatting sqref="L2:R2 L3:O4 L5:R5 L6:O8 L9:R27 L28:O30 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 Q3:R4 Q6:R8 Q28:R30 Q32:R32 Q37:R37 A2:K40">
+    <cfRule type="containsText" dxfId="2" priority="46" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:S41">
-    <cfRule type="containsText" dxfId="7" priority="18" operator="containsText" text="vérifier">
+    <cfRule type="containsText" dxfId="9" priority="20" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",S2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="19" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="8" priority="21" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",S2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="20" operator="containsText" text="retrouver">
+    <cfRule type="containsText" dxfId="7" priority="22" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",S2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G41:L41">
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>G41=TRUE</formula>
+  <conditionalFormatting sqref="H36:J36">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>H36=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
-      <formula>G41=FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A41:R41">
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="vérifier">
-      <formula>NOT(ISERROR(SEARCH("vérifier",A41)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="préciser">
-      <formula>NOT(ISERROR(SEARCH("préciser",A41)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A41:R41">
-    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="retrouver">
-      <formula>NOT(ISERROR(SEARCH("retrouver",A41)))</formula>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>H36=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -4479,177 +4504,177 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="34.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="21" t="s">
+        <v>274</v>
+      </c>
+      <c r="B1" s="20"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="22" t="s">
+        <v>280</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
+        <v>290</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="B1" s="22"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="20" t="s">
         <v>300</v>
       </c>
-      <c r="B2" s="24" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="20" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="20" t="s">
         <v>302</v>
       </c>
-      <c r="B3" s="22" t="s">
+    </row>
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" s="20" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
-        <v>302</v>
-      </c>
-      <c r="B4" s="22" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="20" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
-        <v>302</v>
-      </c>
-      <c r="B5" s="22" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="20" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
-        <v>302</v>
-      </c>
-      <c r="B6" s="22" t="s">
+      <c r="B22" s="20" t="s">
         <v>306</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
-        <v>307</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
-        <v>310</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
-        <v>314</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
-        <v>314</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="22" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="B18" s="22" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
-        <v>325</v>
-      </c>
-      <c r="B22" s="22" t="s">
-        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -4670,61 +4695,23 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
+    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
+    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
+      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
+      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -4995,21 +4982,59 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
 <file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
-    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
-    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
-      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
-      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5021,22 +5046,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
+    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5056,13 +5076,18 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
-    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Shorten the catering, RCC 2023, and NAO 2023 texts to match Excel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2548" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAAB38F6-12CA-4BA0-8EE1-6D90B4F40EBD}"/>
+  <xr:revisionPtr revIDLastSave="2739" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B62C6A79-7D3F-45C6-A417-ACE6E3AAB938}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="8925" yWindow="1995" windowWidth="20295" windowHeight="13650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="accords" sheetId="1" r:id="rId1"/>
     <sheet name="rules" sheetId="2" r:id="rId2"/>
+    <sheet name="taux signatures" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">accords!$A$1:$S$30</definedName>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="334">
   <si>
     <t>Accord ou négociation</t>
   </si>
@@ -871,9 +872,6 @@
     <t>Version finale transmise le 03/07/2023, mise à la signature le 04/07/2023 à Massy.</t>
   </si>
   <si>
-    <t>Pas d'accord. Mesures unilatérales au 01/07/2023 : augmentations individuelles 3,21 % des TTC pour les JG 6 et plus, 5 % pour les JG 5 et moins ; GPP et Unexplained Pay Gap maintenus. Primes de transport +5 % ; prime vélo portée à 500 €/an (60 €/mois) ; IK vélo +40 % à 0,35 €/km. Expire le 30/06/2024.</t>
-  </si>
-  <si>
     <t>Réunions des 24/03, 29/03 et 05/04/2023 ; PV de désaccord du 12/04/2023. Contestation des nombreux 0 % d'augmentation (source : tract, à vérifier).</t>
   </si>
   <si>
@@ -1009,9 +1007,6 @@
     <t>Nokia n'a jamais eu l'intention d'aboutir à un accord : la négociation obligatoire a été menée pour la forme. Pas d'engagement d'embauche ni de remplacement des départs, garanties insuffisantes sur les activités en France.</t>
   </si>
   <si>
-    <t>Choix pragmatique tranché assez facilement pour la première édition de ce dispositif, qui garantissait le volontariat en échange de la signature d'un accord majoritaire. Solide sur ses convictions, la CGT sait aussi faire preuve de pragmatisme quand le contexte le permet : volontariat, mesures individuelles correctes, éviter un PSE à moyen terme. Points d'alerte : pressions au volontariat, affaiblissement des équipes, absence de garanties sur les activités en France, lien RCC / absence d'augmentation.</t>
-  </si>
-  <si>
     <t>Deuxième RCC acceptée car la pyramide des âges et le contexte le permettaient encore (départs volontaires majoritairement en fin de carrière) ; mesures individuelles de départ jugées correctes, alternative à un PSE. Bilan a posteriori critique : délocalisations, perte de savoir-faire, charge de travail, RPS, externalisations.</t>
   </si>
   <si>
@@ -1042,17 +1037,41 @@
     <t>Comme pour la GEPP, négociation menée pour la forme : Nokia n'a jamais cherché d'accord. Seuil inatteignable vu le déficit de NNF, donc aucune prime en pratique. Revendication : du salaire fixe plutôt que des primes.</t>
   </si>
   <si>
-    <t>Suite à la baisse des dépenses de restauration depuis le COVID (confinements, télétravail), qui a réduit la contribution ASC versée aux CSE-E, Nokia verse une indemnité transactionnelle de 145 000 € (protocole via le CSE-C, répartie au prorata des effectifs NPS/Lannion) pour solder les années antérieures à 2026. L'avenant sort la restauration des ASC et encadre la délégation à la Direction, qui assume tous les coûts et rend compte de la facturation et du budget à une commission restauration par CSE-E.</t>
-  </si>
-  <si>
     <t>La Direction (M. Cudot) refuse toute modification du texte et exige une réponse avant le 10/07/2026 12h. Signature électronique le 13/07/2026 (2e procédure, les pages n'ayant pas été paraphées au 1er essai). Avis favorable de toutes les OS sur le projet. Risque relevé en interne qu'un échange de mails remplace une vraie négociation. Estimations du manque à percevoir (réunion Direction/DSC/Syndex, 01/10/2025) : ≈ 800 k€ pour Syndex (Paris-Saclay seul, base masse salariale N) contre ≈ 200 k€ pour la Direction (deux sites, base N-1). CSE-E Paris-Saclay du 24/03/2026 : mandat au CSE-C pour transiger à 145 000 € (unanimité, 25 voix).</t>
+  </si>
+  <si>
+    <t>Choix pragmatique pour la première édition de ce dispositif, qui garantissait le volontariat en échange de la signature d'un accord majoritaire. Solide sur ses convictions, la CGT sait aussi faire preuve de pragmatisme quand le contexte le permet : volontariat, mesures individuelles correctes, éviter un PSE à moyen terme. Points d'alerte : pressions au volontariat, affaiblissement des équipes, absence de garanties sur les activités en France, lien RCC / absence d'augmentation.</t>
+  </si>
+  <si>
+    <t>Baisse des dépenses de restauration post-COVID : Nokia verse 145 000 € aux CSE-E (au prorata des effectifs) pour solder le passé. La restauration sort des ASC ; la Direction en assume tous les coûts et rend compte de la facturation à une commission restauration.</t>
+  </si>
+  <si>
+    <t>Taux de signature par site et par OS (source : feuille accords)</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Nb accords / négos</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Pas d'accord. Mesures unilatérales au 01/07/2023 : augmentations individuelles de 3,21 % (5 % pour les JG 5 et moins), sans augmentation générale ; primes de transport et prime vélo revalorisées.</t>
+  </si>
+  <si>
+    <t>Exclus du calcul</t>
+  </si>
+  <si>
+    <t>Taux = accords signés par l'OS / accords et négociations du site (PV de désaccord inclus), hors lignes listées en H4:H20. CFTC : uniquement NPS (« - » ailleurs).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1111,8 +1130,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1125,8 +1152,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1206,12 +1239,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1279,6 +1321,25 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1963,7 +2024,7 @@
         <v>228</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="Q2" s="15" t="s">
         <v>132</v>
@@ -2094,7 +2155,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>99</v>
@@ -2133,10 +2194,10 @@
         <v>326</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="Q5" s="15" t="s">
         <v>8</v>
@@ -2199,7 +2260,7 @@
         <v>229</v>
       </c>
       <c r="P6" s="17" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="Q6" s="16" t="s">
         <v>8</v>
@@ -2312,13 +2373,13 @@
         <v>81</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="P8" s="17" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="Q8" s="15" t="s">
         <v>8</v>
@@ -2505,7 +2566,7 @@
         <v>254</v>
       </c>
       <c r="P11" s="11" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="Q11" s="15" t="s">
         <v>133</v>
@@ -2687,13 +2748,13 @@
         <v>82</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="O14" s="11" t="s">
         <v>257</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="Q14" s="15" t="s">
         <v>134</v>
@@ -2757,7 +2818,7 @@
         <v>230</v>
       </c>
       <c r="P15" s="11" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="Q15" s="15" t="s">
         <v>8</v>
@@ -2806,19 +2867,19 @@
         <v>8</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="M16" s="12" t="s">
         <v>201</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="P16" s="15" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="Q16" s="15" t="s">
         <v>8</v>
@@ -2990,10 +3051,10 @@
         <v>209</v>
       </c>
       <c r="M19" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="N19" s="11" t="s">
         <v>310</v>
-      </c>
-      <c r="N19" s="11" t="s">
-        <v>311</v>
       </c>
       <c r="O19" s="11" t="s">
         <v>260</v>
@@ -3356,13 +3417,13 @@
         <v>82</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="O25" s="11" t="s">
         <v>231</v>
       </c>
       <c r="P25" s="11" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="Q25" s="15" t="s">
         <v>8</v>
@@ -3422,10 +3483,10 @@
         <v>118</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="P26" s="11" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="Q26" s="15" t="s">
         <v>137</v>
@@ -3789,10 +3850,10 @@
         <v>120</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="P32" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q32" s="15" t="s">
         <v>8</v>
@@ -3932,7 +3993,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="135" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A35" s="10">
         <v>2023</v>
       </c>
@@ -3982,7 +4043,7 @@
         <v>268</v>
       </c>
       <c r="P35" s="11" t="s">
-        <v>315</v>
+        <v>325</v>
       </c>
       <c r="Q35" s="15" t="s">
         <v>140</v>
@@ -3995,7 +4056,7 @@
         <v>Tract Volontariat RCC.pdf</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A36" s="10">
         <v>2023</v>
       </c>
@@ -4038,10 +4099,10 @@
         <v>82</v>
       </c>
       <c r="N36" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="O36" s="11" t="s">
         <v>269</v>
-      </c>
-      <c r="O36" s="11" t="s">
-        <v>270</v>
       </c>
       <c r="P36" s="11" t="s">
         <v>218</v>
@@ -4104,7 +4165,7 @@
         <v>124</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P37" s="17" t="s">
         <v>240</v>
@@ -4230,7 +4291,7 @@
       </c>
       <c r="O39" s="11"/>
       <c r="P39" s="11" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="Q39" s="15"/>
       <c r="R39" s="19"/>
@@ -4285,7 +4346,7 @@
       </c>
       <c r="O40" s="11"/>
       <c r="P40" s="15" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="Q40" s="15"/>
       <c r="R40" s="19"/>
@@ -4505,56 +4566,56 @@
   <sheetData>
     <row r="1" spans="1:2" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
+        <v>279</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>280</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
+        <v>281</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>282</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
+        <v>286</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>287</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -4562,15 +4623,15 @@
         <v>0</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
+        <v>289</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>290</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4578,7 +4639,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -4586,23 +4647,23 @@
         <v>221</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
+        <v>293</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>294</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -4610,7 +4671,7 @@
         <v>50</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4618,7 +4679,7 @@
         <v>24</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -4626,7 +4687,7 @@
         <v>24</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4634,7 +4695,7 @@
         <v>24</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4642,7 +4703,7 @@
         <v>93</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4650,7 +4711,7 @@
         <v>11</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4658,7 +4719,7 @@
         <v>92</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -4666,15 +4727,15 @@
         <v>129</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="B22" s="20" t="s">
         <v>305</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>306</v>
       </c>
     </row>
   </sheetData>
@@ -4682,6 +4743,161 @@
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
   </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C2213F0-5B65-4D3B-9535-4DE25C5383C0}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="3" max="6" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="24" t="s">
+        <v>328</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>329</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="H3" s="24" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="27" cm="1">
+        <f t="array" ref="B4">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A4="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A4))))</f>
+        <v>24</v>
+      </c>
+      <c r="C4" s="28" cm="1">
+        <f t="array" ref="C4">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!H$2:H$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A4="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A4)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D4" s="28" cm="1">
+        <f t="array" ref="D4">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!I$2:I$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A4="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A4)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E4" s="28" cm="1">
+        <f t="array" ref="E4">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!J$2:J$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A4="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A4)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F4" s="28" t="str" cm="1">
+        <f t="array" ref="F4">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!K$2:K$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A4="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A4)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>-</v>
+      </c>
+      <c r="H4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="27" cm="1">
+        <f t="array" ref="B5">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A5="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A5))))</f>
+        <v>8</v>
+      </c>
+      <c r="C5" s="28" cm="1">
+        <f t="array" ref="C5">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!H$2:H$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A5="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A5)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>1</v>
+      </c>
+      <c r="D5" s="28" cm="1">
+        <f t="array" ref="D5">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!I$2:I$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A5="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A5)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>1</v>
+      </c>
+      <c r="E5" s="28" cm="1">
+        <f t="array" ref="E5">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!J$2:J$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A5="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A5)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>1</v>
+      </c>
+      <c r="F5" s="28" cm="1">
+        <f t="array" ref="F5">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!K$2:K$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A5="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A5)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B6" s="27" cm="1">
+        <f t="array" ref="B6">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A6="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A6))))</f>
+        <v>6</v>
+      </c>
+      <c r="C6" s="28" cm="1">
+        <f t="array" ref="C6">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!H$2:H$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A6="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A6)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D6" s="28" cm="1">
+        <f t="array" ref="D6">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!I$2:I$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A6="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A6)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>1</v>
+      </c>
+      <c r="E6" s="28" cm="1">
+        <f t="array" ref="E6">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!J$2:J$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A6="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A6)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="F6" s="28" t="str" cm="1">
+        <f t="array" ref="F6">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!K$2:K$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A6="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A6)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="B7" s="29" cm="1">
+        <f t="array" ref="B7">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A7="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A7))))</f>
+        <v>38</v>
+      </c>
+      <c r="C7" s="30" cm="1">
+        <f t="array" ref="C7">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!H$2:H$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A7="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A7)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.65789473684210531</v>
+      </c>
+      <c r="D7" s="30" cm="1">
+        <f t="array" ref="D7">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!I$2:I$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A7="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A7)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.94736842105263153</v>
+      </c>
+      <c r="E7" s="30" cm="1">
+        <f t="array" ref="E7">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!J$2:J$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A7="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A7)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>0.84210526315789469</v>
+      </c>
+      <c r="F7" s="30" cm="1">
+        <f t="array" ref="F7">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.os,accords!K$2:K$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),_xlpm.sel,IF($A7="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A7)),_xlpm.n,SUM(_xlpm.sel*(_xlpm.os&lt;&gt;"-")),IF(_xlpm.n=0,"-",SUM(_xlpm.sel*(_xlpm.os=TRUE))/_xlpm.n))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="31" t="s">
+        <v>333</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Open signature captures in the SharePoint viewer and align the RCC 2026 wording with Excel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2739" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B62C6A79-7D3F-45C6-A417-ACE6E3AAB938}"/>
+  <xr:revisionPtr revIDLastSave="2783" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E65FED76-B9AE-49DB-BB54-1A98F0A10806}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="8925" yWindow="1995" windowWidth="20295" windowHeight="13650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="accords" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -248,63 +248,6 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Plan-de-transformation/RCC%202025/Avenant%20RCC%202025.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CGF_p10_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2024_p04_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2026_p54_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_no_1_a_l_Accord_CSE_du_21_septembre_2018_p10_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2026_Proces_verbal_d_accord_24_janvier_2026_p07_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_RCC_2025_p07_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Amenagement_Temps_Travail_NPS_2026_19_decembre_2025_p03_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_collectif_portant_sur_une_Rupture_Conventionnelle_Collective_RCC__p52_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Entreprise_au_sein_de_Noki_p17-18_signatures.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Retraite_d_Entreprise_Coll_p20-21_signatures.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CET_24_juillet_2025_p13-14_signatures.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_interessement_2025_2028_p16_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_accord_teletravail_avril_2022_p07_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_don_de_jours_14_novembre_2024_p11_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2024_19_avril_2024_p47_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_cadre_NPS_nouvelle_convention_collective_2024_signe_p06_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_de_substitution_non_cadres_30_novembre_2023_p09_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2023_p49_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_remboursement_sante_2023_p11_signature.jpg</t>
-  </si>
-  <si>
     <t>p.10 : signatures de la Direction, de la CFDT, de la CFE-CGC et de la CGT.</t>
   </si>
   <si>
@@ -329,15 +272,9 @@
     <t>p.16 : signatures de la Direction, de la CFDT, de la CFE-CGC et de la CGT.</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_egalite_professionnelle_p20_signature.jpg</t>
-  </si>
-  <si>
     <t>Aménagement du temps de travail 2023</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2023_p04_signature.jpg</t>
-  </si>
-  <si>
     <t>Comité Groupe France (NNF, ASN, RFS).</t>
   </si>
   <si>
@@ -587,48 +524,9 @@
     <t>https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20am%C3%A9nagement%20temps%20travail%20NPS%202023.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_a_la_situation_de_handicap_NNF_p15-16_signatures.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_2025_NPS_amenagement_temps_de_travail_20_janvier_2025_p04_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_2026_protocole_accord_preectoral_LANNION_signe_p11_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_2026_protocole_accord_preelectoral_signe_p11_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Accord_ARTT_Lannion_20_03_2025_p08_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Accord_Horaire_Variable_Lannion_20_03_2025_p07_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_frais_de_sante_9_avril_2025_p05-06_signatures.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Etablissement_Prorogation_des_Mandats_CSE_E_Lannion_p05_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Etablissement_NNF_Lannion_Mise_en_place_accord_cadre_nouvelle_CCN_p06_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_collectif_mise_en_place_CCN_p06_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_augmentation_nombre_delegues_syndicaux_NPS_2023_p05_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_nombre_delegues_syndicaux_Lannion_24_janvier_2023_p04_signature.jpg</t>
-  </si>
-  <si>
     <t>p.11 : signatures de la Direction, de la CFDT, de la CFE-CGC et de la CGT.</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_harmonisation_taux_variable_cible_salaries_non_sales_du_19_decemb_p10_signature.jpg</t>
-  </si>
-  <si>
     <t>p.54 : signatures de la CFDT et de la CFE-CGC ; aucune signature de la CGT.</t>
   </si>
   <si>
@@ -689,21 +587,6 @@
     <t>p.5 : signatures de la Direction, de la CFDT, de la CFE-CGC, de la CFTC et de la CGT.</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_GEPP_PV_de_desaccord_mis_a_signature_p12_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Proces_verbal_NAO_desaccord_2025_27_mars_2025_p11_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_PV_desaccord_Partage_de_la_valeur_VS_p06_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Proces_verbal_de_desaccord_NAO_2024_9_avril_2024_p05_signature.jpg</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2023_PV_desaccord_p10_signature.jpg</t>
-  </si>
-  <si>
     <t>Abondement concentré sur les actions Nokia, rémunération « TTC », exonérations de cotisations ; préférence pour un 13e mois cotisé.</t>
   </si>
   <si>
@@ -896,9 +779,6 @@
     <t>Source : communication intersyndicale. Résultat obtenu par l'avocat du CSE-C (ce que la Direction proposait en échange d'une signature).</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_accord_collectif_relatif_aux_evolutions_du_regime_AUXAD_VF_p06_signature.jpg</t>
-  </si>
-  <si>
     <t>Vote AG extra CGT du 27/03/2025 : « La CGT signe l'accord AUXAD et ses contreparties ». Réunions des 13/02 et 28/03/2025 ; courriel Direction du 31/03/2025 (mise à la signature au 09/04/2025) ; info-consultation CSE-C extraordinaire du 09/04/2025. Argumentaire AG CGT (mars 2025). Négociation au pas de course, quasi exclusivement en bilatérales DSC, opacité sur les sommes provisionnées.</t>
   </si>
   <si>
@@ -998,9 +878,6 @@
     <t>Pas d'accord majoritaire. Mesures unilatérales : budget d'augmentations individuelles de 2 % des TTC, sans augmentation générale ; GPP et Unexplained Pay Gap maintenus ; primes de transport revalorisées de 5 %.</t>
   </si>
   <si>
-    <t>Trop c'est trop : la CGT a fait preuve de flexibilité et de pragmatisme en accompagnant les deux RCC précédentes (2023, 2024), un dispositif qui échange une signature contre la garantie du volontariat. La Direction semble désormais vouloir se faire un PSE en 4 fois, sans frais : ce sera sans nous. Jusqu'à 421 suppressions de postes non justifiées par la charge de travail ; ni garantie d'emploi ni embauche ; externalisations et perte de compétences ; pression au volontariat.</t>
-  </si>
-  <si>
     <t>Accord technique : il formalise une délégation de la restauration à la Direction déjà en place, sans enjeu de fond défavorable.</t>
   </si>
   <si>
@@ -1065,6 +942,129 @@
   </si>
   <si>
     <t>Taux = accords signés par l'OS / accords et négociations du site (PV de désaccord inclus), hors lignes listées en H4:H20. CFTC : uniquement NPS (« - » ailleurs).</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2026_p54_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_2026_protocole_accord_preectoral_LANNION_signe_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_2026_protocole_accord_preelectoral_signe_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_no_1_a_l_Accord_CSE_du_21_septembre_2018_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_a_la_situation_de_handicap_NNF_p15-16_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Etablissement_Prorogation_des_Mandats_CSE_E_Lannion_p05_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2026_Proces_verbal_d_accord_24_janvier_2026_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_RCC_2025_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Amenagement_Temps_Travail_NPS_2026_19_decembre_2025_p03_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_collectif_portant_sur_une_Rupture_Conventionnelle_Collective_RCC__p52_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Entreprise_au_sein_de_Noki_p17-18_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Retraite_d_Entreprise_Coll_p20-21_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_GEPP_PV_de_desaccord_mis_a_signature_p12_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CET_24_juillet_2025_p13-14_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_accord_collectif_relatif_aux_evolutions_du_regime_AUXAD_VF_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_frais_de_sante_9_avril_2025_p05-06_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_interessement_2025_2028_p16_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Proces_verbal_NAO_desaccord_2025_27_mars_2025_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Accord_ARTT_Lannion_20_03_2025_p08_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Accord_Horaire_Variable_Lannion_20_03_2025_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_accord_teletravail_avril_2022_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_2025_NPS_amenagement_temps_de_travail_20_janvier_2025_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_don_de_jours_14_novembre_2024_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_PV_desaccord_Partage_de_la_valeur_VS_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2024_19_avril_2024_p47_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Proces_verbal_de_desaccord_NAO_2024_9_avril_2024_p05_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CGF_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Etablissement_NNF_Lannion_Mise_en_place_accord_cadre_nouvelle_CCN_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_cadre_NPS_nouvelle_convention_collective_2024_signe_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_collectif_mise_en_place_CCN_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_harmonisation_taux_variable_cible_salaries_non_sales_du_19_decemb_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2024_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_de_substitution_non_cadres_30_novembre_2023_p09_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2023_p49_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2023_PV_desaccord_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_egalite_professionnelle_p20_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2023_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_nombre_delegues_syndicaux_Lannion_24_janvier_2023_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_augmentation_nombre_delegues_syndicaux_NPS_2023_p05_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_remboursement_sante_2023_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>Trop c'est trop : la CGT a fait preuve de flexibilité et de pragmatisme en accompagnant les deux RCC précédentes (2023, 2024), un dispositif qui échange une signature contre la garantie du volontariat. La Direction semble désormais vouloir se faire un PSE EN 4X SANS FRAIS : ce sera sans nous. Jusqu'à 421 suppressions de postes non justifiées par la charge de travail ; ni garantie d'emploi ni embauche ; externalisations et perte de compétences ; pression au volontariat.</t>
   </si>
 </sst>
 </file>
@@ -1347,28 +1347,6 @@
   </cellStyles>
   <dxfs count="29">
     <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1389,28 +1367,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1481,6 +1437,50 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1625,10 +1625,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1926,16 +1922,16 @@
         <v>0</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>10</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>221</v>
+        <v>182</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>1</v>
@@ -1947,7 +1943,7 @@
         <v>3</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>222</v>
+        <v>183</v>
       </c>
       <c r="L1" s="9" t="s">
         <v>50</v>
@@ -1956,22 +1952,22 @@
         <v>24</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="P1" s="8" t="s">
         <v>11</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="105" x14ac:dyDescent="0.25">
@@ -2012,22 +2008,22 @@
         <v>-</v>
       </c>
       <c r="L2" s="19" t="s">
-        <v>63</v>
+        <v>293</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>188</v>
+        <v>154</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>228</v>
+        <v>189</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>306</v>
+        <v>266</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>132</v>
+        <v>111</v>
       </c>
       <c r="R2" s="19" t="s">
         <v>41</v>
@@ -2042,13 +2038,13 @@
         <v>2026</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>152</v>
+        <v>131</v>
       </c>
       <c r="E3" s="11" t="str" cm="1">
         <f t="array" ref="E3">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D3,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2076,17 +2072,17 @@
         <v>-</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>176</v>
+        <v>294</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>186</v>
+        <v>153</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
       <c r="O3" s="11"/>
       <c r="P3" s="17" t="s">
-        <v>232</v>
+        <v>193</v>
       </c>
       <c r="Q3" s="15"/>
       <c r="R3" s="19"/>
@@ -2100,10 +2096,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>143</v>
+        <v>122</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="E4" s="11" t="str" cm="1">
         <f t="array" ref="E4">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D4,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2131,17 +2127,17 @@
         <v>1</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>177</v>
+        <v>295</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
       <c r="O4" s="11"/>
       <c r="P4" s="17" t="s">
-        <v>233</v>
+        <v>194</v>
       </c>
       <c r="Q4" s="15"/>
       <c r="R4" s="19"/>
@@ -2155,10 +2151,10 @@
         <v>13</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>308</v>
+        <v>268</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="E5" s="11" t="str" cm="1">
         <f t="array" ref="E5">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D5,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2185,19 +2181,19 @@
         <v>-</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>64</v>
+        <v>296</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>326</v>
+        <v>285</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>324</v>
+        <v>283</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>312</v>
+        <v>271</v>
       </c>
       <c r="Q5" s="15" t="s">
         <v>8</v>
@@ -2221,7 +2217,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="E6" s="10" t="str" cm="1">
         <f t="array" ref="E6">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D6,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2248,19 +2244,19 @@
         <v>-</v>
       </c>
       <c r="L6" s="19" t="s">
-        <v>174</v>
+        <v>297</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>189</v>
+        <v>155</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>229</v>
+        <v>190</v>
       </c>
       <c r="P6" s="17" t="s">
-        <v>307</v>
+        <v>267</v>
       </c>
       <c r="Q6" s="16" t="s">
         <v>8</v>
@@ -2278,13 +2274,13 @@
         <v>2026</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="E7" s="11" t="str" cm="1">
         <f t="array" ref="E7">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D7,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2312,17 +2308,17 @@
         <v>-</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>181</v>
+        <v>298</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>190</v>
+        <v>156</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="O7" s="11"/>
       <c r="P7" s="17" t="s">
-        <v>250</v>
+        <v>211</v>
       </c>
       <c r="Q7" s="15"/>
       <c r="R7" s="19"/>
@@ -2339,7 +2335,7 @@
         <v>54</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="E8" s="11" t="str" cm="1">
         <f t="array" ref="E8">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D8,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2367,19 +2363,19 @@
         <v>-</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>65</v>
+        <v>299</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>317</v>
+        <v>276</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>274</v>
+        <v>235</v>
       </c>
       <c r="P8" s="17" t="s">
-        <v>318</v>
+        <v>277</v>
       </c>
       <c r="Q8" s="15" t="s">
         <v>8</v>
@@ -2430,19 +2426,19 @@
         <v>-</v>
       </c>
       <c r="L9" s="19" t="s">
-        <v>66</v>
+        <v>300</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>191</v>
+        <v>157</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>251</v>
+        <v>212</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>252</v>
+        <v>213</v>
       </c>
       <c r="Q9" s="15" t="s">
         <v>8</v>
@@ -2493,17 +2489,17 @@
         <v>1</v>
       </c>
       <c r="L10" s="19" t="s">
-        <v>67</v>
+        <v>301</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>192</v>
+        <v>158</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10" t="s">
-        <v>253</v>
+        <v>214</v>
       </c>
       <c r="Q10" s="16" t="s">
         <v>8</v>
@@ -2527,7 +2523,7 @@
         <v>51</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E11" s="11" t="str" cm="1">
         <f t="array" ref="E11">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D11,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2554,22 +2550,22 @@
         <v>-</v>
       </c>
       <c r="L11" s="19" t="s">
-        <v>68</v>
+        <v>302</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="N11" s="11" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="O11" s="11" t="s">
-        <v>254</v>
+        <v>215</v>
       </c>
       <c r="P11" s="11" t="s">
-        <v>311</v>
+        <v>333</v>
       </c>
       <c r="Q11" s="15" t="s">
-        <v>133</v>
+        <v>112</v>
       </c>
       <c r="R11" s="19" t="s">
         <v>42</v>
@@ -2590,7 +2586,7 @@
         <v>17</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="E12" s="11" t="str" cm="1">
         <f t="array" ref="E12">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D12,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2617,19 +2613,19 @@
         <v>-</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>69</v>
+        <v>303</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>194</v>
+        <v>160</v>
       </c>
       <c r="N12" s="11" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="O12" s="11" t="s">
-        <v>255</v>
+        <v>216</v>
       </c>
       <c r="P12" s="11" t="s">
-        <v>213</v>
+        <v>174</v>
       </c>
       <c r="Q12" s="15" t="s">
         <v>8</v>
@@ -2653,7 +2649,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E13" s="11" t="str" cm="1">
         <f t="array" ref="E13">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D13,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2680,19 +2676,19 @@
         <v>-</v>
       </c>
       <c r="L13" s="19" t="s">
-        <v>70</v>
+        <v>304</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>195</v>
+        <v>161</v>
       </c>
       <c r="N13" s="11" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>256</v>
+        <v>217</v>
       </c>
       <c r="P13" s="11" t="s">
-        <v>214</v>
+        <v>175</v>
       </c>
       <c r="Q13" s="15" t="s">
         <v>8</v>
@@ -2713,7 +2709,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>242</v>
+        <v>203</v>
       </c>
       <c r="D14" s="19" t="s">
         <v>28</v>
@@ -2741,23 +2737,23 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="L14" s="19" t="s">
-        <v>208</v>
+      <c r="L14" t="s">
+        <v>305</v>
       </c>
       <c r="M14" s="12" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>319</v>
+        <v>278</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>257</v>
+        <v>218</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>313</v>
+        <v>272</v>
       </c>
       <c r="Q14" s="15" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="R14" s="19" t="s">
         <v>43</v>
@@ -2806,19 +2802,19 @@
         <v>-</v>
       </c>
       <c r="L15" s="19" t="s">
-        <v>71</v>
+        <v>306</v>
       </c>
       <c r="M15" s="12" t="s">
-        <v>196</v>
+        <v>162</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>230</v>
+        <v>191</v>
       </c>
       <c r="P15" s="11" t="s">
-        <v>316</v>
+        <v>275</v>
       </c>
       <c r="Q15" s="15" t="s">
         <v>8</v>
@@ -2839,13 +2835,13 @@
         <v>13</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>249</v>
+        <v>210</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>248</v>
+        <v>209</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="F16" s="12">
         <f>DATE(2025,4,9)</f>
@@ -2867,19 +2863,19 @@
         <v>8</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>277</v>
+        <v>307</v>
       </c>
       <c r="M16" s="12" t="s">
-        <v>201</v>
+        <v>167</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>320</v>
+        <v>279</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>278</v>
+        <v>238</v>
       </c>
       <c r="P16" s="15" t="s">
-        <v>321</v>
+        <v>280</v>
       </c>
       <c r="Q16" s="15" t="s">
         <v>8</v>
@@ -2899,10 +2895,10 @@
         <v>13</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>146</v>
+        <v>125</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>159</v>
+        <v>138</v>
       </c>
       <c r="E17" s="11" t="str" cm="1">
         <f t="array" ref="E17">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D17,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2930,19 +2926,19 @@
         <v>-</v>
       </c>
       <c r="L17" s="19" t="s">
+        <v>308</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="N17" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="O17" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="M17" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="N17" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="O17" s="11" t="s">
+      <c r="P17" s="11" t="s">
         <v>219</v>
-      </c>
-      <c r="P17" s="11" t="s">
-        <v>258</v>
       </c>
       <c r="Q17" s="15"/>
       <c r="R17" s="19"/>
@@ -2959,7 +2955,7 @@
         <v>19</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="E18" s="11" t="str" cm="1">
         <f t="array" ref="E18">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D18,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2986,19 +2982,19 @@
         <v>-</v>
       </c>
       <c r="L18" s="19" t="s">
-        <v>72</v>
+        <v>309</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="O18" s="11" t="s">
-        <v>259</v>
+        <v>220</v>
       </c>
       <c r="P18" s="11" t="s">
-        <v>234</v>
+        <v>195</v>
       </c>
       <c r="Q18" s="15" t="s">
         <v>8</v>
@@ -3019,7 +3015,7 @@
         <v>13</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>243</v>
+        <v>204</v>
       </c>
       <c r="D19" s="19" t="s">
         <v>39</v>
@@ -3048,22 +3044,22 @@
         <v>-</v>
       </c>
       <c r="L19" s="19" t="s">
-        <v>209</v>
+        <v>310</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>309</v>
+        <v>269</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>310</v>
+        <v>270</v>
       </c>
       <c r="O19" s="11" t="s">
-        <v>260</v>
+        <v>221</v>
       </c>
       <c r="P19" s="11" t="s">
-        <v>235</v>
+        <v>196</v>
       </c>
       <c r="Q19" s="15" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="R19" s="19" t="s">
         <v>44</v>
@@ -3078,13 +3074,13 @@
         <v>2025</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>144</v>
+        <v>123</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="E20" s="11" t="str" cm="1">
         <f t="array" ref="E20">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D20,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3111,20 +3107,20 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="L20" s="19" t="s">
-        <v>178</v>
+      <c r="L20" t="s">
+        <v>311</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>198</v>
+        <v>164</v>
       </c>
       <c r="N20" s="11" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="O20" s="11" t="s">
-        <v>261</v>
+        <v>222</v>
       </c>
       <c r="P20" s="11" t="s">
-        <v>236</v>
+        <v>197</v>
       </c>
       <c r="Q20" s="15"/>
       <c r="R20" s="19"/>
@@ -3135,13 +3131,13 @@
         <v>2025</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>145</v>
+        <v>124</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="E21" s="11" t="str" cm="1">
         <f t="array" ref="E21">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D21,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3168,20 +3164,20 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="L21" s="19" t="s">
-        <v>179</v>
+      <c r="L21" t="s">
+        <v>312</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>199</v>
+        <v>165</v>
       </c>
       <c r="N21" s="11" t="s">
-        <v>165</v>
+        <v>144</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>224</v>
+        <v>185</v>
       </c>
       <c r="P21" s="11" t="s">
-        <v>223</v>
+        <v>184</v>
       </c>
       <c r="Q21" s="15"/>
       <c r="R21" s="19"/>
@@ -3198,7 +3194,7 @@
         <v>56</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="E22" s="11" t="str" cm="1">
         <f t="array" ref="E22">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D22,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3225,22 +3221,22 @@
         <v>-</v>
       </c>
       <c r="L22" s="19" t="s">
-        <v>73</v>
+        <v>313</v>
       </c>
       <c r="M22" s="12" t="s">
-        <v>191</v>
+        <v>157</v>
       </c>
       <c r="N22" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="O22" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="P22" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="Q22" s="15" t="s">
         <v>115</v>
-      </c>
-      <c r="O22" s="11" t="s">
-        <v>262</v>
-      </c>
-      <c r="P22" s="11" t="s">
-        <v>263</v>
-      </c>
-      <c r="Q22" s="15" t="s">
-        <v>136</v>
       </c>
       <c r="R22" s="19" t="s">
         <v>45</v>
@@ -3261,7 +3257,7 @@
         <v>57</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="E23" s="10" t="str" cm="1">
         <f t="array" ref="E23">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D23,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3288,17 +3284,17 @@
         <v>1</v>
       </c>
       <c r="L23" s="19" t="s">
-        <v>175</v>
+        <v>314</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="O23" s="10"/>
       <c r="P23" s="10" t="s">
-        <v>253</v>
+        <v>214</v>
       </c>
       <c r="Q23" s="16" t="s">
         <v>8</v>
@@ -3349,19 +3345,19 @@
         <v>-</v>
       </c>
       <c r="L24" s="19" t="s">
-        <v>74</v>
+        <v>315</v>
       </c>
       <c r="M24" s="12" t="s">
-        <v>186</v>
+        <v>153</v>
       </c>
       <c r="N24" s="11" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>264</v>
+        <v>225</v>
       </c>
       <c r="P24" s="11" t="s">
-        <v>215</v>
+        <v>176</v>
       </c>
       <c r="Q24" s="15" t="s">
         <v>8</v>
@@ -3382,10 +3378,10 @@
         <v>13</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>244</v>
+        <v>205</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="E25" s="11" t="str" cm="1">
         <f t="array" ref="E25">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D25,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3411,19 +3407,19 @@
         <v>-</v>
       </c>
       <c r="L25" s="19" t="s">
-        <v>210</v>
+        <v>316</v>
       </c>
       <c r="M25" s="12" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>322</v>
+        <v>281</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>231</v>
+        <v>192</v>
       </c>
       <c r="P25" s="11" t="s">
-        <v>323</v>
+        <v>282</v>
       </c>
       <c r="Q25" s="15" t="s">
         <v>8</v>
@@ -3474,22 +3470,22 @@
         <v>1</v>
       </c>
       <c r="L26" s="19" t="s">
-        <v>75</v>
+        <v>317</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="N26" s="11" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>315</v>
+        <v>274</v>
       </c>
       <c r="P26" s="11" t="s">
-        <v>314</v>
+        <v>273</v>
       </c>
       <c r="Q26" s="15" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="R26" s="19" t="s">
         <v>46</v>
@@ -3507,7 +3503,7 @@
         <v>13</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>245</v>
+        <v>206</v>
       </c>
       <c r="D27" s="19" t="s">
         <v>38</v>
@@ -3537,25 +3533,25 @@
         <v>-</v>
       </c>
       <c r="L27" s="19" t="s">
-        <v>211</v>
+        <v>318</v>
       </c>
       <c r="M27" s="12" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="N27" s="11" t="s">
-        <v>265</v>
+        <v>226</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>266</v>
+        <v>227</v>
       </c>
       <c r="P27" s="11" t="s">
-        <v>237</v>
+        <v>198</v>
       </c>
       <c r="Q27" s="15" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
       <c r="R27" s="19" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="S27" s="11" t="str" cm="1">
         <f t="array" ref="S27">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R27,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3600,19 +3596,19 @@
         <v>-</v>
       </c>
       <c r="L28" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="M28" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="M28" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="N28" s="11" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>267</v>
+        <v>228</v>
       </c>
       <c r="P28" s="17" t="s">
-        <v>216</v>
+        <v>177</v>
       </c>
       <c r="Q28" s="15" t="s">
         <v>8</v>
@@ -3630,13 +3626,13 @@
         <v>2024</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>148</v>
+        <v>127</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="E29" s="11" t="str" cm="1">
         <f t="array" ref="E29">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D29,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3664,19 +3660,19 @@
         <v>-</v>
       </c>
       <c r="L29" s="19" t="s">
-        <v>182</v>
+        <v>320</v>
       </c>
       <c r="M29" s="11" t="s">
-        <v>201</v>
+        <v>167</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>168</v>
+        <v>147</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>225</v>
+        <v>186</v>
       </c>
       <c r="P29" s="17" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="Q29" s="15"/>
       <c r="R29" s="19"/>
@@ -3721,22 +3717,22 @@
         <v>1</v>
       </c>
       <c r="L30" s="19" t="s">
-        <v>76</v>
+        <v>321</v>
       </c>
       <c r="M30" s="12" t="s">
-        <v>202</v>
+        <v>168</v>
       </c>
       <c r="N30" s="11" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>226</v>
+        <v>187</v>
       </c>
       <c r="P30" s="17" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="Q30" s="15" t="s">
-        <v>138</v>
+        <v>117</v>
       </c>
       <c r="R30" s="19" t="s">
         <v>47</v>
@@ -3754,10 +3750,10 @@
         <v>13</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="E31" s="11" t="str" cm="1">
         <f t="array" ref="E31">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D31,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3785,19 +3781,19 @@
         <v>-</v>
       </c>
       <c r="L31" s="19" t="s">
-        <v>183</v>
+        <v>322</v>
       </c>
       <c r="M31" s="11" t="s">
-        <v>201</v>
+        <v>167</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>227</v>
+        <v>188</v>
       </c>
       <c r="P31" s="11" t="s">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="Q31" s="15"/>
       <c r="R31" s="19"/>
@@ -3814,7 +3810,7 @@
         <v>59</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="E32" s="11" t="str" cm="1">
         <f t="array" ref="E32">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D32,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3841,19 +3837,19 @@
         <v>-</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>187</v>
+        <v>323</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="N32" s="11" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>276</v>
+        <v>237</v>
       </c>
       <c r="P32" s="17" t="s">
-        <v>275</v>
+        <v>236</v>
       </c>
       <c r="Q32" s="15" t="s">
         <v>8</v>
@@ -3904,19 +3900,19 @@
         <v>1</v>
       </c>
       <c r="L33" s="19" t="s">
-        <v>62</v>
+        <v>324</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="N33" s="11" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>217</v>
+        <v>178</v>
       </c>
       <c r="P33" s="11" t="s">
-        <v>253</v>
+        <v>214</v>
       </c>
       <c r="Q33" s="15" t="s">
         <v>8</v>
@@ -3968,19 +3964,19 @@
         <v>-</v>
       </c>
       <c r="L34" s="19" t="s">
-        <v>77</v>
+        <v>325</v>
       </c>
       <c r="M34" s="12" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="N34" s="11" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>220</v>
+        <v>181</v>
       </c>
       <c r="P34" s="11" t="s">
-        <v>239</v>
+        <v>200</v>
       </c>
       <c r="Q34" s="15" t="s">
         <v>8</v>
@@ -4031,22 +4027,22 @@
         <v>-</v>
       </c>
       <c r="L35" s="19" t="s">
-        <v>78</v>
+        <v>326</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>204</v>
+        <v>170</v>
       </c>
       <c r="N35" s="11" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>268</v>
+        <v>229</v>
       </c>
       <c r="P35" s="11" t="s">
-        <v>325</v>
+        <v>284</v>
       </c>
       <c r="Q35" s="15" t="s">
-        <v>140</v>
+        <v>119</v>
       </c>
       <c r="R35" s="19" t="s">
         <v>48</v>
@@ -4064,7 +4060,7 @@
         <v>13</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>246</v>
+        <v>207</v>
       </c>
       <c r="D36" s="19" t="s">
         <v>36</v>
@@ -4093,22 +4089,22 @@
         <v>-</v>
       </c>
       <c r="L36" s="19" t="s">
-        <v>212</v>
+        <v>327</v>
       </c>
       <c r="M36" s="12" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="N36" s="11" t="s">
-        <v>331</v>
+        <v>290</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>269</v>
+        <v>230</v>
       </c>
       <c r="P36" s="11" t="s">
-        <v>218</v>
+        <v>179</v>
       </c>
       <c r="Q36" s="15" t="s">
-        <v>141</v>
+        <v>120</v>
       </c>
       <c r="R36" s="19" t="s">
         <v>49</v>
@@ -4156,22 +4152,22 @@
         <v>-</v>
       </c>
       <c r="L37" s="19" t="s">
-        <v>88</v>
+        <v>328</v>
       </c>
       <c r="M37" s="12" t="s">
-        <v>205</v>
+        <v>171</v>
       </c>
       <c r="N37" s="11" t="s">
-        <v>124</v>
+        <v>103</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>270</v>
+        <v>231</v>
       </c>
       <c r="P37" s="17" t="s">
-        <v>240</v>
+        <v>201</v>
       </c>
       <c r="Q37" s="15" t="s">
-        <v>141</v>
+        <v>120</v>
       </c>
       <c r="R37" s="19" t="s">
         <v>49</v>
@@ -4189,10 +4185,10 @@
         <v>14</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>173</v>
+        <v>152</v>
       </c>
       <c r="E38" s="11" t="str" cm="1">
         <f t="array" ref="E38">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D38,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4219,17 +4215,17 @@
         <v>1</v>
       </c>
       <c r="L38" s="19" t="s">
-        <v>90</v>
+        <v>329</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="N38" s="11" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="O38" s="11"/>
       <c r="P38" s="11" t="s">
-        <v>253</v>
+        <v>214</v>
       </c>
       <c r="Q38" s="15" t="s">
         <v>8</v>
@@ -4247,13 +4243,13 @@
         <v>2023</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>151</v>
+        <v>130</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>161</v>
+        <v>140</v>
       </c>
       <c r="E39" s="11" t="str" cm="1">
         <f t="array" ref="E39">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D39,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4281,17 +4277,17 @@
         <v>-</v>
       </c>
       <c r="L39" s="19" t="s">
-        <v>185</v>
+        <v>330</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>206</v>
+        <v>172</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="O39" s="11"/>
       <c r="P39" s="11" t="s">
-        <v>271</v>
+        <v>232</v>
       </c>
       <c r="Q39" s="15"/>
       <c r="R39" s="19"/>
@@ -4305,10 +4301,10 @@
         <v>14</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="E40" s="11" t="str" cm="1">
         <f t="array" ref="E40">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D40,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4336,17 +4332,17 @@
         <v>1</v>
       </c>
       <c r="L40" s="19" t="s">
-        <v>184</v>
+        <v>331</v>
       </c>
       <c r="M40" s="12" t="s">
-        <v>207</v>
+        <v>173</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>170</v>
+        <v>149</v>
       </c>
       <c r="O40" s="11"/>
       <c r="P40" s="15" t="s">
-        <v>272</v>
+        <v>233</v>
       </c>
       <c r="Q40" s="15"/>
       <c r="R40" s="19"/>
@@ -4391,17 +4387,17 @@
         <v>-</v>
       </c>
       <c r="L41" s="19" t="s">
-        <v>79</v>
+        <v>332</v>
       </c>
       <c r="M41" s="12" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>125</v>
+        <v>104</v>
       </c>
       <c r="O41" s="11"/>
       <c r="P41" s="15" t="s">
-        <v>241</v>
+        <v>202</v>
       </c>
       <c r="Q41" s="15" t="s">
         <v>8</v>
@@ -4456,76 +4452,76 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:L30">
-    <cfRule type="expression" dxfId="6" priority="41">
+    <cfRule type="expression" dxfId="18" priority="41">
       <formula>G2=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="42">
+    <cfRule type="expression" dxfId="17" priority="42">
       <formula>G2=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G31:L40">
-    <cfRule type="expression" dxfId="18" priority="10">
+    <cfRule type="expression" dxfId="16" priority="10">
       <formula>G31=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="11">
+    <cfRule type="expression" dxfId="15" priority="11">
       <formula>G31=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G41:L41">
-    <cfRule type="expression" dxfId="16" priority="3">
+    <cfRule type="expression" dxfId="14" priority="3">
       <formula>G41=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="4">
+    <cfRule type="expression" dxfId="13" priority="4">
       <formula>G41=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H36:J36">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>H36=TRUE</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="2">
+      <formula>H36=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L30">
-    <cfRule type="containsText" dxfId="14" priority="12" operator="containsText" text="vérifier">
+    <cfRule type="containsText" dxfId="10" priority="12" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",L30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="13" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="9" priority="13" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",L30)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="14">
+    <cfRule type="expression" dxfId="8" priority="14">
       <formula>L30=TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="15">
+    <cfRule type="expression" dxfId="7" priority="15">
       <formula>L30=FALSE</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="16" operator="containsText" text="retrouver">
+    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",L30)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L28:O30 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 L2:R2 L3:O4 Q3:R4 L5:R5 L6:O8 Q6:R8 L9:R27 Q28:R30 Q32:R32 Q37:R37 A2:K40">
-    <cfRule type="containsText" dxfId="4" priority="26" operator="containsText" text="vérifier">
+  <conditionalFormatting sqref="L28:O30 A2:K40 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 L2:R2 L3:O4 Q3:R4 L5:R5 L6:O8 Q6:R8 L9:R27 Q28:R30 Q32:R32 Q37:R37">
+    <cfRule type="containsText" dxfId="5" priority="26" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="28" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="4" priority="28" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:R2 L3:O4 L5:R5 L6:O8 L9:R27 L28:O30 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 Q3:R4 Q6:R8 Q28:R30 Q32:R32 Q37:R37 A2:K40">
-    <cfRule type="containsText" dxfId="2" priority="46" operator="containsText" text="retrouver">
+  <conditionalFormatting sqref="L2:R2 A2:K40 L3:O4 L5:R5 L6:O8 L9:R27 L28:O30 L31:R31 L32:O32 L33:R36 L37:O37 L38:R40 Q3:R4 Q6:R8 Q28:R30 Q32:R32 Q37:R37">
+    <cfRule type="containsText" dxfId="3" priority="46" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:S41">
-    <cfRule type="containsText" dxfId="9" priority="20" operator="containsText" text="vérifier">
+    <cfRule type="containsText" dxfId="2" priority="20" operator="containsText" text="vérifier">
       <formula>NOT(ISERROR(SEARCH("vérifier",S2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="21" operator="containsText" text="préciser">
+    <cfRule type="containsText" dxfId="1" priority="21" operator="containsText" text="préciser">
       <formula>NOT(ISERROR(SEARCH("préciser",S2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="22" operator="containsText" text="retrouver">
+    <cfRule type="containsText" dxfId="0" priority="22" operator="containsText" text="retrouver">
       <formula>NOT(ISERROR(SEARCH("retrouver",S2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H36:J36">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>H36=TRUE</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>H36=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -4541,14 +4537,11 @@
     <hyperlink ref="D39" r:id="rId10" display="https://nokia.sharepoint.com/:b:/r/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20nombre%20d%C3%A9l%C3%A9gu%C3%A9s%20syndicaux%20Lannion%2024%20janvier%202023.pdf?d=w7f99dd8365c6418eb22acb63a8ac44b2&amp;csf=1&amp;web=1&amp;e=nOfza5" xr:uid="{F1E97C35-916D-446B-B83F-9D8E27B48A78}"/>
     <hyperlink ref="D38" r:id="rId11" xr:uid="{3CA5F90A-37A0-47B4-A593-00FA1CC25A3A}"/>
     <hyperlink ref="D23" r:id="rId12" xr:uid="{953BDEB9-68F0-45C1-BEE6-C570830B2425}"/>
-    <hyperlink ref="L20" r:id="rId13" xr:uid="{9553D652-6925-4255-8B66-56354E6BF3B1}"/>
-    <hyperlink ref="L21" r:id="rId14" xr:uid="{0B7E48E3-FDDE-4B3A-A09C-DE4FFC8D13AF}"/>
-    <hyperlink ref="D25" r:id="rId15" xr:uid="{35FF18B8-C1F8-4ACB-AC18-C9B1639EB410}"/>
-    <hyperlink ref="L14" r:id="rId16" xr:uid="{BA92569F-D437-4A24-9A1C-EDBCBE27EBE4}"/>
-    <hyperlink ref="D16" r:id="rId17" display="https://nokia.sharepoint.com/sites/BDESENNF-CSE-C/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FBDESENNF%2DCSE%2DC%2FShared%20Documents%2F05a%2E%20CSE%2DC%2FCSE%2DC%202025%2F03%2DCSE%2DC%20extraordinaire%209%20avril%202025%2Faccord%20collectif%20relatif%20aux%20%C3%A9volutions%20du%20r%C3%A9gime%20AUXAD%20%2DVF%2Epdf" xr:uid="{22171004-D3FC-446C-9F9D-36C128A50C34}"/>
+    <hyperlink ref="D25" r:id="rId13" xr:uid="{35FF18B8-C1F8-4ACB-AC18-C9B1639EB410}"/>
+    <hyperlink ref="D16" r:id="rId14" display="https://nokia.sharepoint.com/sites/BDESENNF-CSE-C/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FBDESENNF%2DCSE%2DC%2FShared%20Documents%2F05a%2E%20CSE%2DC%2FCSE%2DC%202025%2F03%2DCSE%2DC%20extraordinaire%209%20avril%202025%2Faccord%20collectif%20relatif%20aux%20%C3%A9volutions%20du%20r%C3%A9gime%20AUXAD%20%2DVF%2Epdf" xr:uid="{22171004-D3FC-446C-9F9D-36C128A50C34}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId18"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Nokia internal use</oddFooter>
   </headerFooter>
@@ -4566,56 +4559,56 @@
   <sheetData>
     <row r="1" spans="1:2" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>273</v>
+        <v>234</v>
       </c>
       <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>279</v>
+        <v>239</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>280</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>281</v>
+        <v>241</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>282</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
-        <v>281</v>
+        <v>241</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>283</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
-        <v>281</v>
+        <v>241</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>284</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>281</v>
+        <v>241</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>285</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
-        <v>286</v>
+        <v>246</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>287</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -4623,15 +4616,15 @@
         <v>0</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>288</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
-        <v>289</v>
+        <v>249</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>290</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4639,31 +4632,31 @@
         <v>10</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>291</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
-        <v>221</v>
+        <v>182</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>292</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
-        <v>293</v>
+        <v>253</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>294</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
-        <v>293</v>
+        <v>253</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>295</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -4671,7 +4664,7 @@
         <v>50</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>296</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4679,7 +4672,7 @@
         <v>24</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>297</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -4687,7 +4680,7 @@
         <v>24</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>298</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4695,15 +4688,15 @@
         <v>24</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>299</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>300</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4711,31 +4704,31 @@
         <v>11</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>301</v>
+        <v>261</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>302</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>303</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>304</v>
+        <v>264</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>305</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -4759,15 +4752,15 @@
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
-        <v>327</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>328</v>
+        <v>287</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>329</v>
+        <v>288</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>1</v>
@@ -4779,10 +4772,10 @@
         <v>3</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>222</v>
+        <v>183</v>
       </c>
       <c r="H3" s="24" t="s">
-        <v>332</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -4810,7 +4803,7 @@
         <v>-</v>
       </c>
       <c r="H4" t="s">
-        <v>242</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -4838,12 +4831,12 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>244</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="B6" s="27" cm="1">
         <f t="array" ref="B6">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A6="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A6))))</f>
@@ -4868,7 +4861,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>330</v>
+        <v>289</v>
       </c>
       <c r="B7" s="29" cm="1">
         <f t="array" ref="B7">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A7="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A7))))</f>
@@ -4893,7 +4886,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move the agreements page next to its logo and signature captures, and open the AUXAD agreement as a PDF.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia.sharepoint.com/sites/CGT39/Shared Documents/salariés/accords négociés/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2783" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E65FED76-B9AE-49DB-BB54-1A98F0A10806}"/>
+  <xr:revisionPtr revIDLastSave="2791" documentId="11_F25DC773A252ABDACC1048A741DB65945BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CC6DB05-A7C7-472B-87A4-FDF05B0AD720}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="3315" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="accords" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -149,9 +149,6 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202024/Accord%20am%C3%A9nagement%20temps%20travail%20NPS%202024.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/copies/GEPP%20PV%20de%20d%C3%A9saccord%20mis%20%C3%A0%20signature.pdf</t>
-  </si>
-  <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202023/Accord%20%C3%A9galit%C3%A9%20professionnelle.pdf</t>
   </si>
   <si>
@@ -692,9 +689,6 @@
     <t>accord collectif relatif aux évolutions du régime AUXAD -VF.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/BDESENNF-CSE-C/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FBDESENNF%2DCSE%2DC%2FShared%20Documents%2F05a%2E%20CSE%2DC%2FCSE%2DC%202025%2F03%2DCSE%2DC%20extraordinaire%209%20avril%202025%2Faccord%20collectif%20relatif%20aux%20%C3%A9volutions%20du%20r%C3%A9gime%20AUXAD%20%2DVF%2Epdf</t>
-  </si>
-  <si>
     <t>Évolutions du régime AUXAD</t>
   </si>
   <si>
@@ -944,127 +938,133 @@
     <t>Taux = accords signés par l'OS / accords et négociations du site (PV de désaccord inclus), hors lignes listées en H4:H20. CFTC : uniquement NPS (« - » ailleurs).</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2026_p54_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_2026_protocole_accord_preectoral_LANNION_signe_p11_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_2026_protocole_accord_preelectoral_signe_p11_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_no_1_a_l_Accord_CSE_du_21_septembre_2018_p10_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_a_la_situation_de_handicap_NNF_p15-16_signatures.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Etablissement_Prorogation_des_Mandats_CSE_E_Lannion_p05_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2026_Proces_verbal_d_accord_24_janvier_2026_p07_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_RCC_2025_p07_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Amenagement_Temps_Travail_NPS_2026_19_decembre_2025_p03_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_collectif_portant_sur_une_Rupture_Conventionnelle_Collective_RCC__p52_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Entreprise_au_sein_de_Noki_p17-18_signatures.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Retraite_d_Entreprise_Coll_p20-21_signatures.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/cgt_GEPP_PV_de_desaccord_mis_a_signature_p12_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CET_24_juillet_2025_p13-14_signatures.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_accord_collectif_relatif_aux_evolutions_du_regime_AUXAD_VF_p06_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_frais_de_sante_9_avril_2025_p05-06_signatures.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_d_interessement_2025_2028_p16_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Proces_verbal_NAO_desaccord_2025_27_mars_2025_p11_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Accord_ARTT_Lannion_20_03_2025_p08_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Accord_Horaire_Variable_Lannion_20_03_2025_p07_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_accord_teletravail_avril_2022_p07_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_2025_NPS_amenagement_temps_de_travail_20_janvier_2025_p04_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_don_de_jours_14_novembre_2024_p11_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_PV_desaccord_Partage_de_la_valeur_VS_p06_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2024_19_avril_2024_p47_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Avenant_Proces_verbal_de_desaccord_NAO_2024_9_avril_2024_p05_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_CGF_p10_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_Etablissement_NNF_Lannion_Mise_en_place_accord_cadre_nouvelle_CCN_p06_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_cadre_NPS_nouvelle_convention_collective_2024_signe_p06_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_collectif_mise_en_place_CCN_p06_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_harmonisation_taux_variable_cible_salaries_non_sales_du_19_decemb_p10_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2024_p04_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_de_substitution_non_cadres_30_novembre_2023_p09_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_RCC_2023_p49_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_NAO_2023_PV_desaccord_p10_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_egalite_professionnelle_p20_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_amenagement_temps_travail_NPS_2023_p04_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_nombre_delegues_syndicaux_Lannion_24_janvier_2023_p04_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_augmentation_nombre_delegues_syndicaux_NPS_2023_p05_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/captures_signatures/rh_Accord_remboursement_sante_2023_p11_signature.jpg?csf=1&amp;web=1</t>
-  </si>
-  <si>
     <t>Trop c'est trop : la CGT a fait preuve de flexibilité et de pragmatisme en accompagnant les deux RCC précédentes (2023, 2024), un dispositif qui échange une signature contre la garantie du volontariat. La Direction semble désormais vouloir se faire un PSE EN 4X SANS FRAIS : ce sera sans nous. Jusqu'à 421 suppressions de postes non justifiées par la charge de travail ; ni garantie d'emploi ni embauche ; externalisations et perte de compétences ; pression au volontariat.</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_RCC_2026_p54_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_2026_protocole_accord_preectoral_LANNION_signe_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_2026_protocole_accord_preelectoral_signe_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Avenant_no_1_a_l_Accord_CSE_du_21_septembre_2018_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_d_entreprise_relatif_a_la_situation_de_handicap_NNF_p15-16_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_Etablissement_Prorogation_des_Mandats_CSE_E_Lannion_p05_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_NAO_2026_Proces_verbal_d_accord_24_janvier_2026_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Avenant_RCC_2025_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_Amenagement_Temps_Travail_NPS_2026_19_decembre_2025_p03_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_collectif_portant_sur_une_Rupture_Conventionnelle_Collective_RCC__p52_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Entreprise_au_sein_de_Noki_p17-18_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_d_entreprise_relatif_au_Plan_d_Epargne_Retraite_d_Entreprise_Coll_p20-21_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/cgt_GEPP_PV_de_desaccord_mis_a_signature_p12_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_CET_24_juillet_2025_p13-14_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_accord_collectif_relatif_aux_evolutions_du_regime_AUXAD_VF_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Avenant_frais_de_sante_9_avril_2025_p05-06_signatures.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_d_interessement_2025_2028_p16_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Proces_verbal_NAO_desaccord_2025_27_mars_2025_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Avenant_Accord_ARTT_Lannion_20_03_2025_p08_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Avenant_Accord_Horaire_Variable_Lannion_20_03_2025_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Avenant_accord_teletravail_avril_2022_p07_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_2025_NPS_amenagement_temps_de_travail_20_janvier_2025_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_don_de_jours_14_novembre_2024_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_PV_desaccord_Partage_de_la_valeur_VS_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_RCC_2024_19_avril_2024_p47_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Avenant_Proces_verbal_de_desaccord_NAO_2024_9_avril_2024_p05_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_CGF_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_Etablissement_NNF_Lannion_Mise_en_place_accord_cadre_nouvelle_CCN_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_cadre_NPS_nouvelle_convention_collective_2024_signe_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_collectif_mise_en_place_CCN_p06_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_harmonisation_taux_variable_cible_salaries_non_sales_du_19_decemb_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_amenagement_temps_travail_NPS_2024_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_de_substitution_non_cadres_30_novembre_2023_p09_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_RCC_2023_p49_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_NAO_2023_PV_desaccord_p10_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_egalite_professionnelle_p20_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_amenagement_temps_travail_NPS_2023_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_nombre_delegues_syndicaux_Lannion_24_janvier_2023_p04_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_augmentation_nombre_delegues_syndicaux_NPS_2023_p05_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:i:/r/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/signatures/rh_Accord_remboursement_sante_2023_p11_signature.jpg?csf=1&amp;web=1</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/accords%20n%C3%A9goci%C3%A9s/negos_html_files/copies/GEPP%20PV%20de%20d%C3%A9saccord%20mis%20%C3%A0%20signature.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/:b:/r/sites/BDESENNF-CSE-C/Shared%20Documents/05a.%20CSE-C/CSE-C%202025/03-CSE-C%20extraordinaire%209%20avril%202025/accord%20collectif%20relatif%20aux%20%C3%A9volutions%20du%20r%C3%A9gime%20AUXAD%20-VF.pdf?d=wa55078e44a6a4994b282eaeb8585d27c&amp;csf=1&amp;web=1&amp;e=Qi12JQ</t>
   </si>
 </sst>
 </file>
@@ -1922,16 +1922,16 @@
         <v>0</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>10</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>1</v>
@@ -1943,31 +1943,31 @@
         <v>3</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M1" s="8" t="s">
         <v>24</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P1" s="8" t="s">
         <v>11</v>
       </c>
       <c r="Q1" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="R1" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="R1" s="9" t="s">
-        <v>109</v>
-      </c>
       <c r="S1" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="105" x14ac:dyDescent="0.25">
@@ -1981,7 +1981,7 @@
         <v>23</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" s="11" t="str" cm="1">
         <f t="array" ref="E2">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D2,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2008,25 +2008,25 @@
         <v>-</v>
       </c>
       <c r="L2" s="19" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="R2" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="S2" s="11" t="str" cm="1">
         <f t="array" ref="S2">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R2,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2038,13 +2038,13 @@
         <v>2026</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E3" s="11" t="str" cm="1">
         <f t="array" ref="E3">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D3,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2072,17 +2072,17 @@
         <v>-</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O3" s="11"/>
       <c r="P3" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q3" s="15"/>
       <c r="R3" s="19"/>
@@ -2096,10 +2096,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E4" s="11" t="str" cm="1">
         <f t="array" ref="E4">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D4,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2127,17 +2127,17 @@
         <v>1</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O4" s="11"/>
       <c r="P4" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="Q4" s="15"/>
       <c r="R4" s="19"/>
@@ -2151,10 +2151,10 @@
         <v>13</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E5" s="11" t="str" cm="1">
         <f t="array" ref="E5">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D5,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2181,19 +2181,19 @@
         <v>-</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="Q5" s="15" t="s">
         <v>8</v>
@@ -2217,7 +2217,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E6" s="10" t="str" cm="1">
         <f t="array" ref="E6">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D6,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2244,19 +2244,19 @@
         <v>-</v>
       </c>
       <c r="L6" s="19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P6" s="17" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="Q6" s="16" t="s">
         <v>8</v>
@@ -2274,13 +2274,13 @@
         <v>2026</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E7" s="11" t="str" cm="1">
         <f t="array" ref="E7">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D7,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2308,17 +2308,17 @@
         <v>-</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O7" s="11"/>
       <c r="P7" s="17" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="Q7" s="15"/>
       <c r="R7" s="19"/>
@@ -2332,10 +2332,10 @@
         <v>13</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E8" s="11" t="str" cm="1">
         <f t="array" ref="E8">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D8,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2363,19 +2363,19 @@
         <v>-</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="P8" s="17" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="Q8" s="15" t="s">
         <v>8</v>
@@ -2396,10 +2396,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E9" s="11" t="str" cm="1">
         <f t="array" ref="E9">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D9,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2426,19 +2426,19 @@
         <v>-</v>
       </c>
       <c r="L9" s="19" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="Q9" s="15" t="s">
         <v>8</v>
@@ -2459,10 +2459,10 @@
         <v>14</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E10" s="10" t="str" cm="1">
         <f t="array" ref="E10">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D10,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2489,17 +2489,17 @@
         <v>1</v>
       </c>
       <c r="L10" s="19" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="Q10" s="16" t="s">
         <v>8</v>
@@ -2520,10 +2520,10 @@
         <v>13</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E11" s="11" t="str" cm="1">
         <f t="array" ref="E11">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D11,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2550,25 +2550,25 @@
         <v>-</v>
       </c>
       <c r="L11" s="19" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="N11" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O11" s="11" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="P11" s="11" t="s">
-        <v>333</v>
+        <v>291</v>
       </c>
       <c r="Q11" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="R11" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S11" s="11" t="str" cm="1">
         <f t="array" ref="S11">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R11,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2586,7 +2586,7 @@
         <v>17</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E12" s="11" t="str" cm="1">
         <f t="array" ref="E12">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D12,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2613,19 +2613,19 @@
         <v>-</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N12" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O12" s="11" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="P12" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Q12" s="15" t="s">
         <v>8</v>
@@ -2649,7 +2649,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E13" s="11" t="str" cm="1">
         <f t="array" ref="E13">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D13,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2676,19 +2676,19 @@
         <v>-</v>
       </c>
       <c r="L13" s="19" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N13" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="P13" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="Q13" s="15" t="s">
         <v>8</v>
@@ -2709,10 +2709,10 @@
         <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>28</v>
+        <v>332</v>
       </c>
       <c r="E14" s="11" t="str" cm="1">
         <f t="array" ref="E14">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D14,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2738,25 +2738,25 @@
         <v>-</v>
       </c>
       <c r="L14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="M14" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="Q14" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R14" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S14" s="11" t="str" cm="1">
         <f t="array" ref="S14">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R14,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2802,19 +2802,19 @@
         <v>-</v>
       </c>
       <c r="L15" s="19" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="M15" s="12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P15" s="11" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="Q15" s="15" t="s">
         <v>8</v>
@@ -2835,13 +2835,13 @@
         <v>13</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>209</v>
+        <v>333</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F16" s="12">
         <f>DATE(2025,4,9)</f>
@@ -2863,19 +2863,19 @@
         <v>8</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="M16" s="12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="P16" s="15" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="Q16" s="15" t="s">
         <v>8</v>
@@ -2895,10 +2895,10 @@
         <v>13</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E17" s="11" t="str" cm="1">
         <f t="array" ref="E17">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D17,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2926,19 +2926,19 @@
         <v>-</v>
       </c>
       <c r="L17" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="Q17" s="15"/>
       <c r="R17" s="19"/>
@@ -2955,7 +2955,7 @@
         <v>19</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E18" s="11" t="str" cm="1">
         <f t="array" ref="E18">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D18,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -2982,19 +2982,19 @@
         <v>-</v>
       </c>
       <c r="L18" s="19" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O18" s="11" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="P18" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="Q18" s="15" t="s">
         <v>8</v>
@@ -3015,10 +3015,10 @@
         <v>13</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E19" s="11" t="str" cm="1">
         <f t="array" ref="E19">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D19,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3044,25 +3044,25 @@
         <v>-</v>
       </c>
       <c r="L19" s="19" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="O19" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="P19" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Q19" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="R19" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S19" s="11" t="str" cm="1">
         <f t="array" ref="S19">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R19,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3074,13 +3074,13 @@
         <v>2025</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E20" s="11" t="str" cm="1">
         <f t="array" ref="E20">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D20,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3108,19 +3108,19 @@
         <v>-</v>
       </c>
       <c r="L20" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N20" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O20" s="11" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="P20" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Q20" s="15"/>
       <c r="R20" s="19"/>
@@ -3131,13 +3131,13 @@
         <v>2025</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E21" s="11" t="str" cm="1">
         <f t="array" ref="E21">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D21,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3165,19 +3165,19 @@
         <v>-</v>
       </c>
       <c r="L21" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N21" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="P21" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Q21" s="15"/>
       <c r="R21" s="19"/>
@@ -3191,10 +3191,10 @@
         <v>13</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E22" s="11" t="str" cm="1">
         <f t="array" ref="E22">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D22,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3221,25 +3221,25 @@
         <v>-</v>
       </c>
       <c r="L22" s="19" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M22" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="N22" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O22" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="P22" s="11" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="Q22" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="R22" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S22" s="11" t="str" cm="1">
         <f t="array" ref="S22">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R22,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3254,10 +3254,10 @@
         <v>14</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E23" s="10" t="str" cm="1">
         <f t="array" ref="E23">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D23,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3284,17 +3284,17 @@
         <v>1</v>
       </c>
       <c r="L23" s="19" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O23" s="10"/>
       <c r="P23" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="Q23" s="16" t="s">
         <v>8</v>
@@ -3318,7 +3318,7 @@
         <v>6</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E24" s="11" t="str" cm="1">
         <f t="array" ref="E24">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D24,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3345,19 +3345,19 @@
         <v>-</v>
       </c>
       <c r="L24" s="19" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M24" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N24" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="P24" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q24" s="15" t="s">
         <v>8</v>
@@ -3378,10 +3378,10 @@
         <v>13</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E25" s="11" t="str" cm="1">
         <f t="array" ref="E25">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D25,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3407,19 +3407,19 @@
         <v>-</v>
       </c>
       <c r="L25" s="19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M25" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P25" s="11" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="Q25" s="15" t="s">
         <v>8</v>
@@ -3443,7 +3443,7 @@
         <v>7</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E26" s="11" t="str" cm="1">
         <f t="array" ref="E26">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D26,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3470,25 +3470,25 @@
         <v>1</v>
       </c>
       <c r="L26" s="19" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N26" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="P26" s="11" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="Q26" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R26" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S26" s="11" t="str" cm="1">
         <f t="array" ref="S26">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R26,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3503,10 +3503,10 @@
         <v>13</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E27" s="11" t="str" cm="1">
         <f t="array" ref="E27">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D27,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3533,25 +3533,25 @@
         <v>-</v>
       </c>
       <c r="L27" s="19" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="M27" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N27" s="11" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="P27" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="Q27" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R27" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S27" s="11" t="str" cm="1">
         <f t="array" ref="S27">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R27,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3569,7 +3569,7 @@
         <v>20</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E28" s="11" t="str" cm="1">
         <f t="array" ref="E28">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D28,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3596,19 +3596,19 @@
         <v>-</v>
       </c>
       <c r="L28" s="19" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="M28" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N28" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="P28" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q28" s="15" t="s">
         <v>8</v>
@@ -3626,13 +3626,13 @@
         <v>2024</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E29" s="11" t="str" cm="1">
         <f t="array" ref="E29">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D29,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3660,19 +3660,19 @@
         <v>-</v>
       </c>
       <c r="L29" s="19" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="M29" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="P29" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q29" s="15"/>
       <c r="R29" s="19"/>
@@ -3686,7 +3686,7 @@
         <v>14</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" s="19" t="s">
         <v>26</v>
@@ -3717,25 +3717,25 @@
         <v>1</v>
       </c>
       <c r="L30" s="19" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="M30" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N30" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P30" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q30" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="R30" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S30" s="11" t="str" cm="1">
         <f t="array" ref="S30">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R30,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3750,10 +3750,10 @@
         <v>13</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E31" s="11" t="str" cm="1">
         <f t="array" ref="E31">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D31,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3781,19 +3781,19 @@
         <v>-</v>
       </c>
       <c r="L31" s="19" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M31" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P31" s="11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q31" s="15"/>
       <c r="R31" s="19"/>
@@ -3807,10 +3807,10 @@
         <v>13</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E32" s="11" t="str" cm="1">
         <f t="array" ref="E32">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D32,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3837,19 +3837,19 @@
         <v>-</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N32" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="P32" s="17" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="Q32" s="15" t="s">
         <v>8</v>
@@ -3870,7 +3870,7 @@
         <v>14</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D33" s="19" t="s">
         <v>27</v>
@@ -3900,19 +3900,19 @@
         <v>1</v>
       </c>
       <c r="L33" s="19" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="N33" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="P33" s="11" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="Q33" s="15" t="s">
         <v>8</v>
@@ -3936,7 +3936,7 @@
         <v>21</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E34" s="11" t="str" cm="1">
         <f t="array" ref="E34">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D34,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -3964,19 +3964,19 @@
         <v>-</v>
       </c>
       <c r="L34" s="19" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="M34" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N34" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P34" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Q34" s="15" t="s">
         <v>8</v>
@@ -4000,7 +4000,7 @@
         <v>5</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E35" s="11" t="str" cm="1">
         <f t="array" ref="E35">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D35,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4027,25 +4027,25 @@
         <v>-</v>
       </c>
       <c r="L35" s="19" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N35" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="P35" s="11" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="Q35" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R35" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S35" s="11" t="str" cm="1">
         <f t="array" ref="S35">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R35,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4060,10 +4060,10 @@
         <v>13</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E36" s="11" t="str" cm="1">
         <f t="array" ref="E36">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D36,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4089,25 +4089,25 @@
         <v>-</v>
       </c>
       <c r="L36" s="19" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="M36" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N36" s="11" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="P36" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q36" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R36" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S36" s="11" t="str" cm="1">
         <f t="array" ref="S36">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R36,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4125,7 +4125,7 @@
         <v>4</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E37" s="11" t="str" cm="1">
         <f t="array" ref="E37">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D37,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4152,25 +4152,25 @@
         <v>-</v>
       </c>
       <c r="L37" s="19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M37" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="N37" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="P37" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Q37" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R37" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S37" s="11" t="str" cm="1">
         <f t="array" ref="S37">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(R37,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4185,10 +4185,10 @@
         <v>14</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E38" s="11" t="str" cm="1">
         <f t="array" ref="E38">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D38,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4215,17 +4215,17 @@
         <v>1</v>
       </c>
       <c r="L38" s="19" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="N38" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O38" s="11"/>
       <c r="P38" s="11" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="Q38" s="15" t="s">
         <v>8</v>
@@ -4243,13 +4243,13 @@
         <v>2023</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E39" s="11" t="str" cm="1">
         <f t="array" ref="E39">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D39,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4277,17 +4277,17 @@
         <v>-</v>
       </c>
       <c r="L39" s="19" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O39" s="11"/>
       <c r="P39" s="11" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="Q39" s="15"/>
       <c r="R39" s="19"/>
@@ -4301,10 +4301,10 @@
         <v>14</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E40" s="11" t="str" cm="1">
         <f t="array" ref="E40">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D40,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4332,17 +4332,17 @@
         <v>1</v>
       </c>
       <c r="L40" s="19" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="M40" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O40" s="11"/>
       <c r="P40" s="15" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="Q40" s="15"/>
       <c r="R40" s="19"/>
@@ -4359,7 +4359,7 @@
         <v>22</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E41" s="11" t="str" cm="1">
         <f t="array" ref="E41">_xlfn.LET(_xlpm.n,IFERROR(_xlfn.TEXTAFTER(D41,"/",-1),""),_xlpm.c,{"%20","%27","%28","%29","%2C","%C3%A9","%C3%A8","%C3%AA","%C3%A0","%C3%A2","%C3%A7","%C3%B4","%C3%AE","%C3%B9","%C3%BB","%C3%89","%C2%BA","%C2%B0"},_xlpm.r,{" ","'","(",")",",","é","è","ê","à","â","ç","ô","î","ù","û","É","º","°"},_xlfn.REDUCE(_xlpm.n,_xlfn.SEQUENCE(COLUMNS(_xlpm.c)),_xlfn.LAMBDA(_xlpm.a,_xlpm.i,SUBSTITUTE(_xlpm.a,INDEX(_xlpm.c,_xlpm.i),INDEX(_xlpm.r,_xlpm.i)))))</f>
@@ -4387,17 +4387,17 @@
         <v>-</v>
       </c>
       <c r="L41" s="19" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="M41" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="O41" s="11"/>
       <c r="P41" s="15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Q41" s="15" t="s">
         <v>8</v>
@@ -4559,56 +4559,56 @@
   <sheetData>
     <row r="1" spans="1:2" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>241</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -4616,15 +4616,15 @@
         <v>0</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4632,39 +4632,39 @@
         <v>10</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>253</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4672,7 +4672,7 @@
         <v>24</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -4680,7 +4680,7 @@
         <v>24</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4688,15 +4688,15 @@
         <v>24</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -4704,31 +4704,31 @@
         <v>11</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -4752,15 +4752,15 @@
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>1</v>
@@ -4772,10 +4772,10 @@
         <v>3</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H3" s="24" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -4803,7 +4803,7 @@
         <v>-</v>
       </c>
       <c r="H4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -4831,12 +4831,12 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B6" s="27" cm="1">
         <f t="array" ref="B6">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A6="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A6))))</f>
@@ -4861,7 +4861,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B7" s="29" cm="1">
         <f t="array" ref="B7">_xlfn.LET(_xlpm.site,accords!$B$2:$B$1000,_xlpm.inc,ISNA(MATCH(accords!$C$2:$C$1000,$H$4:$H$20,0))*(_xlpm.site&lt;&gt;""),SUM(IF($A7="Total",_xlpm.inc,_xlpm.inc*(_xlpm.site=$A7))))</f>
@@ -4886,7 +4886,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -4895,32 +4895,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
-    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
-    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
-      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
-      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -5191,12 +5165,12 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -5246,26 +5220,33 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
-    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">AUIRPTAIMRO3-1066683228-25558</_dlc_DocId>
+    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
+    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
+      <Url>https://nokia.sharepoint.com/sites/CGT39/_layouts/15/DocIdRedir.aspx?ID=AUIRPTAIMRO3-1066683228-25558</Url>
+      <Description>AUIRPTAIMRO3-1066683228-25558</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a0c25b5-f40f-4aa1-8c63-969f2512d63e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5285,7 +5266,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F206293D-C2BD-4A18-87E2-049D4E2924C4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
@@ -5293,10 +5274,29 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEF070B-3FE9-48F0-B828-11286F698DFA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00212693-9A04-49E1-8889-2B5CE2179943}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEAC870E-20A6-413C-B639-D560014F1A64}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
+    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Note that the RCC 2024 talks were moved to NPS, where CFDT and CFTC already held a majority.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -878,7 +878,7 @@
     <t>Nokia n'a jamais eu l'intention d'aboutir à un accord : la négociation obligatoire a été menée pour la forme. Pas d'engagement d'embauche ni de remplacement des départs, garanties insuffisantes sur les activités en France.</t>
   </si>
   <si>
-    <t>Deuxième RCC acceptée car la pyramide des âges et le contexte le permettaient encore (départs volontaires majoritairement en fin de carrière) ; mesures individuelles de départ jugées correctes, alternative à un PSE. Bilan a posteriori critique : délocalisations, perte de savoir-faire, charge de travail, RPS, externalisations.</t>
+    <t>Deuxième RCC acceptée car la pyramide des âges et le contexte le permettaient encore (départs volontaires majoritairement en fin de carrière) ; mesures individuelles de départ jugées correctes, alternative à un PSE. La négociation avait été dépaysée au niveau de l'établissement NPS : la CFDT et la CFTC y étant majoritaires, l'accord majoritaire ne faisait aucun doute. Bilan a posteriori critique : délocalisations, perte de savoir-faire, charge de travail, RPS, externalisations.</t>
   </si>
   <si>
     <t>Après de longs débats internes, la CGT vote finalement la signature. Nouvelle réduction d'effectifs : 231 suppressions de postes en 2024 (non retrouvé dans le PDF, qui indique 347 maximum).</t>
@@ -4895,8 +4895,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="598b0ce14474b8a06003600b576ad2b7">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f3517c15821bb310180c621d8d765fa" ns2:_="" ns3:_="" ns4:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005C9E45C7454FD54C9F3832CA2EC2299C" ma:contentTypeVersion="18" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f12b8f105f65fc626cd1ca7eb8beb4c8">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="4a0c25b5-f40f-4aa1-8c63-969f2512d63e" xmlns:ns4="98344022-9d6c-42ca-8763-b68a110aeabc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="982fd3aadd5e0000c6cf8d705096d1e3" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
     <xsd:import namespace="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
     <xsd:import namespace="98344022-9d6c-42ca-8763-b68a110aeabc"/>
@@ -4950,12 +4950,12 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="_dlc_DocId" ma:index="24" nillable="true" ma:displayName="Document ID Value" ma:description="The value of the document ID assigned to this item." ma:indexed="true" ma:internalName="_dlc_DocId" ma:readOnly="true">
+    <xsd:element name="_dlc_DocId" ma:index="24" nillable="true" ma:displayName="Valeur d’ID de document" ma:description="Valeur de l’ID de document affecté à cet élément." ma:indexed="true" ma:internalName="_dlc_DocId" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="_dlc_DocIdUrl" ma:index="25" nillable="true" ma:displayName="Document ID" ma:description="Permanent link to this document." ma:hidden="true" ma:internalName="_dlc_DocIdUrl" ma:readOnly="true">
+    <xsd:element name="_dlc_DocIdUrl" ma:index="25" nillable="true" ma:displayName="ID de document" ma:description="Lien permanent vers ce document." ma:hidden="true" ma:internalName="_dlc_DocIdUrl" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:URL">
@@ -4996,7 +4996,7 @@
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -5039,7 +5039,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="98344022-9d6c-42ca-8763-b68a110aeabc" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="11" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="11" nillable="true" ma:displayName="Partagé avec" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -5058,7 +5058,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="12" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="12" nillable="true" ma:displayName="Partagé avec détails" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -5075,8 +5075,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -5247,23 +5247,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15AD6385-0C64-4344-9EFB-A995A9D73E48}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
-    <ds:schemaRef ds:uri="4a0c25b5-f40f-4aa1-8c63-969f2512d63e"/>
-    <ds:schemaRef ds:uri="98344022-9d6c-42ca-8763-b68a110aeabc"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38D2123B-851A-4844-B755-63151B1DE5F2}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Update tract links after moving PDFs into the shared copies folder.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/accords.xlsx
+++ b/accords.xlsx
@@ -185,31 +185,31 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Temps%20de%20travail/Accord%20Am%C3%A9nagement%20Temps%20Travail%20NPS%202026%20(19%20d%C3%A9cembre%202025).pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2026/2026_06_TRACT-RetourSondageRCC2026-2.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract_pour_ceux_qui_restent.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract_rcc_2026.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract-salaires-2025.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2025/tract-avenant-TL-v2.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2024/tract_bilan_rcc24_v4.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2023/ncc%20cotation%203.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2023/Tract%20Volontariat%20RCC.pdf</t>
-  </si>
-  <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2023/Tract%20br%C3%A8ves%20de%20printemps.pdf</t>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/2026_06_TRACT-RetourSondageRCC2026-2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_pour_ceux_qui_restent.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_rcc_2026.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract-salaires-2025.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract-avenant-TL-v2.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_bilan_rcc24_v4.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/ncc%20cotation%203.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20Volontariat%20RCC.pdf</t>
+  </si>
+  <si>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/Tract%20br%C3%A8ves%20de%20printemps.pdf</t>
   </si>
   <si>
     <t>page signature</t>
@@ -293,7 +293,7 @@
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/Archive/Archives/Accords%20Nokia/Accord%20harmonisation%20taux%20variable%20cible%20salari%C3%A9s%20non%20sales%20du%2019%20d%C3%A9cembre%202023.pdf</t>
   </si>
   <si>
-    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/2024/tract_retour_salaires_2024_v1.pdf</t>
+    <t>https://nokia.sharepoint.com/sites/CGT39/Shared%20Documents/salari%C3%A9s/tracts%20diffus%C3%A9s/tracts_html_files/copies/tract_retour_salaires_2024_v1.pdf</t>
   </si>
   <si>
     <t>https://nokia.sharepoint.com/sites/HRLibrary/Controlled%20Documents/HR%20Regions/Europe%20South/France/HR%20SOPs-Guidelines-Policy/Harmonized/Accords%20conventions%202026/Avenant%20n%C2%BA%201%20%C3%A0%20l'Accord%20CSE%20du%2021%20septembre%202018.pdf</t>

</xml_diff>